<commit_message>
Aggiornamento automatico del sito — 03/08/2026 10:14
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA904FA-37F9-40E3-BABD-02D0A33B6C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C165AC-73C9-4AD8-990B-C144DE265D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1054,8 +1054,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:O110" totalsRowShown="0">
-  <autoFilter ref="A1:O110" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:O150" totalsRowShown="0">
+  <autoFilter ref="A1:O150" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{40EB6498-034B-4FD2-B823-BD9BDE560AB5}" name="ID"/>
     <tableColumn id="2" xr3:uid="{E00E7517-D29A-46F7-B049-8E1F1ECC043C}" name="Titolo"/>
@@ -1398,9 +1398,10 @@
     <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="10" max="10" width="19.33203125" customWidth="1"/>
     <col min="11" max="11" width="25.44140625" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" customWidth="1"/>
-    <col min="14" max="14" width="21.109375" customWidth="1"/>
-    <col min="15" max="15" width="22.5546875" customWidth="1"/>
+    <col min="12" max="12" width="114.5546875" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="14" width="23.5546875" customWidth="1"/>
+    <col min="15" max="15" width="24.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 03/08/2026 11:30
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C165AC-73C9-4AD8-990B-C144DE265D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13ACCCAA-7F29-4879-B891-CDF861E11BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -1393,6 +1393,7 @@
   <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="83.88671875" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" customWidth="1"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 03/08/2026 11:48
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13ACCCAA-7F29-4879-B891-CDF861E11BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D38B9B-C284-44BC-993D-61A6E9E62B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -813,9 +813,6 @@
     <t>AMI-0057</t>
   </si>
   <si>
-    <t>Congresso di fondazione del Partito Comunista d'Italia</t>
-  </si>
-  <si>
     <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista d'Italia (marxista-leninista) - Lotta di lunga; Partito Marxista-Leninista-Maoista Italiano</t>
   </si>
   <si>
@@ -976,6 +973,9 @@
   </si>
   <si>
     <t>Rivista</t>
+  </si>
+  <si>
+    <t>Congresso di fondazione del Partito Comunista Unificato d'Italia</t>
   </si>
 </sst>
 </file>
@@ -3249,7 +3249,7 @@
         <v>262</v>
       </c>
       <c r="B58" t="s">
-        <v>263</v>
+        <v>317</v>
       </c>
       <c r="C58" t="s">
         <v>249</v>
@@ -3276,13 +3276,13 @@
         <v>252</v>
       </c>
       <c r="K58" t="s">
+        <v>263</v>
+      </c>
+      <c r="L58" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="L58" s="4" t="s">
+      <c r="M58" t="s">
         <v>265</v>
-      </c>
-      <c r="M58" t="s">
-        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3362,19 +3362,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B1" t="s">
         <v>267</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>268</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>269</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>270</v>
-      </c>
-      <c r="E1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -3382,7 +3382,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C2">
         <v>1893</v>
@@ -3391,15 +3391,15 @@
         <v>1976</v>
       </c>
       <c r="E2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B3" t="s">
         <v>274</v>
-      </c>
-      <c r="B3" t="s">
-        <v>275</v>
       </c>
       <c r="C3">
         <v>1921</v>
@@ -3408,7 +3408,7 @@
         <v>1993</v>
       </c>
       <c r="E3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -3416,16 +3416,16 @@
         <v>252</v>
       </c>
       <c r="B4" t="s">
+        <v>276</v>
+      </c>
+      <c r="C4" t="s">
         <v>277</v>
-      </c>
-      <c r="C4" t="s">
-        <v>278</v>
       </c>
       <c r="D4">
         <v>2021</v>
       </c>
       <c r="E4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -3433,7 +3433,7 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C5">
         <v>1931</v>
@@ -3444,10 +3444,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B6" t="s">
         <v>281</v>
-      </c>
-      <c r="B6" t="s">
-        <v>282</v>
       </c>
       <c r="C6">
         <v>1960</v>
@@ -3461,23 +3461,23 @@
         <v>158</v>
       </c>
       <c r="B7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>283</v>
+      </c>
+      <c r="B8" t="s">
         <v>284</v>
-      </c>
-      <c r="B8" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B9" t="s">
         <v>286</v>
-      </c>
-      <c r="B9" t="s">
-        <v>287</v>
       </c>
       <c r="C9">
         <v>1907</v>
@@ -3488,10 +3488,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>287</v>
+      </c>
+      <c r="B10" t="s">
         <v>288</v>
-      </c>
-      <c r="B10" t="s">
-        <v>289</v>
       </c>
       <c r="C10">
         <v>1898</v>
@@ -3502,10 +3502,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B11" t="s">
         <v>290</v>
-      </c>
-      <c r="B11" t="s">
-        <v>291</v>
       </c>
       <c r="C11">
         <v>1898</v>
@@ -3516,10 +3516,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B12" t="s">
         <v>292</v>
-      </c>
-      <c r="B12" t="s">
-        <v>293</v>
       </c>
       <c r="C12">
         <v>1904</v>
@@ -3530,10 +3530,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>293</v>
+      </c>
+      <c r="B13" t="s">
         <v>294</v>
-      </c>
-      <c r="B13" t="s">
-        <v>295</v>
       </c>
       <c r="C13">
         <v>1914</v>
@@ -3544,10 +3544,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>295</v>
+      </c>
+      <c r="B14" t="s">
         <v>296</v>
-      </c>
-      <c r="B14" t="s">
-        <v>297</v>
       </c>
       <c r="C14">
         <v>1920</v>
@@ -3561,7 +3561,7 @@
         <v>207</v>
       </c>
       <c r="B15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C15">
         <v>1920</v>
@@ -3588,19 +3588,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1" t="s">
         <v>299</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>300</v>
       </c>
-      <c r="D1" t="s">
-        <v>301</v>
-      </c>
       <c r="E1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -3608,13 +3608,13 @@
         <v>208</v>
       </c>
       <c r="B2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C2">
         <v>1962</v>
       </c>
       <c r="D2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -3622,7 +3622,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C3">
         <v>1952</v>
@@ -3633,7 +3633,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C4">
         <v>1963</v>
@@ -3647,7 +3647,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C5">
         <v>1948</v>
@@ -3655,10 +3655,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C6">
         <v>1958</v>
@@ -3672,7 +3672,7 @@
         <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C7">
         <v>1964</v>
@@ -3683,10 +3683,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C8">
         <v>1956</v>
@@ -3697,7 +3697,7 @@
         <v>117</v>
       </c>
       <c r="B9" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -3705,7 +3705,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C10">
         <v>1966</v>
@@ -3719,7 +3719,7 @@
         <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C11">
         <v>1968</v>
@@ -3730,10 +3730,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B12" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C12">
         <v>1966</v>
@@ -3747,7 +3747,7 @@
         <v>188</v>
       </c>
       <c r="B13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C13">
         <v>1921</v>
@@ -3758,7 +3758,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C14">
         <v>1966</v>
@@ -3767,7 +3767,7 @@
         <v>1991</v>
       </c>
       <c r="E14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -3775,7 +3775,7 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C15">
         <v>1968</v>
@@ -3784,7 +3784,7 @@
         <v>1972</v>
       </c>
       <c r="E15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -3792,21 +3792,21 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C16">
         <v>1921</v>
       </c>
       <c r="E16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B17" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C17">
         <v>1968</v>
@@ -3820,7 +3820,7 @@
         <v>156</v>
       </c>
       <c r="B18" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C18">
         <v>1969</v>
@@ -3834,13 +3834,13 @@
         <v>239</v>
       </c>
       <c r="B19" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C19">
         <v>1968</v>
       </c>
       <c r="D19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -3848,7 +3848,7 @@
         <v>245</v>
       </c>
       <c r="B20" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C20">
         <v>1972</v>
@@ -3862,7 +3862,7 @@
         <v>116</v>
       </c>
       <c r="B21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C21">
         <v>1967</v>
@@ -3876,7 +3876,7 @@
         <v>249</v>
       </c>
       <c r="B22" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C22">
         <v>1977</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 04/08/2026 19:32
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D38B9B-C284-44BC-993D-61A6E9E62B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4369D5F5-222C-46C9-94D9-8AE6AC28548B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="327">
   <si>
     <t>ID</t>
   </si>
@@ -976,13 +976,40 @@
   </si>
   <si>
     <t>Congresso di fondazione del Partito Comunista Unificato d'Italia</t>
+  </si>
+  <si>
+    <t>AMI-0058</t>
+  </si>
+  <si>
+    <t>AMI-0059</t>
+  </si>
+  <si>
+    <t>Proletari senza rivoluzione: Storia delle classi subalterne italiane dal 1860 al 1950, Vol. 2</t>
+  </si>
+  <si>
+    <t>Proletari senza rivoluzione: Storia delle classi subalterne italiane dal 1860 al 1950, Vol. 1</t>
+  </si>
+  <si>
+    <t>Renzo del Carria</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/proletari-senza-rivoluzione-2/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/proletari-senza-rivoluzione-1/mode/2up</t>
+  </si>
+  <si>
+    <t>Provenienza</t>
+  </si>
+  <si>
+    <t>Archivio Storico della Nuova Sinistra "Marco Pezzi"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -994,6 +1021,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1054,9 +1087,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:O150" totalsRowShown="0">
-  <autoFilter ref="A1:O150" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:P150" totalsRowShown="0">
+  <autoFilter ref="A1:P150" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{40EB6498-034B-4FD2-B823-BD9BDE560AB5}" name="ID"/>
     <tableColumn id="2" xr3:uid="{E00E7517-D29A-46F7-B049-8E1F1ECC043C}" name="Titolo"/>
     <tableColumn id="3" xr3:uid="{12EB6F9C-1D8F-4A95-872D-EB8DF3CC2DA3}" name="Organizzazione"/>
@@ -1068,6 +1101,7 @@
     <tableColumn id="9" xr3:uid="{95A8BDEE-2111-4C66-8F45-95353EF33A2F}" name="Serie"/>
     <tableColumn id="10" xr3:uid="{90BC9D87-1BF0-48A2-868D-6C56548FCEB4}" name="Persone_collegate"/>
     <tableColumn id="11" xr3:uid="{C8BD21B7-C8B1-4984-92F4-1D47F4D1DDE8}" name="Organizzazioni_collegate"/>
+    <tableColumn id="16" xr3:uid="{2EA96E38-185B-4190-9E45-A3915A9F5041}" name="Provenienza"/>
     <tableColumn id="12" xr3:uid="{39126A50-DCAA-4469-B47D-EEF765E35B2A}" name="URL"/>
     <tableColumn id="13" xr3:uid="{2CA56103-9CDF-40D7-9D80-7561D0C1F54A}" name="Nome_file"/>
     <tableColumn id="14" xr3:uid="{031C733F-A723-4277-8E99-4BFF4677306D}" name="Nome_file_originale"/>
@@ -1390,7 +1424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -1399,13 +1433,13 @@
     <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="10" max="10" width="19.33203125" customWidth="1"/>
     <col min="11" max="11" width="25.44140625" customWidth="1"/>
-    <col min="12" max="12" width="114.5546875" customWidth="1"/>
+    <col min="12" max="12" width="43" customWidth="1"/>
     <col min="13" max="13" width="26" customWidth="1"/>
     <col min="14" max="14" width="23.5546875" customWidth="1"/>
     <col min="15" max="15" width="24.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1440,19 +1474,22 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
+        <v>325</v>
+      </c>
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1480,11 +1517,11 @@
       <c r="I2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1512,11 +1549,11 @@
       <c r="I3" t="s">
         <v>27</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1544,11 +1581,11 @@
       <c r="I4" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="M4" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1576,11 +1613,11 @@
       <c r="I5" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="M5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -1608,11 +1645,11 @@
       <c r="I6" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="M6" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1640,11 +1677,11 @@
       <c r="I7" t="s">
         <v>27</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="M7" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -1672,11 +1709,11 @@
       <c r="I8" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="M8" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -1704,11 +1741,11 @@
       <c r="I9" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="M9" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -1736,11 +1773,11 @@
       <c r="I10" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="M10" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -1768,11 +1805,11 @@
       <c r="I11" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="M11" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -1803,11 +1840,11 @@
       <c r="K12" t="s">
         <v>17</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="M12" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>58</v>
       </c>
@@ -1835,11 +1872,11 @@
       <c r="I13" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="M13" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>62</v>
       </c>
@@ -1873,11 +1910,11 @@
       <c r="K14" t="s">
         <v>70</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="M14" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>72</v>
       </c>
@@ -1905,14 +1942,14 @@
       <c r="J15" t="s">
         <v>76</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="M15" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -1940,14 +1977,14 @@
       <c r="J16" t="s">
         <v>82</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="M16" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -1975,14 +2012,14 @@
       <c r="J17" t="s">
         <v>87</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="M17" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>90</v>
       </c>
@@ -2007,11 +2044,11 @@
       <c r="I18" t="s">
         <v>68</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="M18" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>97</v>
       </c>
@@ -2036,14 +2073,14 @@
       <c r="I19" t="s">
         <v>68</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="M19" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="M19" t="s">
+      <c r="N19" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -2065,11 +2102,11 @@
       <c r="I20" t="s">
         <v>106</v>
       </c>
-      <c r="L20" s="4" t="s">
+      <c r="M20" s="4" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>108</v>
       </c>
@@ -2094,11 +2131,11 @@
       <c r="I21" t="s">
         <v>106</v>
       </c>
-      <c r="L21" s="4" t="s">
+      <c r="M21" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>114</v>
       </c>
@@ -2123,11 +2160,14 @@
       <c r="I22" t="s">
         <v>120</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" t="s">
+        <v>326</v>
+      </c>
+      <c r="M22" s="4" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>122</v>
       </c>
@@ -2152,11 +2192,14 @@
       <c r="I23" t="s">
         <v>120</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="L23" t="s">
+        <v>326</v>
+      </c>
+      <c r="M23" s="4" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>125</v>
       </c>
@@ -2181,11 +2224,14 @@
       <c r="I24" t="s">
         <v>120</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="L24" t="s">
+        <v>326</v>
+      </c>
+      <c r="M24" s="4" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>128</v>
       </c>
@@ -2210,11 +2256,14 @@
       <c r="I25" t="s">
         <v>120</v>
       </c>
-      <c r="L25" s="4" t="s">
+      <c r="L25" t="s">
+        <v>326</v>
+      </c>
+      <c r="M25" s="4" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>131</v>
       </c>
@@ -2239,11 +2288,14 @@
       <c r="I26" t="s">
         <v>120</v>
       </c>
-      <c r="L26" s="4" t="s">
+      <c r="L26" t="s">
+        <v>326</v>
+      </c>
+      <c r="M26" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>134</v>
       </c>
@@ -2268,11 +2320,14 @@
       <c r="I27" t="s">
         <v>120</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="L27" t="s">
+        <v>326</v>
+      </c>
+      <c r="M27" s="4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>137</v>
       </c>
@@ -2297,11 +2352,14 @@
       <c r="I28" t="s">
         <v>120</v>
       </c>
-      <c r="L28" s="4" t="s">
+      <c r="L28" t="s">
+        <v>326</v>
+      </c>
+      <c r="M28" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>140</v>
       </c>
@@ -2329,11 +2387,14 @@
       <c r="K29" t="s">
         <v>64</v>
       </c>
-      <c r="L29" s="4" t="s">
+      <c r="L29" t="s">
+        <v>326</v>
+      </c>
+      <c r="M29" s="4" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -2361,11 +2422,14 @@
       <c r="K30" t="s">
         <v>145</v>
       </c>
-      <c r="L30" s="4" t="s">
+      <c r="L30" t="s">
+        <v>326</v>
+      </c>
+      <c r="M30" s="4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>147</v>
       </c>
@@ -2393,11 +2457,11 @@
       <c r="I31" t="s">
         <v>34</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="M31" s="4" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>151</v>
       </c>
@@ -2425,11 +2489,11 @@
       <c r="I32" t="s">
         <v>34</v>
       </c>
-      <c r="L32" s="4" t="s">
+      <c r="M32" s="4" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>154</v>
       </c>
@@ -2451,14 +2515,14 @@
       <c r="J33" t="s">
         <v>158</v>
       </c>
-      <c r="L33" s="4" t="s">
+      <c r="M33" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="M33" t="s">
+      <c r="N33" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>161</v>
       </c>
@@ -2486,17 +2550,17 @@
       <c r="K34" t="s">
         <v>17</v>
       </c>
-      <c r="L34" s="4" t="s">
+      <c r="M34" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="N34" t="s">
+      <c r="O34" t="s">
         <v>166</v>
       </c>
-      <c r="O34" t="s">
+      <c r="P34" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>168</v>
       </c>
@@ -2527,17 +2591,17 @@
       <c r="K35" t="s">
         <v>64</v>
       </c>
-      <c r="L35" s="4" t="s">
+      <c r="M35" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="N35" t="s">
+      <c r="O35" t="s">
         <v>172</v>
       </c>
-      <c r="O35" t="s">
+      <c r="P35" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>174</v>
       </c>
@@ -2559,11 +2623,11 @@
       <c r="I36" t="s">
         <v>68</v>
       </c>
-      <c r="L36" s="4" t="s">
+      <c r="M36" s="4" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>178</v>
       </c>
@@ -2594,11 +2658,11 @@
       <c r="K37" t="s">
         <v>156</v>
       </c>
-      <c r="L37" s="4" t="s">
+      <c r="M37" s="4" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>183</v>
       </c>
@@ -2626,11 +2690,11 @@
       <c r="I38" t="s">
         <v>34</v>
       </c>
-      <c r="L38" s="4" t="s">
+      <c r="M38" s="4" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>186</v>
       </c>
@@ -2661,11 +2725,11 @@
       <c r="J39" t="s">
         <v>189</v>
       </c>
-      <c r="L39" s="4" t="s">
+      <c r="M39" s="4" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>191</v>
       </c>
@@ -2693,11 +2757,11 @@
       <c r="I40" t="s">
         <v>193</v>
       </c>
-      <c r="L40" s="4" t="s">
+      <c r="M40" s="4" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>195</v>
       </c>
@@ -2725,11 +2789,11 @@
       <c r="I41" t="s">
         <v>34</v>
       </c>
-      <c r="L41" s="4" t="s">
+      <c r="M41" s="4" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>199</v>
       </c>
@@ -2754,11 +2818,11 @@
       <c r="I42" t="s">
         <v>202</v>
       </c>
-      <c r="L42" s="4" t="s">
+      <c r="M42" s="4" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>204</v>
       </c>
@@ -2789,11 +2853,11 @@
       <c r="K43" t="s">
         <v>208</v>
       </c>
-      <c r="L43" s="4" t="s">
+      <c r="M43" s="4" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>210</v>
       </c>
@@ -2821,11 +2885,11 @@
       <c r="I44" t="s">
         <v>27</v>
       </c>
-      <c r="L44" s="4" t="s">
+      <c r="M44" s="4" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>213</v>
       </c>
@@ -2853,11 +2917,11 @@
       <c r="I45" t="s">
         <v>27</v>
       </c>
-      <c r="L45" s="4" t="s">
+      <c r="M45" s="4" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>216</v>
       </c>
@@ -2885,11 +2949,11 @@
       <c r="I46" t="s">
         <v>27</v>
       </c>
-      <c r="L46" s="4" t="s">
+      <c r="M46" s="4" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>219</v>
       </c>
@@ -2917,11 +2981,11 @@
       <c r="I47" t="s">
         <v>34</v>
       </c>
-      <c r="L47" s="4" t="s">
+      <c r="M47" s="4" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>222</v>
       </c>
@@ -2949,11 +3013,11 @@
       <c r="I48" t="s">
         <v>34</v>
       </c>
-      <c r="L48" s="4" t="s">
+      <c r="M48" s="4" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>225</v>
       </c>
@@ -2981,11 +3045,11 @@
       <c r="I49" t="s">
         <v>27</v>
       </c>
-      <c r="L49" s="4" t="s">
+      <c r="M49" s="4" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>228</v>
       </c>
@@ -3013,11 +3077,11 @@
       <c r="I50" t="s">
         <v>27</v>
       </c>
-      <c r="L50" s="4" t="s">
+      <c r="M50" s="4" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>231</v>
       </c>
@@ -3045,11 +3109,11 @@
       <c r="I51" t="s">
         <v>27</v>
       </c>
-      <c r="L51" s="4" t="s">
+      <c r="M51" s="4" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>234</v>
       </c>
@@ -3077,11 +3141,11 @@
       <c r="I52" t="s">
         <v>34</v>
       </c>
-      <c r="L52" s="4" t="s">
+      <c r="M52" s="4" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>237</v>
       </c>
@@ -3109,11 +3173,11 @@
       <c r="I53" t="s">
         <v>68</v>
       </c>
-      <c r="L53" s="4" t="s">
+      <c r="M53" s="4" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>242</v>
       </c>
@@ -3138,11 +3202,11 @@
       <c r="K54" t="s">
         <v>245</v>
       </c>
-      <c r="L54" s="4" t="s">
+      <c r="M54" s="4" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>247</v>
       </c>
@@ -3173,14 +3237,14 @@
       <c r="J55" t="s">
         <v>252</v>
       </c>
-      <c r="L55" s="4" t="s">
+      <c r="M55" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="M55" t="s">
+      <c r="N55" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>255</v>
       </c>
@@ -3205,14 +3269,14 @@
       <c r="I56" t="s">
         <v>68</v>
       </c>
-      <c r="L56" s="4" t="s">
+      <c r="M56" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="M56" t="s">
+      <c r="N56" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>259</v>
       </c>
@@ -3240,11 +3304,11 @@
       <c r="I57" t="s">
         <v>202</v>
       </c>
-      <c r="L57" s="4" t="s">
+      <c r="M57" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>262</v>
       </c>
@@ -3278,76 +3342,143 @@
       <c r="K58" t="s">
         <v>263</v>
       </c>
-      <c r="L58" s="4" t="s">
+      <c r="M58" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="M58" t="s">
+      <c r="N58" t="s">
         <v>265</v>
       </c>
     </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>318</v>
+      </c>
+      <c r="B59" t="s">
+        <v>321</v>
+      </c>
+      <c r="C59" t="s">
+        <v>99</v>
+      </c>
+      <c r="D59" t="s">
+        <v>322</v>
+      </c>
+      <c r="E59" t="s">
+        <v>99</v>
+      </c>
+      <c r="F59">
+        <v>1970</v>
+      </c>
+      <c r="G59" t="s">
+        <v>20</v>
+      </c>
+      <c r="H59" t="s">
+        <v>176</v>
+      </c>
+      <c r="I59" t="s">
+        <v>106</v>
+      </c>
+      <c r="M59" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>319</v>
+      </c>
+      <c r="B60" t="s">
+        <v>320</v>
+      </c>
+      <c r="C60" t="s">
+        <v>99</v>
+      </c>
+      <c r="D60" t="s">
+        <v>322</v>
+      </c>
+      <c r="E60" t="s">
+        <v>99</v>
+      </c>
+      <c r="F60">
+        <v>1970</v>
+      </c>
+      <c r="G60" t="s">
+        <v>20</v>
+      </c>
+      <c r="H60" t="s">
+        <v>176</v>
+      </c>
+      <c r="I60" t="s">
+        <v>106</v>
+      </c>
+      <c r="M60" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="L15" r:id="rId1" xr:uid="{070CD713-285D-499E-AAF3-CA6E04F2E67D}"/>
-    <hyperlink ref="L16" r:id="rId2" xr:uid="{84CDC93C-1C17-4B8A-99AF-92002F858E35}"/>
-    <hyperlink ref="L17" r:id="rId3" xr:uid="{D28CC0D1-FF9B-45E5-8C06-32AA0A3E53A9}"/>
-    <hyperlink ref="L18" r:id="rId4" xr:uid="{B48EE935-D4BB-42A2-BD03-F7462BDAA973}"/>
-    <hyperlink ref="L19" r:id="rId5" xr:uid="{FC1907F3-06C3-44E2-85AA-D0706308A852}"/>
-    <hyperlink ref="L20" r:id="rId6" xr:uid="{FDA55CF4-B32E-4DB1-9DD2-2EFA7CF0ABA3}"/>
-    <hyperlink ref="L21" r:id="rId7" xr:uid="{7D576BEC-A372-4CAE-BF84-2F0963043CDC}"/>
-    <hyperlink ref="L22" r:id="rId8" xr:uid="{F23954CB-9B25-4B73-8617-4ADD50A0FE7D}"/>
-    <hyperlink ref="L24" r:id="rId9" xr:uid="{7A4658DA-5DD5-47F2-85C1-73F1BDE8C8F1}"/>
-    <hyperlink ref="L3" r:id="rId10" xr:uid="{049E9471-667A-44C7-B555-6B41CDEA4334}"/>
-    <hyperlink ref="L2" r:id="rId11" xr:uid="{A94FBB18-F767-4034-AB25-89E99187EDC8}"/>
-    <hyperlink ref="L4" r:id="rId12" xr:uid="{90B8B390-068D-4C88-BDE5-E99B638462B8}"/>
-    <hyperlink ref="L5" r:id="rId13" xr:uid="{01D903FA-154C-4673-BAA8-E8DA92B9B8EF}"/>
-    <hyperlink ref="L6" r:id="rId14" xr:uid="{682D036E-FC9A-4F6A-98CD-4CC91B1FB74F}"/>
-    <hyperlink ref="L7" r:id="rId15" xr:uid="{3F4DD620-2B56-494F-A792-A22FC9B8558D}"/>
-    <hyperlink ref="L8" r:id="rId16" xr:uid="{98CD4C7F-B63B-4FF7-9B9D-848EB9126C18}"/>
-    <hyperlink ref="L9" r:id="rId17" xr:uid="{21EFE2D2-97B6-4C85-A920-0CB2A7EC194D}"/>
-    <hyperlink ref="L10" r:id="rId18" xr:uid="{243006E2-0318-4FEE-83E6-AE585C338675}"/>
-    <hyperlink ref="L11" r:id="rId19" xr:uid="{1C7440C2-41CA-429B-80DC-4C69183A7CB9}"/>
-    <hyperlink ref="L12" r:id="rId20" xr:uid="{02E0AD7E-CEF6-4B6C-AB17-6CFDCF494509}"/>
-    <hyperlink ref="L13" r:id="rId21" xr:uid="{ABEF46E4-5EAF-4B10-9C40-A0B5F240E5BE}"/>
-    <hyperlink ref="L14" r:id="rId22" xr:uid="{B047393B-2E22-4ABF-A937-7D3E0B2FACB6}"/>
-    <hyperlink ref="L23" r:id="rId23" xr:uid="{A4B37D7B-D4FE-4B50-A01A-19BC8F084672}"/>
-    <hyperlink ref="L25" r:id="rId24" xr:uid="{46495F89-39F5-46CA-B3F0-960411F5BC3C}"/>
-    <hyperlink ref="L26" r:id="rId25" xr:uid="{5AD82D9D-0E76-446D-9312-7E6628A684B1}"/>
-    <hyperlink ref="L27" r:id="rId26" xr:uid="{C2001CED-BED9-4C03-B640-920A41146810}"/>
-    <hyperlink ref="L29" r:id="rId27" xr:uid="{DA89E417-4E4A-4547-B9AE-B031E332AA2A}"/>
-    <hyperlink ref="L28" r:id="rId28" xr:uid="{A051F0A1-FCEF-4CBB-9900-7D1A10FDEAE5}"/>
-    <hyperlink ref="L30" r:id="rId29" xr:uid="{D3924AA9-86C0-4DF6-B403-67F371618448}"/>
-    <hyperlink ref="L31" r:id="rId30" xr:uid="{FBF9CB2D-4BDE-4C09-A9B9-E188D6960A6D}"/>
-    <hyperlink ref="L32" r:id="rId31" xr:uid="{4BE15358-8230-40C1-9063-AA9B0E3B3CD2}"/>
-    <hyperlink ref="L33" r:id="rId32" xr:uid="{1F894DFD-3BA6-465A-AF03-CDD08322754B}"/>
-    <hyperlink ref="L34" r:id="rId33" xr:uid="{581D5573-91DC-48B0-B727-966BB2028F03}"/>
-    <hyperlink ref="L35" r:id="rId34" xr:uid="{A2BF5663-A951-44D0-8055-DEB448E680FA}"/>
-    <hyperlink ref="L36" r:id="rId35" xr:uid="{617F5B23-3270-413A-A61D-68FDD54E7A5D}"/>
-    <hyperlink ref="L58" r:id="rId36" xr:uid="{51AC1783-6AF1-44A4-B660-485062AF29AC}"/>
-    <hyperlink ref="L57" r:id="rId37" xr:uid="{FB7BD1A0-AC49-43FC-854E-AC6789AE027F}"/>
-    <hyperlink ref="L56" r:id="rId38" xr:uid="{39FD45C0-8BE5-49BB-820B-F4B1C9541F87}"/>
-    <hyperlink ref="L55" r:id="rId39" xr:uid="{7E342A29-2423-4FDD-810C-FE73FAB7AE34}"/>
-    <hyperlink ref="L54" r:id="rId40" xr:uid="{1E92ED11-F3F3-4DA7-9D48-EE7BC4656DBE}"/>
-    <hyperlink ref="L53" r:id="rId41" xr:uid="{23968C0E-AA65-46EC-BCA7-5E09457FFE21}"/>
-    <hyperlink ref="L52" r:id="rId42" xr:uid="{ECC4B67E-553A-48BB-AA46-D6D3B7E711A3}"/>
-    <hyperlink ref="L51" r:id="rId43" xr:uid="{EE7680E7-C97C-4D61-BAA2-B6338763FDC4}"/>
-    <hyperlink ref="L50" r:id="rId44" xr:uid="{F5DF849D-6410-4191-95D4-230AC66C7CA4}"/>
-    <hyperlink ref="L49" r:id="rId45" xr:uid="{503C1BAA-9ECB-4C41-80ED-8DC52510E0A4}"/>
-    <hyperlink ref="L48" r:id="rId46" xr:uid="{E8C1A178-DA4F-4B05-A76D-351144E0C9EE}"/>
-    <hyperlink ref="L47" r:id="rId47" xr:uid="{A39623B0-D279-45D6-85E1-31AB955D11CE}"/>
-    <hyperlink ref="L46" r:id="rId48" xr:uid="{83AE49A5-F427-4C3C-8E4E-242DC5D2A5AF}"/>
-    <hyperlink ref="L45" r:id="rId49" xr:uid="{EC0B0B03-23A7-4F85-9ED1-54CB0A297766}"/>
-    <hyperlink ref="L44" r:id="rId50" xr:uid="{31DB0E58-E325-4889-9CE7-6655563392AD}"/>
-    <hyperlink ref="L43" r:id="rId51" xr:uid="{7885CACE-875F-47AD-A333-D5F2BE7CB53A}"/>
-    <hyperlink ref="L42" r:id="rId52" xr:uid="{B6324CEB-644A-4010-9BEB-3901A9D50E96}"/>
-    <hyperlink ref="L41" r:id="rId53" xr:uid="{934B93F5-8138-42E6-80D5-481369F37014}"/>
-    <hyperlink ref="L40" r:id="rId54" xr:uid="{35BD77ED-E319-4F1A-A811-144D37AAB8D6}"/>
-    <hyperlink ref="L39" r:id="rId55" xr:uid="{AC96C58D-63A8-4720-903B-4B77FAE765E0}"/>
-    <hyperlink ref="L38" r:id="rId56" xr:uid="{AE5C737D-7C90-4D7C-873F-3C60101D039A}"/>
-    <hyperlink ref="L37" r:id="rId57" xr:uid="{B05C7093-7AA4-486E-ABD2-DF7A65B8D535}"/>
+    <hyperlink ref="M15" r:id="rId1" xr:uid="{070CD713-285D-499E-AAF3-CA6E04F2E67D}"/>
+    <hyperlink ref="M16" r:id="rId2" xr:uid="{84CDC93C-1C17-4B8A-99AF-92002F858E35}"/>
+    <hyperlink ref="M17" r:id="rId3" xr:uid="{D28CC0D1-FF9B-45E5-8C06-32AA0A3E53A9}"/>
+    <hyperlink ref="M18" r:id="rId4" xr:uid="{B48EE935-D4BB-42A2-BD03-F7462BDAA973}"/>
+    <hyperlink ref="M19" r:id="rId5" xr:uid="{FC1907F3-06C3-44E2-85AA-D0706308A852}"/>
+    <hyperlink ref="M20" r:id="rId6" xr:uid="{FDA55CF4-B32E-4DB1-9DD2-2EFA7CF0ABA3}"/>
+    <hyperlink ref="M21" r:id="rId7" xr:uid="{7D576BEC-A372-4CAE-BF84-2F0963043CDC}"/>
+    <hyperlink ref="M22" r:id="rId8" xr:uid="{F23954CB-9B25-4B73-8617-4ADD50A0FE7D}"/>
+    <hyperlink ref="M24" r:id="rId9" xr:uid="{7A4658DA-5DD5-47F2-85C1-73F1BDE8C8F1}"/>
+    <hyperlink ref="M3" r:id="rId10" xr:uid="{049E9471-667A-44C7-B555-6B41CDEA4334}"/>
+    <hyperlink ref="M2" r:id="rId11" xr:uid="{A94FBB18-F767-4034-AB25-89E99187EDC8}"/>
+    <hyperlink ref="M4" r:id="rId12" xr:uid="{90B8B390-068D-4C88-BDE5-E99B638462B8}"/>
+    <hyperlink ref="M5" r:id="rId13" xr:uid="{01D903FA-154C-4673-BAA8-E8DA92B9B8EF}"/>
+    <hyperlink ref="M6" r:id="rId14" xr:uid="{682D036E-FC9A-4F6A-98CD-4CC91B1FB74F}"/>
+    <hyperlink ref="M7" r:id="rId15" xr:uid="{3F4DD620-2B56-494F-A792-A22FC9B8558D}"/>
+    <hyperlink ref="M8" r:id="rId16" xr:uid="{98CD4C7F-B63B-4FF7-9B9D-848EB9126C18}"/>
+    <hyperlink ref="M9" r:id="rId17" xr:uid="{21EFE2D2-97B6-4C85-A920-0CB2A7EC194D}"/>
+    <hyperlink ref="M10" r:id="rId18" xr:uid="{243006E2-0318-4FEE-83E6-AE585C338675}"/>
+    <hyperlink ref="M11" r:id="rId19" xr:uid="{1C7440C2-41CA-429B-80DC-4C69183A7CB9}"/>
+    <hyperlink ref="M12" r:id="rId20" xr:uid="{02E0AD7E-CEF6-4B6C-AB17-6CFDCF494509}"/>
+    <hyperlink ref="M13" r:id="rId21" xr:uid="{ABEF46E4-5EAF-4B10-9C40-A0B5F240E5BE}"/>
+    <hyperlink ref="M14" r:id="rId22" xr:uid="{B047393B-2E22-4ABF-A937-7D3E0B2FACB6}"/>
+    <hyperlink ref="M23" r:id="rId23" xr:uid="{A4B37D7B-D4FE-4B50-A01A-19BC8F084672}"/>
+    <hyperlink ref="M25" r:id="rId24" xr:uid="{46495F89-39F5-46CA-B3F0-960411F5BC3C}"/>
+    <hyperlink ref="M26" r:id="rId25" xr:uid="{5AD82D9D-0E76-446D-9312-7E6628A684B1}"/>
+    <hyperlink ref="M27" r:id="rId26" xr:uid="{C2001CED-BED9-4C03-B640-920A41146810}"/>
+    <hyperlink ref="M29" r:id="rId27" xr:uid="{DA89E417-4E4A-4547-B9AE-B031E332AA2A}"/>
+    <hyperlink ref="M28" r:id="rId28" xr:uid="{A051F0A1-FCEF-4CBB-9900-7D1A10FDEAE5}"/>
+    <hyperlink ref="M30" r:id="rId29" xr:uid="{D3924AA9-86C0-4DF6-B403-67F371618448}"/>
+    <hyperlink ref="M31" r:id="rId30" xr:uid="{FBF9CB2D-4BDE-4C09-A9B9-E188D6960A6D}"/>
+    <hyperlink ref="M32" r:id="rId31" xr:uid="{4BE15358-8230-40C1-9063-AA9B0E3B3CD2}"/>
+    <hyperlink ref="M33" r:id="rId32" xr:uid="{1F894DFD-3BA6-465A-AF03-CDD08322754B}"/>
+    <hyperlink ref="M34" r:id="rId33" xr:uid="{581D5573-91DC-48B0-B727-966BB2028F03}"/>
+    <hyperlink ref="M35" r:id="rId34" xr:uid="{A2BF5663-A951-44D0-8055-DEB448E680FA}"/>
+    <hyperlink ref="M36" r:id="rId35" xr:uid="{617F5B23-3270-413A-A61D-68FDD54E7A5D}"/>
+    <hyperlink ref="M58" r:id="rId36" xr:uid="{51AC1783-6AF1-44A4-B660-485062AF29AC}"/>
+    <hyperlink ref="M57" r:id="rId37" xr:uid="{FB7BD1A0-AC49-43FC-854E-AC6789AE027F}"/>
+    <hyperlink ref="M56" r:id="rId38" xr:uid="{39FD45C0-8BE5-49BB-820B-F4B1C9541F87}"/>
+    <hyperlink ref="M55" r:id="rId39" xr:uid="{7E342A29-2423-4FDD-810C-FE73FAB7AE34}"/>
+    <hyperlink ref="M54" r:id="rId40" xr:uid="{1E92ED11-F3F3-4DA7-9D48-EE7BC4656DBE}"/>
+    <hyperlink ref="M53" r:id="rId41" xr:uid="{23968C0E-AA65-46EC-BCA7-5E09457FFE21}"/>
+    <hyperlink ref="M52" r:id="rId42" xr:uid="{ECC4B67E-553A-48BB-AA46-D6D3B7E711A3}"/>
+    <hyperlink ref="M51" r:id="rId43" xr:uid="{EE7680E7-C97C-4D61-BAA2-B6338763FDC4}"/>
+    <hyperlink ref="M50" r:id="rId44" xr:uid="{F5DF849D-6410-4191-95D4-230AC66C7CA4}"/>
+    <hyperlink ref="M49" r:id="rId45" xr:uid="{503C1BAA-9ECB-4C41-80ED-8DC52510E0A4}"/>
+    <hyperlink ref="M48" r:id="rId46" xr:uid="{E8C1A178-DA4F-4B05-A76D-351144E0C9EE}"/>
+    <hyperlink ref="M47" r:id="rId47" xr:uid="{A39623B0-D279-45D6-85E1-31AB955D11CE}"/>
+    <hyperlink ref="M46" r:id="rId48" xr:uid="{83AE49A5-F427-4C3C-8E4E-242DC5D2A5AF}"/>
+    <hyperlink ref="M45" r:id="rId49" xr:uid="{EC0B0B03-23A7-4F85-9ED1-54CB0A297766}"/>
+    <hyperlink ref="M44" r:id="rId50" xr:uid="{31DB0E58-E325-4889-9CE7-6655563392AD}"/>
+    <hyperlink ref="M43" r:id="rId51" xr:uid="{7885CACE-875F-47AD-A333-D5F2BE7CB53A}"/>
+    <hyperlink ref="M42" r:id="rId52" xr:uid="{B6324CEB-644A-4010-9BEB-3901A9D50E96}"/>
+    <hyperlink ref="M41" r:id="rId53" xr:uid="{934B93F5-8138-42E6-80D5-481369F37014}"/>
+    <hyperlink ref="M40" r:id="rId54" xr:uid="{35BD77ED-E319-4F1A-A811-144D37AAB8D6}"/>
+    <hyperlink ref="M39" r:id="rId55" xr:uid="{AC96C58D-63A8-4720-903B-4B77FAE765E0}"/>
+    <hyperlink ref="M38" r:id="rId56" xr:uid="{AE5C737D-7C90-4D7C-873F-3C60101D039A}"/>
+    <hyperlink ref="M37" r:id="rId57" xr:uid="{B05C7093-7AA4-486E-ABD2-DF7A65B8D535}"/>
+    <hyperlink ref="M60" r:id="rId58" xr:uid="{C5EB4BB3-59E1-4C20-A245-98D06E913CD4}"/>
+    <hyperlink ref="M59" r:id="rId59" xr:uid="{FE9971B9-AD52-4DFF-86F3-668D687F4985}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId58"/>
+    <tablePart r:id="rId60"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 05/08/2026 09:24
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4369D5F5-222C-46C9-94D9-8AE6AC28548B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00669BBA-DADD-4E1A-92AB-E0E96AEAD657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="329">
   <si>
     <t>ID</t>
   </si>
@@ -1003,6 +1003,12 @@
   </si>
   <si>
     <t>Archivio Storico della Nuova Sinistra "Marco Pezzi"</t>
+  </si>
+  <si>
+    <t>Fondo Filippo Grossi</t>
+  </si>
+  <si>
+    <t>Collezione personale</t>
   </si>
 </sst>
 </file>
@@ -1517,6 +1523,9 @@
       <c r="I2" t="s">
         <v>22</v>
       </c>
+      <c r="L2" t="s">
+        <v>328</v>
+      </c>
       <c r="M2" s="4" t="s">
         <v>23</v>
       </c>
@@ -1549,6 +1558,9 @@
       <c r="I3" t="s">
         <v>27</v>
       </c>
+      <c r="L3" t="s">
+        <v>328</v>
+      </c>
       <c r="M3" s="4" t="s">
         <v>28</v>
       </c>
@@ -1581,6 +1593,9 @@
       <c r="I4" t="s">
         <v>27</v>
       </c>
+      <c r="L4" t="s">
+        <v>328</v>
+      </c>
       <c r="M4" s="4" t="s">
         <v>31</v>
       </c>
@@ -1613,6 +1628,9 @@
       <c r="I5" t="s">
         <v>34</v>
       </c>
+      <c r="L5" t="s">
+        <v>327</v>
+      </c>
       <c r="M5" s="4" t="s">
         <v>35</v>
       </c>
@@ -1645,6 +1663,9 @@
       <c r="I6" t="s">
         <v>34</v>
       </c>
+      <c r="L6" t="s">
+        <v>327</v>
+      </c>
       <c r="M6" s="4" t="s">
         <v>38</v>
       </c>
@@ -1677,6 +1698,9 @@
       <c r="I7" t="s">
         <v>27</v>
       </c>
+      <c r="L7" t="s">
+        <v>328</v>
+      </c>
       <c r="M7" s="4" t="s">
         <v>41</v>
       </c>
@@ -1709,6 +1733,9 @@
       <c r="I8" t="s">
         <v>34</v>
       </c>
+      <c r="L8" t="s">
+        <v>328</v>
+      </c>
       <c r="M8" s="4" t="s">
         <v>44</v>
       </c>
@@ -1741,6 +1768,9 @@
       <c r="I9" t="s">
         <v>34</v>
       </c>
+      <c r="L9" t="s">
+        <v>328</v>
+      </c>
       <c r="M9" s="4" t="s">
         <v>47</v>
       </c>
@@ -1773,6 +1803,9 @@
       <c r="I10" t="s">
         <v>34</v>
       </c>
+      <c r="L10" t="s">
+        <v>328</v>
+      </c>
       <c r="M10" s="4" t="s">
         <v>50</v>
       </c>
@@ -1805,6 +1838,9 @@
       <c r="I11" t="s">
         <v>34</v>
       </c>
+      <c r="L11" t="s">
+        <v>328</v>
+      </c>
       <c r="M11" s="4" t="s">
         <v>53</v>
       </c>
@@ -1840,6 +1876,9 @@
       <c r="K12" t="s">
         <v>17</v>
       </c>
+      <c r="L12" t="s">
+        <v>328</v>
+      </c>
       <c r="M12" s="4" t="s">
         <v>57</v>
       </c>
@@ -1872,6 +1911,9 @@
       <c r="I13" t="s">
         <v>34</v>
       </c>
+      <c r="L13" t="s">
+        <v>328</v>
+      </c>
       <c r="M13" s="4" t="s">
         <v>61</v>
       </c>
@@ -1910,6 +1952,9 @@
       <c r="K14" t="s">
         <v>70</v>
       </c>
+      <c r="L14" t="s">
+        <v>328</v>
+      </c>
       <c r="M14" s="4" t="s">
         <v>71</v>
       </c>
@@ -1942,6 +1987,9 @@
       <c r="J15" t="s">
         <v>76</v>
       </c>
+      <c r="L15" t="s">
+        <v>328</v>
+      </c>
       <c r="M15" s="4" t="s">
         <v>77</v>
       </c>
@@ -1977,6 +2025,9 @@
       <c r="J16" t="s">
         <v>82</v>
       </c>
+      <c r="L16" t="s">
+        <v>328</v>
+      </c>
       <c r="M16" s="4" t="s">
         <v>83</v>
       </c>
@@ -2012,6 +2063,9 @@
       <c r="J17" t="s">
         <v>87</v>
       </c>
+      <c r="L17" t="s">
+        <v>328</v>
+      </c>
       <c r="M17" s="4" t="s">
         <v>88</v>
       </c>
@@ -2044,6 +2098,9 @@
       <c r="I18" t="s">
         <v>68</v>
       </c>
+      <c r="L18" t="s">
+        <v>328</v>
+      </c>
       <c r="M18" s="4" t="s">
         <v>96</v>
       </c>
@@ -2073,6 +2130,9 @@
       <c r="I19" t="s">
         <v>68</v>
       </c>
+      <c r="L19" t="s">
+        <v>328</v>
+      </c>
       <c r="M19" s="4" t="s">
         <v>100</v>
       </c>
@@ -2102,6 +2162,9 @@
       <c r="I20" t="s">
         <v>106</v>
       </c>
+      <c r="L20" t="s">
+        <v>328</v>
+      </c>
       <c r="M20" s="4" t="s">
         <v>107</v>
       </c>
@@ -2131,6 +2194,9 @@
       <c r="I21" t="s">
         <v>106</v>
       </c>
+      <c r="L21" t="s">
+        <v>328</v>
+      </c>
       <c r="M21" s="4" t="s">
         <v>113</v>
       </c>
@@ -2457,6 +2523,9 @@
       <c r="I31" t="s">
         <v>34</v>
       </c>
+      <c r="L31" t="s">
+        <v>328</v>
+      </c>
       <c r="M31" s="4" t="s">
         <v>150</v>
       </c>
@@ -2489,6 +2558,9 @@
       <c r="I32" t="s">
         <v>34</v>
       </c>
+      <c r="L32" t="s">
+        <v>327</v>
+      </c>
       <c r="M32" s="4" t="s">
         <v>153</v>
       </c>
@@ -2515,6 +2587,9 @@
       <c r="J33" t="s">
         <v>158</v>
       </c>
+      <c r="L33" t="s">
+        <v>328</v>
+      </c>
       <c r="M33" s="4" t="s">
         <v>159</v>
       </c>
@@ -2550,6 +2625,9 @@
       <c r="K34" t="s">
         <v>17</v>
       </c>
+      <c r="L34" t="s">
+        <v>328</v>
+      </c>
       <c r="M34" s="4" t="s">
         <v>165</v>
       </c>
@@ -2591,6 +2669,9 @@
       <c r="K35" t="s">
         <v>64</v>
       </c>
+      <c r="L35" t="s">
+        <v>328</v>
+      </c>
       <c r="M35" s="4" t="s">
         <v>171</v>
       </c>
@@ -2623,6 +2704,9 @@
       <c r="I36" t="s">
         <v>68</v>
       </c>
+      <c r="L36" t="s">
+        <v>328</v>
+      </c>
       <c r="M36" s="4" t="s">
         <v>177</v>
       </c>
@@ -2658,6 +2742,9 @@
       <c r="K37" t="s">
         <v>156</v>
       </c>
+      <c r="L37" t="s">
+        <v>328</v>
+      </c>
       <c r="M37" s="4" t="s">
         <v>182</v>
       </c>
@@ -2690,6 +2777,9 @@
       <c r="I38" t="s">
         <v>34</v>
       </c>
+      <c r="L38" t="s">
+        <v>328</v>
+      </c>
       <c r="M38" s="4" t="s">
         <v>185</v>
       </c>
@@ -2725,6 +2815,9 @@
       <c r="J39" t="s">
         <v>189</v>
       </c>
+      <c r="L39" t="s">
+        <v>328</v>
+      </c>
       <c r="M39" s="4" t="s">
         <v>190</v>
       </c>
@@ -2757,6 +2850,9 @@
       <c r="I40" t="s">
         <v>193</v>
       </c>
+      <c r="L40" t="s">
+        <v>328</v>
+      </c>
       <c r="M40" s="4" t="s">
         <v>194</v>
       </c>
@@ -2789,6 +2885,9 @@
       <c r="I41" t="s">
         <v>34</v>
       </c>
+      <c r="L41" t="s">
+        <v>328</v>
+      </c>
       <c r="M41" s="4" t="s">
         <v>198</v>
       </c>
@@ -2818,6 +2917,9 @@
       <c r="I42" t="s">
         <v>202</v>
       </c>
+      <c r="L42" t="s">
+        <v>328</v>
+      </c>
       <c r="M42" s="4" t="s">
         <v>203</v>
       </c>
@@ -2853,6 +2955,9 @@
       <c r="K43" t="s">
         <v>208</v>
       </c>
+      <c r="L43" t="s">
+        <v>328</v>
+      </c>
       <c r="M43" s="4" t="s">
         <v>209</v>
       </c>
@@ -2885,6 +2990,9 @@
       <c r="I44" t="s">
         <v>27</v>
       </c>
+      <c r="L44" t="s">
+        <v>328</v>
+      </c>
       <c r="M44" s="4" t="s">
         <v>212</v>
       </c>
@@ -2917,6 +3025,9 @@
       <c r="I45" t="s">
         <v>27</v>
       </c>
+      <c r="L45" t="s">
+        <v>328</v>
+      </c>
       <c r="M45" s="4" t="s">
         <v>215</v>
       </c>
@@ -2949,6 +3060,9 @@
       <c r="I46" t="s">
         <v>27</v>
       </c>
+      <c r="L46" t="s">
+        <v>328</v>
+      </c>
       <c r="M46" s="4" t="s">
         <v>218</v>
       </c>
@@ -2981,6 +3095,9 @@
       <c r="I47" t="s">
         <v>34</v>
       </c>
+      <c r="L47" t="s">
+        <v>328</v>
+      </c>
       <c r="M47" s="4" t="s">
         <v>221</v>
       </c>
@@ -3013,6 +3130,9 @@
       <c r="I48" t="s">
         <v>34</v>
       </c>
+      <c r="L48" t="s">
+        <v>328</v>
+      </c>
       <c r="M48" s="4" t="s">
         <v>224</v>
       </c>
@@ -3045,6 +3165,9 @@
       <c r="I49" t="s">
         <v>27</v>
       </c>
+      <c r="L49" t="s">
+        <v>328</v>
+      </c>
       <c r="M49" s="4" t="s">
         <v>227</v>
       </c>
@@ -3077,6 +3200,9 @@
       <c r="I50" t="s">
         <v>27</v>
       </c>
+      <c r="L50" t="s">
+        <v>328</v>
+      </c>
       <c r="M50" s="4" t="s">
         <v>230</v>
       </c>
@@ -3109,6 +3235,9 @@
       <c r="I51" t="s">
         <v>27</v>
       </c>
+      <c r="L51" t="s">
+        <v>328</v>
+      </c>
       <c r="M51" s="4" t="s">
         <v>233</v>
       </c>
@@ -3141,6 +3270,9 @@
       <c r="I52" t="s">
         <v>34</v>
       </c>
+      <c r="L52" t="s">
+        <v>328</v>
+      </c>
       <c r="M52" s="4" t="s">
         <v>236</v>
       </c>
@@ -3173,6 +3305,9 @@
       <c r="I53" t="s">
         <v>68</v>
       </c>
+      <c r="L53" t="s">
+        <v>328</v>
+      </c>
       <c r="M53" s="4" t="s">
         <v>241</v>
       </c>
@@ -3202,6 +3337,9 @@
       <c r="K54" t="s">
         <v>245</v>
       </c>
+      <c r="L54" t="s">
+        <v>328</v>
+      </c>
       <c r="M54" s="4" t="s">
         <v>246</v>
       </c>
@@ -3237,6 +3375,9 @@
       <c r="J55" t="s">
         <v>252</v>
       </c>
+      <c r="L55" t="s">
+        <v>328</v>
+      </c>
       <c r="M55" s="4" t="s">
         <v>253</v>
       </c>
@@ -3269,6 +3410,9 @@
       <c r="I56" t="s">
         <v>68</v>
       </c>
+      <c r="L56" t="s">
+        <v>328</v>
+      </c>
       <c r="M56" s="4" t="s">
         <v>257</v>
       </c>
@@ -3304,6 +3448,9 @@
       <c r="I57" t="s">
         <v>202</v>
       </c>
+      <c r="L57" t="s">
+        <v>328</v>
+      </c>
       <c r="M57" s="4" t="s">
         <v>261</v>
       </c>
@@ -3342,6 +3489,9 @@
       <c r="K58" t="s">
         <v>263</v>
       </c>
+      <c r="L58" t="s">
+        <v>328</v>
+      </c>
       <c r="M58" s="4" t="s">
         <v>264</v>
       </c>
@@ -3377,6 +3527,9 @@
       <c r="I59" t="s">
         <v>106</v>
       </c>
+      <c r="L59" t="s">
+        <v>328</v>
+      </c>
       <c r="M59" s="4" t="s">
         <v>324</v>
       </c>
@@ -3408,6 +3561,9 @@
       </c>
       <c r="I60" t="s">
         <v>106</v>
+      </c>
+      <c r="L60" t="s">
+        <v>328</v>
       </c>
       <c r="M60" s="4" t="s">
         <v>323</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 05/08/2026 11:34
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00669BBA-DADD-4E1A-92AB-E0E96AEAD657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B45408-4720-4088-991D-E0F8D9E118BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="334">
   <si>
     <t>ID</t>
   </si>
@@ -363,9 +363,6 @@
     <t>Bologna</t>
   </si>
   <si>
-    <t>https://archive.org/details/ribellarsi-e-giusto//mode/2up</t>
-  </si>
-  <si>
     <t>AMI-0021</t>
   </si>
   <si>
@@ -396,9 +393,6 @@
     <t>Lavoro Politico no. 2</t>
   </si>
   <si>
-    <t>https://archive.org/details/lavoro-politico-02//mode/2up</t>
-  </si>
-  <si>
     <t>AMI-0023</t>
   </si>
   <si>
@@ -432,9 +426,6 @@
     <t>Lavoro Politico no. 7</t>
   </si>
   <si>
-    <t>https://archive.org/details/lavoro-politico-07//mode/2up</t>
-  </si>
-  <si>
     <t>AMI-0027</t>
   </si>
   <si>
@@ -1009,6 +1000,30 @@
   </si>
   <si>
     <t>Collezione personale</t>
+  </si>
+  <si>
+    <t>AMI-0060</t>
+  </si>
+  <si>
+    <t>Come diventare un buon comunista</t>
+  </si>
+  <si>
+    <t>Liu Shaoqi</t>
+  </si>
+  <si>
+    <t>Arnaldo Bressan</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/come-diventare-un-buon-comunista/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lavoro-politico-02/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lavoro-politico-07/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/ribellarsi-e-giusto/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -1430,7 +1445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -1480,7 +1495,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="M1" t="s">
         <v>11</v>
@@ -1524,7 +1539,7 @@
         <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>23</v>
@@ -1559,7 +1574,7 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>28</v>
@@ -1594,7 +1609,7 @@
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>31</v>
@@ -1629,7 +1644,7 @@
         <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>35</v>
@@ -1664,7 +1679,7 @@
         <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="M6" s="4" t="s">
         <v>38</v>
@@ -1699,7 +1714,7 @@
         <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>41</v>
@@ -1734,7 +1749,7 @@
         <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>44</v>
@@ -1769,7 +1784,7 @@
         <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>47</v>
@@ -1804,7 +1819,7 @@
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>50</v>
@@ -1839,7 +1854,7 @@
         <v>34</v>
       </c>
       <c r="L11" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>53</v>
@@ -1877,7 +1892,7 @@
         <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>57</v>
@@ -1912,7 +1927,7 @@
         <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>61</v>
@@ -1953,7 +1968,7 @@
         <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>71</v>
@@ -1988,7 +2003,7 @@
         <v>76</v>
       </c>
       <c r="L15" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M15" s="4" t="s">
         <v>77</v>
@@ -2026,7 +2041,7 @@
         <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M16" s="4" t="s">
         <v>83</v>
@@ -2064,7 +2079,7 @@
         <v>87</v>
       </c>
       <c r="L17" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M17" s="4" t="s">
         <v>88</v>
@@ -2099,7 +2114,7 @@
         <v>68</v>
       </c>
       <c r="L18" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M18" s="4" t="s">
         <v>96</v>
@@ -2131,7 +2146,7 @@
         <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M19" s="4" t="s">
         <v>100</v>
@@ -2163,7 +2178,7 @@
         <v>106</v>
       </c>
       <c r="L20" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M20" s="4" t="s">
         <v>107</v>
@@ -2195,318 +2210,318 @@
         <v>106</v>
       </c>
       <c r="L21" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>113</v>
+        <v>333</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
         <v>114</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>115</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>116</v>
-      </c>
-      <c r="E22" t="s">
-        <v>117</v>
       </c>
       <c r="F22" s="3">
         <v>24746</v>
       </c>
       <c r="G22" t="s">
+        <v>117</v>
+      </c>
+      <c r="H22" t="s">
         <v>118</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>119</v>
       </c>
-      <c r="I22" t="s">
+      <c r="L22" t="s">
+        <v>323</v>
+      </c>
+      <c r="M22" s="4" t="s">
         <v>120</v>
-      </c>
-      <c r="L22" t="s">
-        <v>326</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" t="s">
         <v>122</v>
       </c>
-      <c r="B23" t="s">
-        <v>123</v>
-      </c>
       <c r="C23" t="s">
+        <v>115</v>
+      </c>
+      <c r="E23" t="s">
         <v>116</v>
-      </c>
-      <c r="E23" t="s">
-        <v>117</v>
       </c>
       <c r="F23" s="3">
         <v>24777</v>
       </c>
       <c r="G23" t="s">
+        <v>117</v>
+      </c>
+      <c r="H23" t="s">
         <v>118</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>119</v>
       </c>
-      <c r="I23" t="s">
-        <v>120</v>
-      </c>
       <c r="L23" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>124</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C24" t="s">
+        <v>115</v>
+      </c>
+      <c r="E24" t="s">
         <v>116</v>
-      </c>
-      <c r="E24" t="s">
-        <v>117</v>
       </c>
       <c r="F24" s="3">
         <v>24838</v>
       </c>
       <c r="G24" t="s">
+        <v>117</v>
+      </c>
+      <c r="H24" t="s">
         <v>118</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>119</v>
       </c>
-      <c r="I24" t="s">
-        <v>120</v>
-      </c>
       <c r="L24" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C25" t="s">
+        <v>115</v>
+      </c>
+      <c r="E25" t="s">
         <v>116</v>
-      </c>
-      <c r="E25" t="s">
-        <v>117</v>
       </c>
       <c r="F25" s="3">
         <v>24869</v>
       </c>
       <c r="G25" t="s">
+        <v>117</v>
+      </c>
+      <c r="H25" t="s">
         <v>118</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>119</v>
       </c>
-      <c r="I25" t="s">
-        <v>120</v>
-      </c>
       <c r="L25" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M25" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C26" t="s">
+        <v>115</v>
+      </c>
+      <c r="E26" t="s">
         <v>116</v>
-      </c>
-      <c r="E26" t="s">
-        <v>117</v>
       </c>
       <c r="F26" s="3">
         <v>24898</v>
       </c>
       <c r="G26" t="s">
+        <v>117</v>
+      </c>
+      <c r="H26" t="s">
         <v>118</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>119</v>
       </c>
-      <c r="I26" t="s">
-        <v>120</v>
-      </c>
       <c r="L26" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B27" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C27" t="s">
+        <v>115</v>
+      </c>
+      <c r="E27" t="s">
         <v>116</v>
-      </c>
-      <c r="E27" t="s">
-        <v>117</v>
       </c>
       <c r="F27" s="3">
         <v>24959</v>
       </c>
       <c r="G27" t="s">
+        <v>117</v>
+      </c>
+      <c r="H27" t="s">
         <v>118</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>119</v>
       </c>
-      <c r="I27" t="s">
-        <v>120</v>
-      </c>
       <c r="L27" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M27" s="4" t="s">
-        <v>136</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B28" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C28" t="s">
+        <v>115</v>
+      </c>
+      <c r="E28" t="s">
         <v>116</v>
-      </c>
-      <c r="E28" t="s">
-        <v>117</v>
       </c>
       <c r="F28" s="3">
         <v>24990</v>
       </c>
       <c r="G28" t="s">
+        <v>117</v>
+      </c>
+      <c r="H28" t="s">
         <v>118</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>119</v>
       </c>
-      <c r="I28" t="s">
-        <v>120</v>
-      </c>
       <c r="L28" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C29" t="s">
+        <v>115</v>
+      </c>
+      <c r="E29" t="s">
         <v>116</v>
-      </c>
-      <c r="E29" t="s">
-        <v>117</v>
       </c>
       <c r="F29" s="3">
         <v>25082</v>
       </c>
       <c r="G29" t="s">
+        <v>117</v>
+      </c>
+      <c r="H29" t="s">
         <v>118</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>119</v>
-      </c>
-      <c r="I29" t="s">
-        <v>120</v>
       </c>
       <c r="K29" t="s">
         <v>64</v>
       </c>
       <c r="L29" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C30" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" t="s">
         <v>116</v>
-      </c>
-      <c r="E30" t="s">
-        <v>117</v>
       </c>
       <c r="F30" s="3">
         <v>25173</v>
       </c>
       <c r="G30" t="s">
+        <v>117</v>
+      </c>
+      <c r="H30" t="s">
         <v>118</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>119</v>
       </c>
-      <c r="I30" t="s">
-        <v>120</v>
-      </c>
       <c r="K30" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="L30" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="M30" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C31" t="s">
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E31" t="s">
         <v>19</v>
@@ -2524,18 +2539,18 @@
         <v>34</v>
       </c>
       <c r="L31" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B32" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C32" t="s">
         <v>17</v>
@@ -2559,50 +2574,50 @@
         <v>34</v>
       </c>
       <c r="L32" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B33" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C33" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F33" s="1">
         <v>1970</v>
       </c>
       <c r="G33" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I33" t="s">
         <v>68</v>
       </c>
       <c r="J33" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="L33" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M33" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="N33" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B34" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C34" t="s">
         <v>64</v>
@@ -2611,7 +2626,7 @@
         <v>25063</v>
       </c>
       <c r="G34" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H34" t="s">
         <v>21</v>
@@ -2620,30 +2635,30 @@
         <v>68</v>
       </c>
       <c r="J34" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K34" t="s">
         <v>17</v>
       </c>
       <c r="L34" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M34" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="O34" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="P34" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B35" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
@@ -2655,7 +2670,7 @@
         <v>25081</v>
       </c>
       <c r="G35" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H35" t="s">
         <v>21</v>
@@ -2664,30 +2679,30 @@
         <v>68</v>
       </c>
       <c r="J35" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K35" t="s">
         <v>64</v>
       </c>
       <c r="L35" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M35" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="O35" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="P35" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B36" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C36" t="s">
         <v>92</v>
@@ -2696,36 +2711,36 @@
         <v>25416</v>
       </c>
       <c r="G36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H36" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I36" t="s">
         <v>68</v>
       </c>
       <c r="L36" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B37" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C37" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D37" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E37" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F37" s="1">
         <v>1975</v>
@@ -2734,27 +2749,27 @@
         <v>20</v>
       </c>
       <c r="H37" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I37" t="s">
         <v>106</v>
       </c>
       <c r="K37" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="L37" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M37" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B38" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C38" t="s">
         <v>17</v>
@@ -2778,24 +2793,24 @@
         <v>34</v>
       </c>
       <c r="L38" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M38" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B39" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C39" t="s">
         <v>17</v>
       </c>
       <c r="D39" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E39" t="s">
         <v>19</v>
@@ -2813,21 +2828,21 @@
         <v>34</v>
       </c>
       <c r="J39" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="L39" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M39" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B40" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C40" t="s">
         <v>17</v>
@@ -2848,27 +2863,27 @@
         <v>21</v>
       </c>
       <c r="I40" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="L40" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B41" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E41" t="s">
         <v>19</v>
@@ -2886,24 +2901,24 @@
         <v>34</v>
       </c>
       <c r="L41" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M41" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B42" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
       </c>
       <c r="E42" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F42" s="1">
         <v>1968</v>
@@ -2912,30 +2927,30 @@
         <v>20</v>
       </c>
       <c r="H42" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I42" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L42" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M42" s="4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B43" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
       </c>
       <c r="E43" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F43" s="1">
         <v>1967</v>
@@ -2944,30 +2959,30 @@
         <v>20</v>
       </c>
       <c r="H43" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I43" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="J43" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="K43" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="L43" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B44" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C44" t="s">
         <v>17</v>
@@ -2991,18 +3006,18 @@
         <v>27</v>
       </c>
       <c r="L44" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M44" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B45" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C45" t="s">
         <v>17</v>
@@ -3026,18 +3041,18 @@
         <v>27</v>
       </c>
       <c r="L45" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M45" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B46" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C46" t="s">
         <v>17</v>
@@ -3061,18 +3076,18 @@
         <v>27</v>
       </c>
       <c r="L46" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M46" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B47" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C47" t="s">
         <v>17</v>
@@ -3096,18 +3111,18 @@
         <v>34</v>
       </c>
       <c r="L47" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M47" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B48" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C48" t="s">
         <v>17</v>
@@ -3131,18 +3146,18 @@
         <v>34</v>
       </c>
       <c r="L48" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M48" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B49" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C49" t="s">
         <v>17</v>
@@ -3166,18 +3181,18 @@
         <v>27</v>
       </c>
       <c r="L49" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M49" s="4" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B50" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C50" t="s">
         <v>17</v>
@@ -3201,18 +3216,18 @@
         <v>27</v>
       </c>
       <c r="L50" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M50" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B51" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C51" t="s">
         <v>17</v>
@@ -3236,18 +3251,18 @@
         <v>27</v>
       </c>
       <c r="L51" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M51" s="4" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B52" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C52" t="s">
         <v>17</v>
@@ -3271,27 +3286,27 @@
         <v>34</v>
       </c>
       <c r="L52" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M52" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>234</v>
+      </c>
+      <c r="B53" t="s">
+        <v>235</v>
+      </c>
+      <c r="C53" t="s">
+        <v>236</v>
+      </c>
+      <c r="D53" t="s">
+        <v>236</v>
+      </c>
+      <c r="E53" t="s">
         <v>237</v>
-      </c>
-      <c r="B53" t="s">
-        <v>238</v>
-      </c>
-      <c r="C53" t="s">
-        <v>239</v>
-      </c>
-      <c r="D53" t="s">
-        <v>239</v>
-      </c>
-      <c r="E53" t="s">
-        <v>240</v>
       </c>
       <c r="F53" s="1">
         <v>1969</v>
@@ -3300,24 +3315,24 @@
         <v>20</v>
       </c>
       <c r="H53" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I53" t="s">
         <v>68</v>
       </c>
       <c r="L53" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M53" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B54" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C54" t="s">
         <v>92</v>
@@ -3329,68 +3344,68 @@
         <v>94</v>
       </c>
       <c r="H54" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="I54" t="s">
         <v>68</v>
       </c>
       <c r="K54" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="L54" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M54" s="4" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>244</v>
+      </c>
+      <c r="B55" t="s">
+        <v>245</v>
+      </c>
+      <c r="C55" t="s">
+        <v>246</v>
+      </c>
+      <c r="D55" t="s">
+        <v>246</v>
+      </c>
+      <c r="E55" t="s">
         <v>247</v>
-      </c>
-      <c r="B55" t="s">
-        <v>248</v>
-      </c>
-      <c r="C55" t="s">
-        <v>249</v>
-      </c>
-      <c r="D55" t="s">
-        <v>249</v>
-      </c>
-      <c r="E55" t="s">
-        <v>250</v>
       </c>
       <c r="F55" s="3">
         <v>28550</v>
       </c>
       <c r="G55" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="H55" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I55" t="s">
         <v>68</v>
       </c>
       <c r="J55" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="L55" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M55" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="N55" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B56" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C56" t="s">
         <v>64</v>
@@ -3405,27 +3420,27 @@
         <v>1967</v>
       </c>
       <c r="G56" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I56" t="s">
         <v>68</v>
       </c>
       <c r="L56" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M56" s="4" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="N56" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B57" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C57" t="s">
         <v>99</v>
@@ -3443,33 +3458,33 @@
         <v>20</v>
       </c>
       <c r="H57" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I57" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L57" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M57" s="4" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B58" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C58" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D58" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E58" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F58" s="2">
         <v>28253</v>
@@ -3478,39 +3493,39 @@
         <v>75</v>
       </c>
       <c r="H58" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I58" t="s">
         <v>68</v>
       </c>
       <c r="J58" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="K58" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="L58" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M58" s="4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="N58" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>315</v>
+      </c>
+      <c r="B59" t="s">
         <v>318</v>
-      </c>
-      <c r="B59" t="s">
-        <v>321</v>
       </c>
       <c r="C59" t="s">
         <v>99</v>
       </c>
       <c r="D59" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E59" t="s">
         <v>99</v>
@@ -3522,30 +3537,30 @@
         <v>20</v>
       </c>
       <c r="H59" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I59" t="s">
         <v>106</v>
       </c>
       <c r="L59" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="M59" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B60" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C60" t="s">
         <v>99</v>
       </c>
       <c r="D60" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E60" t="s">
         <v>99</v>
@@ -3557,16 +3572,54 @@
         <v>20</v>
       </c>
       <c r="H60" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I60" t="s">
         <v>106</v>
       </c>
       <c r="L60" t="s">
+        <v>325</v>
+      </c>
+      <c r="M60" s="4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>326</v>
+      </c>
+      <c r="B61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C61" t="s">
+        <v>99</v>
+      </c>
+      <c r="D61" t="s">
         <v>328</v>
       </c>
-      <c r="M60" s="4" t="s">
-        <v>323</v>
+      <c r="E61" t="s">
+        <v>99</v>
+      </c>
+      <c r="F61">
+        <v>1965</v>
+      </c>
+      <c r="G61" t="s">
+        <v>20</v>
+      </c>
+      <c r="H61" t="s">
+        <v>173</v>
+      </c>
+      <c r="I61" t="s">
+        <v>106</v>
+      </c>
+      <c r="J61" t="s">
+        <v>329</v>
+      </c>
+      <c r="L61" t="s">
+        <v>325</v>
+      </c>
+      <c r="M61" s="4" t="s">
+        <v>330</v>
       </c>
     </row>
   </sheetData>
@@ -3631,10 +3684,11 @@
     <hyperlink ref="M37" r:id="rId57" xr:uid="{B05C7093-7AA4-486E-ABD2-DF7A65B8D535}"/>
     <hyperlink ref="M60" r:id="rId58" xr:uid="{C5EB4BB3-59E1-4C20-A245-98D06E913CD4}"/>
     <hyperlink ref="M59" r:id="rId59" xr:uid="{FE9971B9-AD52-4DFF-86F3-668D687F4985}"/>
+    <hyperlink ref="M61" r:id="rId60" xr:uid="{84225D9C-CA52-466B-B2BD-B20C11AFA762}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId60"/>
+    <tablePart r:id="rId61"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3649,19 +3703,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D1" t="s">
         <v>266</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>267</v>
-      </c>
-      <c r="C1" t="s">
-        <v>268</v>
-      </c>
-      <c r="D1" t="s">
-        <v>269</v>
-      </c>
-      <c r="E1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -3669,7 +3723,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C2">
         <v>1893</v>
@@ -3678,15 +3732,15 @@
         <v>1976</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B3" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C3">
         <v>1921</v>
@@ -3695,24 +3749,24 @@
         <v>1993</v>
       </c>
       <c r="E3" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C4" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D4">
         <v>2021</v>
       </c>
       <c r="E4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -3720,7 +3774,7 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C5">
         <v>1931</v>
@@ -3731,10 +3785,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B6" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C6">
         <v>1960</v>
@@ -3745,26 +3799,26 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B8" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B9" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C9">
         <v>1907</v>
@@ -3775,10 +3829,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B10" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C10">
         <v>1898</v>
@@ -3789,10 +3843,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B11" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C11">
         <v>1898</v>
@@ -3803,10 +3857,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B12" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C12">
         <v>1904</v>
@@ -3817,10 +3871,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B13" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C13">
         <v>1914</v>
@@ -3831,10 +3885,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B14" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C14">
         <v>1920</v>
@@ -3845,10 +3899,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B15" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C15">
         <v>1920</v>
@@ -3875,33 +3929,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E1" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C2">
         <v>1962</v>
       </c>
       <c r="D2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -3909,7 +3963,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C3">
         <v>1952</v>
@@ -3920,7 +3974,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C4">
         <v>1963</v>
@@ -3934,7 +3988,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C5">
         <v>1948</v>
@@ -3942,10 +3996,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B6" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C6">
         <v>1958</v>
@@ -3959,7 +4013,7 @@
         <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C7">
         <v>1964</v>
@@ -3970,10 +4024,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B8" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C8">
         <v>1956</v>
@@ -3981,10 +4035,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -3992,7 +4046,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C10">
         <v>1966</v>
@@ -4006,7 +4060,7 @@
         <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C11">
         <v>1968</v>
@@ -4017,10 +4071,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B12" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C12">
         <v>1966</v>
@@ -4031,10 +4085,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B13" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C13">
         <v>1921</v>
@@ -4045,7 +4099,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C14">
         <v>1966</v>
@@ -4054,7 +4108,7 @@
         <v>1991</v>
       </c>
       <c r="E14" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -4062,7 +4116,7 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C15">
         <v>1968</v>
@@ -4071,7 +4125,7 @@
         <v>1972</v>
       </c>
       <c r="E15" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -4079,21 +4133,21 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C16">
         <v>1921</v>
       </c>
       <c r="E16" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B17" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C17">
         <v>1968</v>
@@ -4104,10 +4158,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B18" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C18">
         <v>1969</v>
@@ -4118,24 +4172,24 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B19" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C19">
         <v>1968</v>
       </c>
       <c r="D19" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B20" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C20">
         <v>1972</v>
@@ -4146,10 +4200,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B21" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C21">
         <v>1967</v>
@@ -4160,10 +4214,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B22" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C22">
         <v>1977</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 05/08/2026 17:37
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B45408-4720-4088-991D-E0F8D9E118BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA960BE5-19A6-42C5-887F-1740A129CBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="335">
   <si>
     <t>ID</t>
   </si>
@@ -1024,6 +1024,9 @@
   </si>
   <si>
     <t>https://archive.org/details/ribellarsi-e-giusto/mode/2up</t>
+  </si>
+  <si>
+    <t>Liu</t>
   </si>
 </sst>
 </file>
@@ -3695,10 +3698,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="5" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -3909,6 +3913,20 @@
       </c>
       <c r="D15">
         <v>1997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>328</v>
+      </c>
+      <c r="B16" t="s">
+        <v>334</v>
+      </c>
+      <c r="C16">
+        <v>1898</v>
+      </c>
+      <c r="D16">
+        <v>1969</v>
       </c>
     </row>
   </sheetData>
@@ -3924,7 +3942,8 @@
   <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="50.33203125" customWidth="1"/>
+    <col min="2" max="5" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 10/08/2026 16:26
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA960BE5-19A6-42C5-887F-1740A129CBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE82C6C8-A61B-47FC-BC3E-AE0A23207CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="338">
   <si>
     <t>ID</t>
   </si>
@@ -1027,6 +1027,15 @@
   </si>
   <si>
     <t>Liu</t>
+  </si>
+  <si>
+    <t>AMI-0061</t>
+  </si>
+  <si>
+    <t>Sulla guerra di lunga durata</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/guerra-di-lunga-durata/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -1448,7 +1457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -3623,6 +3632,41 @@
       </c>
       <c r="M61" s="4" t="s">
         <v>330</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>335</v>
+      </c>
+      <c r="B62" t="s">
+        <v>336</v>
+      </c>
+      <c r="C62" t="s">
+        <v>17</v>
+      </c>
+      <c r="D62" t="s">
+        <v>18</v>
+      </c>
+      <c r="E62" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" s="1">
+        <v>1971</v>
+      </c>
+      <c r="G62" t="s">
+        <v>26</v>
+      </c>
+      <c r="H62" t="s">
+        <v>21</v>
+      </c>
+      <c r="I62" t="s">
+        <v>27</v>
+      </c>
+      <c r="L62" t="s">
+        <v>325</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -3688,10 +3732,11 @@
     <hyperlink ref="M60" r:id="rId58" xr:uid="{C5EB4BB3-59E1-4C20-A245-98D06E913CD4}"/>
     <hyperlink ref="M59" r:id="rId59" xr:uid="{FE9971B9-AD52-4DFF-86F3-668D687F4985}"/>
     <hyperlink ref="M61" r:id="rId60" xr:uid="{84225D9C-CA52-466B-B2BD-B20C11AFA762}"/>
+    <hyperlink ref="M62" r:id="rId61" xr:uid="{7C0E21C7-5F11-4346-9647-7720BC7FADE0}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId61"/>
+    <tablePart r:id="rId62"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 11/08/2026 14:46
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE82C6C8-A61B-47FC-BC3E-AE0A23207CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A4763E-F23E-42EB-9697-5E39C4F76C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="343">
   <si>
     <t>ID</t>
   </si>
@@ -1036,6 +1036,21 @@
   </si>
   <si>
     <t>https://archive.org/details/guerra-di-lunga-durata/mode/2up</t>
+  </si>
+  <si>
+    <t>AMI-0062</t>
+  </si>
+  <si>
+    <t>Delegazione del movimento studentesco dell'Università di Trieste sulla nave cinese Jinsha</t>
+  </si>
+  <si>
+    <t>Trieste</t>
+  </si>
+  <si>
+    <t>Partito Comunista d'Italia (marxista-leninista); Movimento Studentesco</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1968-delegazione-nave-jinsha</t>
   </si>
 </sst>
 </file>
@@ -1095,12 +1110,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1457,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -3667,6 +3683,35 @@
       </c>
       <c r="M62" s="4" t="s">
         <v>337</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>338</v>
+      </c>
+      <c r="B63" t="s">
+        <v>339</v>
+      </c>
+      <c r="F63" s="5">
+        <v>24917</v>
+      </c>
+      <c r="G63" t="s">
+        <v>75</v>
+      </c>
+      <c r="H63" t="s">
+        <v>340</v>
+      </c>
+      <c r="I63" t="s">
+        <v>106</v>
+      </c>
+      <c r="K63" t="s">
+        <v>341</v>
+      </c>
+      <c r="L63" t="s">
+        <v>325</v>
+      </c>
+      <c r="M63" s="4" t="s">
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -3733,10 +3778,11 @@
     <hyperlink ref="M59" r:id="rId59" xr:uid="{FE9971B9-AD52-4DFF-86F3-668D687F4985}"/>
     <hyperlink ref="M61" r:id="rId60" xr:uid="{84225D9C-CA52-466B-B2BD-B20C11AFA762}"/>
     <hyperlink ref="M62" r:id="rId61" xr:uid="{7C0E21C7-5F11-4346-9647-7720BC7FADE0}"/>
+    <hyperlink ref="M63" r:id="rId62" xr:uid="{5EE44639-4FF3-43AB-A33E-7E859265AB4E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId62"/>
+    <tablePart r:id="rId63"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 11/08/2026 14:50
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A4763E-F23E-42EB-9697-5E39C4F76C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED8B864-D41A-4D17-87CB-433851432866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="344">
   <si>
     <t>ID</t>
   </si>
@@ -1051,6 +1051,9 @@
   </si>
   <si>
     <t>https://archive.org/details/1968-delegazione-nave-jinsha</t>
+  </si>
+  <si>
+    <t>1968-Delegazione-Nave-Jinsha.png</t>
   </si>
 </sst>
 </file>
@@ -3713,6 +3716,9 @@
       <c r="M63" s="4" t="s">
         <v>342</v>
       </c>
+      <c r="N63" t="s">
+        <v>343</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 12/08/2026 17:16
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED8B864-D41A-4D17-87CB-433851432866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE9E9A3-E90F-4A8C-AA1F-83511EDBA163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="355">
   <si>
     <t>ID</t>
   </si>
@@ -1054,6 +1054,39 @@
   </si>
   <si>
     <t>1968-Delegazione-Nave-Jinsha.png</t>
+  </si>
+  <si>
+    <t>AMI-0063</t>
+  </si>
+  <si>
+    <t>AMI-0064</t>
+  </si>
+  <si>
+    <t>Brindisi</t>
+  </si>
+  <si>
+    <t>Archivio Storico Benedetto Petrone</t>
+  </si>
+  <si>
+    <t>Organizzazione Comunista (marxista-leninista) Fronte Unito</t>
+  </si>
+  <si>
+    <t>Volantino del PC(m-l)I contro il carovita sotto il governo Rumor</t>
+  </si>
+  <si>
+    <t>Volantino dell'OC(m-l) - Fronte Unito contro l'aumento del costo della benzina</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1974-volantino-contro-rumor</t>
+  </si>
+  <si>
+    <t>1974-Volantino-contro-rumor.jpg</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1973-volantino-anti-rumor-ocm-l</t>
+  </si>
+  <si>
+    <t>1973-Volantino-anti-rumor-OC(m-l).jpg</t>
   </si>
 </sst>
 </file>
@@ -1113,13 +1146,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1476,7 +1510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -3718,6 +3752,76 @@
       </c>
       <c r="N63" t="s">
         <v>343</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>344</v>
+      </c>
+      <c r="B64" t="s">
+        <v>349</v>
+      </c>
+      <c r="C64" t="s">
+        <v>242</v>
+      </c>
+      <c r="D64" t="s">
+        <v>242</v>
+      </c>
+      <c r="F64" s="6">
+        <v>27030</v>
+      </c>
+      <c r="G64" t="s">
+        <v>94</v>
+      </c>
+      <c r="H64" t="s">
+        <v>346</v>
+      </c>
+      <c r="I64" t="s">
+        <v>68</v>
+      </c>
+      <c r="L64" t="s">
+        <v>347</v>
+      </c>
+      <c r="M64" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="N64" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>345</v>
+      </c>
+      <c r="B65" t="s">
+        <v>350</v>
+      </c>
+      <c r="C65" t="s">
+        <v>348</v>
+      </c>
+      <c r="D65" t="s">
+        <v>348</v>
+      </c>
+      <c r="F65" s="5">
+        <v>26956</v>
+      </c>
+      <c r="G65" t="s">
+        <v>94</v>
+      </c>
+      <c r="H65" t="s">
+        <v>346</v>
+      </c>
+      <c r="I65" t="s">
+        <v>68</v>
+      </c>
+      <c r="L65" t="s">
+        <v>347</v>
+      </c>
+      <c r="M65" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="N65" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -3785,10 +3889,12 @@
     <hyperlink ref="M61" r:id="rId60" xr:uid="{84225D9C-CA52-466B-B2BD-B20C11AFA762}"/>
     <hyperlink ref="M62" r:id="rId61" xr:uid="{7C0E21C7-5F11-4346-9647-7720BC7FADE0}"/>
     <hyperlink ref="M63" r:id="rId62" xr:uid="{5EE44639-4FF3-43AB-A33E-7E859265AB4E}"/>
+    <hyperlink ref="M64" r:id="rId63" xr:uid="{5D3389C0-C71F-4CF3-93D8-DFF5AF7892D2}"/>
+    <hyperlink ref="M65" r:id="rId64" xr:uid="{705AEFBC-C508-48F1-BEC0-89DB7C3BD430}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId63"/>
+    <tablePart r:id="rId65"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 16/08/2026 19:03
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE9E9A3-E90F-4A8C-AA1F-83511EDBA163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AA779D-F0D3-4707-A88F-C320A5390674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="365">
   <si>
     <t>ID</t>
   </si>
@@ -1087,6 +1087,36 @@
   </si>
   <si>
     <t>1973-Volantino-anti-rumor-OC(m-l).jpg</t>
+  </si>
+  <si>
+    <t>AMI-0065</t>
+  </si>
+  <si>
+    <t>Manifestazione del Partito Comunista d'Italia (marxista-leninista)</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1968.manifestazione.PCDI</t>
+  </si>
+  <si>
+    <t>1968.Manifestazione.PCDI.jpg</t>
+  </si>
+  <si>
+    <t>AMI-0066</t>
+  </si>
+  <si>
+    <t>Manifestazione del Movimento Studentesco</t>
+  </si>
+  <si>
+    <t>Movimento Studentesco</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1970-movimento-studentesco-pensierodi-mao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                           </t>
+  </si>
+  <si>
+    <t>1970.Movimento.Studentesco.PensierodiMao.jpg</t>
   </si>
 </sst>
 </file>
@@ -1510,7 +1540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -3822,6 +3852,75 @@
       </c>
       <c r="N65" t="s">
         <v>354</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>355</v>
+      </c>
+      <c r="B66" t="s">
+        <v>356</v>
+      </c>
+      <c r="C66" t="s">
+        <v>64</v>
+      </c>
+      <c r="F66">
+        <v>1968</v>
+      </c>
+      <c r="G66" t="s">
+        <v>75</v>
+      </c>
+      <c r="H66" t="s">
+        <v>173</v>
+      </c>
+      <c r="I66" t="s">
+        <v>68</v>
+      </c>
+      <c r="L66" t="s">
+        <v>325</v>
+      </c>
+      <c r="M66" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="N66" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>359</v>
+      </c>
+      <c r="B67" t="s">
+        <v>360</v>
+      </c>
+      <c r="C67" t="s">
+        <v>361</v>
+      </c>
+      <c r="F67">
+        <v>1970</v>
+      </c>
+      <c r="G67" t="s">
+        <v>75</v>
+      </c>
+      <c r="H67" t="s">
+        <v>173</v>
+      </c>
+      <c r="I67" t="s">
+        <v>68</v>
+      </c>
+      <c r="L67" t="s">
+        <v>325</v>
+      </c>
+      <c r="M67" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="N67" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N68" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -3891,10 +3990,12 @@
     <hyperlink ref="M63" r:id="rId62" xr:uid="{5EE44639-4FF3-43AB-A33E-7E859265AB4E}"/>
     <hyperlink ref="M64" r:id="rId63" xr:uid="{5D3389C0-C71F-4CF3-93D8-DFF5AF7892D2}"/>
     <hyperlink ref="M65" r:id="rId64" xr:uid="{705AEFBC-C508-48F1-BEC0-89DB7C3BD430}"/>
+    <hyperlink ref="M66" r:id="rId65" xr:uid="{8365E924-D46C-4D93-9FDD-E2A533CDCEF8}"/>
+    <hyperlink ref="M67" r:id="rId66" xr:uid="{9E0E6191-2474-42FA-BA40-68DA6CAC11D8}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId65"/>
+    <tablePart r:id="rId67"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 16/08/2026 19:08
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AA779D-F0D3-4707-A88F-C320A5390674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FC96FF-B201-455B-BA3D-74A451EFB80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -1098,9 +1098,6 @@
     <t>https://archive.org/details/1968.manifestazione.PCDI</t>
   </si>
   <si>
-    <t>1968.Manifestazione.PCDI.jpg</t>
-  </si>
-  <si>
     <t>AMI-0066</t>
   </si>
   <si>
@@ -1117,6 +1114,9 @@
   </si>
   <si>
     <t>1970.Movimento.Studentesco.PensierodiMao.jpg</t>
+  </si>
+  <si>
+    <t>1968.Mantifestazione.PCDI.jpg</t>
   </si>
 </sst>
 </file>
@@ -3883,18 +3883,18 @@
         <v>357</v>
       </c>
       <c r="N66" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>358</v>
+      </c>
+      <c r="B67" t="s">
         <v>359</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>360</v>
-      </c>
-      <c r="C67" t="s">
-        <v>361</v>
       </c>
       <c r="F67">
         <v>1970</v>
@@ -3912,15 +3912,15 @@
         <v>325</v>
       </c>
       <c r="M67" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="N67" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="N68" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 17/08/2026 23:10
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED03F46-2A69-4713-A92F-0E3B7C6A3BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1862FB96-2499-4CC9-AF2A-211F8C116933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="366">
   <si>
     <t>ID</t>
   </si>
@@ -1077,12 +1077,6 @@
     <t>Volantino dell'OC(m-l) - Fronte Unito contro l'aumento del costo della benzina</t>
   </si>
   <si>
-    <t>https://archive.org/details/1974-volantino-contro-rumor</t>
-  </si>
-  <si>
-    <t>https://archive.org/details/1973-volantino-anti-rumor-ocm-l</t>
-  </si>
-  <si>
     <t>AMI-0065</t>
   </si>
   <si>
@@ -1117,6 +1111,15 @@
   </si>
   <si>
     <t>Volantino del PCd'I(m-l) contro l'eccidio di Avola</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1968-volantino-pcdi-avola</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/ocml-volantino-anti-rumor</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/pcmli-volantino-contro-rumor</t>
   </si>
 </sst>
 </file>
@@ -3813,7 +3816,7 @@
         <v>347</v>
       </c>
       <c r="M64" s="4" t="s">
-        <v>351</v>
+        <v>365</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
@@ -3845,15 +3848,15 @@
         <v>347</v>
       </c>
       <c r="M65" s="4" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B66" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C66" t="s">
         <v>64</v>
@@ -3874,21 +3877,21 @@
         <v>325</v>
       </c>
       <c r="M66" s="4" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="N66" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>354</v>
+      </c>
+      <c r="B67" t="s">
+        <v>355</v>
+      </c>
+      <c r="C67" t="s">
         <v>356</v>
-      </c>
-      <c r="B67" t="s">
-        <v>357</v>
-      </c>
-      <c r="C67" t="s">
-        <v>358</v>
       </c>
       <c r="F67">
         <v>1970</v>
@@ -3906,18 +3909,18 @@
         <v>325</v>
       </c>
       <c r="M67" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="N67" t="s">
         <v>359</v>
-      </c>
-      <c r="N67" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B68" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C68" t="s">
         <v>64</v>
@@ -3937,8 +3940,11 @@
       <c r="L68" t="s">
         <v>325</v>
       </c>
+      <c r="M68" s="4" t="s">
+        <v>363</v>
+      </c>
       <c r="N68" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -4010,10 +4016,11 @@
     <hyperlink ref="M65" r:id="rId64" xr:uid="{705AEFBC-C508-48F1-BEC0-89DB7C3BD430}"/>
     <hyperlink ref="M66" r:id="rId65" xr:uid="{8365E924-D46C-4D93-9FDD-E2A533CDCEF8}"/>
     <hyperlink ref="M67" r:id="rId66" xr:uid="{9E0E6191-2474-42FA-BA40-68DA6CAC11D8}"/>
+    <hyperlink ref="M68" r:id="rId67" xr:uid="{7538D10C-1B89-41F2-8EF8-6C51156B9F3D}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId67"/>
+    <tablePart r:id="rId68"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 18/08/2026 09:27
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1862FB96-2499-4CC9-AF2A-211F8C116933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7080407B-557F-4BF9-BC66-216A34AC028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="378">
   <si>
     <t>ID</t>
   </si>
@@ -1120,6 +1120,42 @@
   </si>
   <si>
     <t>https://archive.org/details/pcmli-volantino-contro-rumor</t>
+  </si>
+  <si>
+    <t>12/1968</t>
+  </si>
+  <si>
+    <t>01/1974</t>
+  </si>
+  <si>
+    <t>03/1978</t>
+  </si>
+  <si>
+    <t>08/1969</t>
+  </si>
+  <si>
+    <t>09/1968</t>
+  </si>
+  <si>
+    <t>06/1968</t>
+  </si>
+  <si>
+    <t>05/1968</t>
+  </si>
+  <si>
+    <t>03/1968</t>
+  </si>
+  <si>
+    <t>02/1968</t>
+  </si>
+  <si>
+    <t>01/1968</t>
+  </si>
+  <si>
+    <t>11/1967</t>
+  </si>
+  <si>
+    <t>10/1967</t>
   </si>
 </sst>
 </file>
@@ -1183,10 +1219,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1639,7 +1675,7 @@
       <c r="L2" t="s">
         <v>325</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1674,7 +1710,7 @@
       <c r="L3" t="s">
         <v>325</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1709,7 +1745,7 @@
       <c r="L4" t="s">
         <v>325</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1744,7 +1780,7 @@
       <c r="L5" t="s">
         <v>324</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1779,7 +1815,7 @@
       <c r="L6" t="s">
         <v>324</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="3" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1814,7 +1850,7 @@
       <c r="L7" t="s">
         <v>325</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="3" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1849,7 +1885,7 @@
       <c r="L8" t="s">
         <v>325</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1884,7 +1920,7 @@
       <c r="L9" t="s">
         <v>325</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1919,7 +1955,7 @@
       <c r="L10" t="s">
         <v>325</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="3" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1954,7 +1990,7 @@
       <c r="L11" t="s">
         <v>325</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="3" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1992,7 +2028,7 @@
       <c r="L12" t="s">
         <v>325</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="3" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2027,7 +2063,7 @@
       <c r="L13" t="s">
         <v>325</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="3" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2068,7 +2104,7 @@
       <c r="L14" t="s">
         <v>325</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="3" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2103,7 +2139,7 @@
       <c r="L15" t="s">
         <v>325</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="3" t="s">
         <v>77</v>
       </c>
       <c r="N15" t="s">
@@ -2141,7 +2177,7 @@
       <c r="L16" t="s">
         <v>325</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="3" t="s">
         <v>83</v>
       </c>
       <c r="N16" t="s">
@@ -2179,7 +2215,7 @@
       <c r="L17" t="s">
         <v>325</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="3" t="s">
         <v>88</v>
       </c>
       <c r="N17" t="s">
@@ -2214,7 +2250,7 @@
       <c r="L18" t="s">
         <v>325</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="M18" s="3" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2246,7 +2282,7 @@
       <c r="L19" t="s">
         <v>325</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="3" t="s">
         <v>100</v>
       </c>
       <c r="N19" t="s">
@@ -2278,7 +2314,7 @@
       <c r="L20" t="s">
         <v>325</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="3" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2310,7 +2346,7 @@
       <c r="L21" t="s">
         <v>325</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="3" t="s">
         <v>333</v>
       </c>
     </row>
@@ -2327,8 +2363,8 @@
       <c r="E22" t="s">
         <v>116</v>
       </c>
-      <c r="F22" s="3">
-        <v>24746</v>
+      <c r="F22" s="6" t="s">
+        <v>377</v>
       </c>
       <c r="G22" t="s">
         <v>117</v>
@@ -2342,7 +2378,7 @@
       <c r="L22" t="s">
         <v>323</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="3" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2359,8 +2395,8 @@
       <c r="E23" t="s">
         <v>116</v>
       </c>
-      <c r="F23" s="3">
-        <v>24777</v>
+      <c r="F23" s="6" t="s">
+        <v>376</v>
       </c>
       <c r="G23" t="s">
         <v>117</v>
@@ -2374,7 +2410,7 @@
       <c r="L23" t="s">
         <v>323</v>
       </c>
-      <c r="M23" s="4" t="s">
+      <c r="M23" s="3" t="s">
         <v>331</v>
       </c>
     </row>
@@ -2391,8 +2427,8 @@
       <c r="E24" t="s">
         <v>116</v>
       </c>
-      <c r="F24" s="3">
-        <v>24838</v>
+      <c r="F24" s="6" t="s">
+        <v>375</v>
       </c>
       <c r="G24" t="s">
         <v>117</v>
@@ -2406,7 +2442,7 @@
       <c r="L24" t="s">
         <v>323</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="3" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2423,8 +2459,8 @@
       <c r="E25" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="3">
-        <v>24869</v>
+      <c r="F25" s="6" t="s">
+        <v>374</v>
       </c>
       <c r="G25" t="s">
         <v>117</v>
@@ -2438,7 +2474,7 @@
       <c r="L25" t="s">
         <v>323</v>
       </c>
-      <c r="M25" s="4" t="s">
+      <c r="M25" s="3" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2455,8 +2491,8 @@
       <c r="E26" t="s">
         <v>116</v>
       </c>
-      <c r="F26" s="3">
-        <v>24898</v>
+      <c r="F26" s="6" t="s">
+        <v>373</v>
       </c>
       <c r="G26" t="s">
         <v>117</v>
@@ -2470,7 +2506,7 @@
       <c r="L26" t="s">
         <v>323</v>
       </c>
-      <c r="M26" s="4" t="s">
+      <c r="M26" s="3" t="s">
         <v>131</v>
       </c>
     </row>
@@ -2487,8 +2523,8 @@
       <c r="E27" t="s">
         <v>116</v>
       </c>
-      <c r="F27" s="3">
-        <v>24959</v>
+      <c r="F27" s="6" t="s">
+        <v>372</v>
       </c>
       <c r="G27" t="s">
         <v>117</v>
@@ -2502,7 +2538,7 @@
       <c r="L27" t="s">
         <v>323</v>
       </c>
-      <c r="M27" s="4" t="s">
+      <c r="M27" s="3" t="s">
         <v>332</v>
       </c>
     </row>
@@ -2519,8 +2555,8 @@
       <c r="E28" t="s">
         <v>116</v>
       </c>
-      <c r="F28" s="3">
-        <v>24990</v>
+      <c r="F28" s="6" t="s">
+        <v>371</v>
       </c>
       <c r="G28" t="s">
         <v>117</v>
@@ -2534,7 +2570,7 @@
       <c r="L28" t="s">
         <v>323</v>
       </c>
-      <c r="M28" s="4" t="s">
+      <c r="M28" s="3" t="s">
         <v>136</v>
       </c>
     </row>
@@ -2551,8 +2587,8 @@
       <c r="E29" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="3">
-        <v>25082</v>
+      <c r="F29" s="6" t="s">
+        <v>370</v>
       </c>
       <c r="G29" t="s">
         <v>117</v>
@@ -2569,7 +2605,7 @@
       <c r="L29" t="s">
         <v>323</v>
       </c>
-      <c r="M29" s="4" t="s">
+      <c r="M29" s="3" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2586,8 +2622,8 @@
       <c r="E30" t="s">
         <v>116</v>
       </c>
-      <c r="F30" s="3">
-        <v>25173</v>
+      <c r="F30" s="6" t="s">
+        <v>366</v>
       </c>
       <c r="G30" t="s">
         <v>117</v>
@@ -2604,7 +2640,7 @@
       <c r="L30" t="s">
         <v>323</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="M30" s="3" t="s">
         <v>143</v>
       </c>
     </row>
@@ -2639,7 +2675,7 @@
       <c r="L31" t="s">
         <v>325</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="M31" s="3" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2674,7 +2710,7 @@
       <c r="L32" t="s">
         <v>324</v>
       </c>
-      <c r="M32" s="4" t="s">
+      <c r="M32" s="3" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2703,7 +2739,7 @@
       <c r="L33" t="s">
         <v>325</v>
       </c>
-      <c r="M33" s="4" t="s">
+      <c r="M33" s="3" t="s">
         <v>156</v>
       </c>
       <c r="N33" t="s">
@@ -2741,7 +2777,7 @@
       <c r="L34" t="s">
         <v>325</v>
       </c>
-      <c r="M34" s="4" t="s">
+      <c r="M34" s="3" t="s">
         <v>162</v>
       </c>
       <c r="O34" t="s">
@@ -2785,7 +2821,7 @@
       <c r="L35" t="s">
         <v>325</v>
       </c>
-      <c r="M35" s="4" t="s">
+      <c r="M35" s="3" t="s">
         <v>168</v>
       </c>
       <c r="O35" t="s">
@@ -2805,8 +2841,8 @@
       <c r="C36" t="s">
         <v>92</v>
       </c>
-      <c r="F36" s="3">
-        <v>25416</v>
+      <c r="F36" s="6" t="s">
+        <v>369</v>
       </c>
       <c r="G36" t="s">
         <v>117</v>
@@ -2820,7 +2856,7 @@
       <c r="L36" t="s">
         <v>325</v>
       </c>
-      <c r="M36" s="4" t="s">
+      <c r="M36" s="3" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2858,7 +2894,7 @@
       <c r="L37" t="s">
         <v>325</v>
       </c>
-      <c r="M37" s="4" t="s">
+      <c r="M37" s="3" t="s">
         <v>179</v>
       </c>
     </row>
@@ -2893,7 +2929,7 @@
       <c r="L38" t="s">
         <v>325</v>
       </c>
-      <c r="M38" s="4" t="s">
+      <c r="M38" s="3" t="s">
         <v>182</v>
       </c>
     </row>
@@ -2931,7 +2967,7 @@
       <c r="L39" t="s">
         <v>325</v>
       </c>
-      <c r="M39" s="4" t="s">
+      <c r="M39" s="3" t="s">
         <v>187</v>
       </c>
     </row>
@@ -2966,7 +3002,7 @@
       <c r="L40" t="s">
         <v>325</v>
       </c>
-      <c r="M40" s="4" t="s">
+      <c r="M40" s="3" t="s">
         <v>191</v>
       </c>
     </row>
@@ -3001,7 +3037,7 @@
       <c r="L41" t="s">
         <v>325</v>
       </c>
-      <c r="M41" s="4" t="s">
+      <c r="M41" s="3" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3033,7 +3069,7 @@
       <c r="L42" t="s">
         <v>325</v>
       </c>
-      <c r="M42" s="4" t="s">
+      <c r="M42" s="3" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3071,7 +3107,7 @@
       <c r="L43" t="s">
         <v>325</v>
       </c>
-      <c r="M43" s="4" t="s">
+      <c r="M43" s="3" t="s">
         <v>206</v>
       </c>
     </row>
@@ -3106,7 +3142,7 @@
       <c r="L44" t="s">
         <v>325</v>
       </c>
-      <c r="M44" s="4" t="s">
+      <c r="M44" s="3" t="s">
         <v>209</v>
       </c>
     </row>
@@ -3141,7 +3177,7 @@
       <c r="L45" t="s">
         <v>325</v>
       </c>
-      <c r="M45" s="4" t="s">
+      <c r="M45" s="3" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3176,7 +3212,7 @@
       <c r="L46" t="s">
         <v>325</v>
       </c>
-      <c r="M46" s="4" t="s">
+      <c r="M46" s="3" t="s">
         <v>215</v>
       </c>
     </row>
@@ -3211,7 +3247,7 @@
       <c r="L47" t="s">
         <v>325</v>
       </c>
-      <c r="M47" s="4" t="s">
+      <c r="M47" s="3" t="s">
         <v>218</v>
       </c>
     </row>
@@ -3246,7 +3282,7 @@
       <c r="L48" t="s">
         <v>325</v>
       </c>
-      <c r="M48" s="4" t="s">
+      <c r="M48" s="3" t="s">
         <v>221</v>
       </c>
     </row>
@@ -3281,7 +3317,7 @@
       <c r="L49" t="s">
         <v>325</v>
       </c>
-      <c r="M49" s="4" t="s">
+      <c r="M49" s="3" t="s">
         <v>224</v>
       </c>
     </row>
@@ -3316,7 +3352,7 @@
       <c r="L50" t="s">
         <v>325</v>
       </c>
-      <c r="M50" s="4" t="s">
+      <c r="M50" s="3" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3351,7 +3387,7 @@
       <c r="L51" t="s">
         <v>325</v>
       </c>
-      <c r="M51" s="4" t="s">
+      <c r="M51" s="3" t="s">
         <v>230</v>
       </c>
     </row>
@@ -3386,7 +3422,7 @@
       <c r="L52" t="s">
         <v>325</v>
       </c>
-      <c r="M52" s="4" t="s">
+      <c r="M52" s="3" t="s">
         <v>233</v>
       </c>
     </row>
@@ -3421,7 +3457,7 @@
       <c r="L53" t="s">
         <v>325</v>
       </c>
-      <c r="M53" s="4" t="s">
+      <c r="M53" s="3" t="s">
         <v>238</v>
       </c>
     </row>
@@ -3453,7 +3489,7 @@
       <c r="L54" t="s">
         <v>325</v>
       </c>
-      <c r="M54" s="4" t="s">
+      <c r="M54" s="3" t="s">
         <v>243</v>
       </c>
     </row>
@@ -3473,8 +3509,8 @@
       <c r="E55" t="s">
         <v>247</v>
       </c>
-      <c r="F55" s="3">
-        <v>28550</v>
+      <c r="F55" s="6" t="s">
+        <v>368</v>
       </c>
       <c r="G55" t="s">
         <v>248</v>
@@ -3491,7 +3527,7 @@
       <c r="L55" t="s">
         <v>325</v>
       </c>
-      <c r="M55" s="4" t="s">
+      <c r="M55" s="3" t="s">
         <v>250</v>
       </c>
       <c r="N55" t="s">
@@ -3526,7 +3562,7 @@
       <c r="L56" t="s">
         <v>325</v>
       </c>
-      <c r="M56" s="4" t="s">
+      <c r="M56" s="3" t="s">
         <v>254</v>
       </c>
       <c r="N56" t="s">
@@ -3564,7 +3600,7 @@
       <c r="L57" t="s">
         <v>325</v>
       </c>
-      <c r="M57" s="4" t="s">
+      <c r="M57" s="3" t="s">
         <v>258</v>
       </c>
     </row>
@@ -3605,7 +3641,7 @@
       <c r="L58" t="s">
         <v>325</v>
       </c>
-      <c r="M58" s="4" t="s">
+      <c r="M58" s="3" t="s">
         <v>261</v>
       </c>
       <c r="N58" t="s">
@@ -3643,7 +3679,7 @@
       <c r="L59" t="s">
         <v>325</v>
       </c>
-      <c r="M59" s="4" t="s">
+      <c r="M59" s="3" t="s">
         <v>321</v>
       </c>
     </row>
@@ -3678,7 +3714,7 @@
       <c r="L60" t="s">
         <v>325</v>
       </c>
-      <c r="M60" s="4" t="s">
+      <c r="M60" s="3" t="s">
         <v>320</v>
       </c>
     </row>
@@ -3716,7 +3752,7 @@
       <c r="L61" t="s">
         <v>325</v>
       </c>
-      <c r="M61" s="4" t="s">
+      <c r="M61" s="3" t="s">
         <v>330</v>
       </c>
     </row>
@@ -3751,7 +3787,7 @@
       <c r="L62" t="s">
         <v>325</v>
       </c>
-      <c r="M62" s="4" t="s">
+      <c r="M62" s="3" t="s">
         <v>337</v>
       </c>
     </row>
@@ -3762,7 +3798,7 @@
       <c r="B63" t="s">
         <v>339</v>
       </c>
-      <c r="F63" s="5">
+      <c r="F63" s="4">
         <v>24917</v>
       </c>
       <c r="G63" t="s">
@@ -3780,7 +3816,7 @@
       <c r="L63" t="s">
         <v>325</v>
       </c>
-      <c r="M63" s="4" t="s">
+      <c r="M63" s="3" t="s">
         <v>342</v>
       </c>
       <c r="N63" t="s">
@@ -3800,8 +3836,8 @@
       <c r="D64" t="s">
         <v>242</v>
       </c>
-      <c r="F64" s="6">
-        <v>27030</v>
+      <c r="F64" s="5" t="s">
+        <v>367</v>
       </c>
       <c r="G64" t="s">
         <v>94</v>
@@ -3815,7 +3851,7 @@
       <c r="L64" t="s">
         <v>347</v>
       </c>
-      <c r="M64" s="4" t="s">
+      <c r="M64" s="3" t="s">
         <v>365</v>
       </c>
     </row>
@@ -3832,7 +3868,7 @@
       <c r="D65" t="s">
         <v>348</v>
       </c>
-      <c r="F65" s="5">
+      <c r="F65" s="4">
         <v>26956</v>
       </c>
       <c r="G65" t="s">
@@ -3847,7 +3883,7 @@
       <c r="L65" t="s">
         <v>347</v>
       </c>
-      <c r="M65" s="4" t="s">
+      <c r="M65" s="3" t="s">
         <v>364</v>
       </c>
     </row>
@@ -3876,7 +3912,7 @@
       <c r="L66" t="s">
         <v>325</v>
       </c>
-      <c r="M66" s="4" t="s">
+      <c r="M66" s="3" t="s">
         <v>353</v>
       </c>
       <c r="N66" t="s">
@@ -3908,7 +3944,7 @@
       <c r="L67" t="s">
         <v>325</v>
       </c>
-      <c r="M67" s="4" t="s">
+      <c r="M67" s="3" t="s">
         <v>357</v>
       </c>
       <c r="N67" t="s">
@@ -3925,8 +3961,8 @@
       <c r="C68" t="s">
         <v>64</v>
       </c>
-      <c r="F68" s="6">
-        <v>25173</v>
+      <c r="F68" s="5" t="s">
+        <v>366</v>
       </c>
       <c r="G68" t="s">
         <v>94</v>
@@ -3940,7 +3976,7 @@
       <c r="L68" t="s">
         <v>325</v>
       </c>
-      <c r="M68" s="4" t="s">
+      <c r="M68" s="3" t="s">
         <v>363</v>
       </c>
       <c r="N68" t="s">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 18/08/2026 12:22
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7080407B-557F-4BF9-BC66-216A34AC028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4409CBC-B7AB-4DB0-93DB-8F3FEC310ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="449">
   <si>
     <t>ID</t>
   </si>
@@ -366,9 +366,6 @@
     <t>AMI-0021</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 1</t>
-  </si>
-  <si>
     <t>Lavoro Politico</t>
   </si>
   <si>
@@ -390,66 +387,42 @@
     <t>AMI-0022</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 2</t>
-  </si>
-  <si>
     <t>AMI-0023</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 3</t>
-  </si>
-  <si>
     <t>https://archive.org/details/lavoro-politico-03/mode/2up</t>
   </si>
   <si>
     <t>AMI-0024</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 4</t>
-  </si>
-  <si>
     <t>https://archive.org/details/lavoro-politico-04/mode/2up</t>
   </si>
   <si>
     <t>AMI-0025</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 5/6</t>
-  </si>
-  <si>
     <t>https://archive.org/details/lavoro-politico-05-06/mode/2up</t>
   </si>
   <si>
     <t>AMI-0026</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 7</t>
-  </si>
-  <si>
     <t>AMI-0027</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 8/9</t>
-  </si>
-  <si>
     <t>https://archive.org/details/lavoro-politico-08-09/mode/2up</t>
   </si>
   <si>
     <t>AMI-0028</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 10</t>
-  </si>
-  <si>
     <t>https://archive.org/details/lavoro-politico-10/mode/2up</t>
   </si>
   <si>
     <t>AMI-0029</t>
   </si>
   <si>
-    <t>Lavoro Politico no. 11/12</t>
-  </si>
-  <si>
     <t>Partito Comunista d'Italia (marxista-leninista); Partito Comunista d'Italia (marxista-leninista) - linea rossa</t>
   </si>
   <si>
@@ -1113,15 +1086,6 @@
     <t>Volantino del PCd'I(m-l) contro l'eccidio di Avola</t>
   </si>
   <si>
-    <t>https://archive.org/details/1968-volantino-pcdi-avola</t>
-  </si>
-  <si>
-    <t>https://archive.org/details/ocml-volantino-anti-rumor</t>
-  </si>
-  <si>
-    <t>https://archive.org/details/pcmli-volantino-contro-rumor</t>
-  </si>
-  <si>
     <t>12/1968</t>
   </si>
   <si>
@@ -1156,6 +1120,255 @@
   </si>
   <si>
     <t>10/1967</t>
+  </si>
+  <si>
+    <t>AMI-0068</t>
+  </si>
+  <si>
+    <t>AMI-0069</t>
+  </si>
+  <si>
+    <t>AMI-0070</t>
+  </si>
+  <si>
+    <t>AMI-0071</t>
+  </si>
+  <si>
+    <t>AMI-0072</t>
+  </si>
+  <si>
+    <t>AMI-0073</t>
+  </si>
+  <si>
+    <t>AMI-0074</t>
+  </si>
+  <si>
+    <t>AMI-0075</t>
+  </si>
+  <si>
+    <t>AMI-0076</t>
+  </si>
+  <si>
+    <t>AMI-0077</t>
+  </si>
+  <si>
+    <t>AMI-0078</t>
+  </si>
+  <si>
+    <t>AMI-0079</t>
+  </si>
+  <si>
+    <t>AMI-0080</t>
+  </si>
+  <si>
+    <t>AMI-0081</t>
+  </si>
+  <si>
+    <t>AMI-0082</t>
+  </si>
+  <si>
+    <t>AMI-0083</t>
+  </si>
+  <si>
+    <t>AMI-0084</t>
+  </si>
+  <si>
+    <t>AMI-0085</t>
+  </si>
+  <si>
+    <t>AMI-0086</t>
+  </si>
+  <si>
+    <t>AMI-0087</t>
+  </si>
+  <si>
+    <t>AMI-0088</t>
+  </si>
+  <si>
+    <t>AMI-0089</t>
+  </si>
+  <si>
+    <t>AMI-0090</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno III, no. 1</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno III, no. 2/3</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno III, no. 4/5</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno III, no. 6</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno IV, no. 1</t>
+  </si>
+  <si>
+    <t>Circoli Lenin dell'Emilia Romagna</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 1</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 2</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 3</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 4</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 5/6</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 7</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 8/9</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 10</t>
+  </si>
+  <si>
+    <t>Lavoro Politico, no. 11/12</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-01/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-02-suppl/mode/2up</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, supplemento al no. 2</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 1</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 3</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 4</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 5/6</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 7/8</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 9/10</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 11</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 12</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 13</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 14</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 15/16</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 17/18</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 19/20</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 21</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 22</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 23</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 24/25</t>
+  </si>
+  <si>
+    <t>05/1970</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1972-04-05/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1973-01-02/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-03/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-04/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-05-06/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-07-08/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-09-10/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-11/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-12/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-13/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-14/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-15-16/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-17-18/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-19-20/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-21/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-22/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-23/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1968-volantino-pcdi-avola/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/ocml-volantino-anti-rumor/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/pcmli-volantino-contro-rumor/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1971-24-25/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1972-01/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1972-02-03/mode/2up</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1972-06/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -1215,7 +1428,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1223,6 +1436,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1579,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P91"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -1629,7 +1843,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="M1" t="s">
         <v>11</v>
@@ -1673,7 +1887,7 @@
         <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>23</v>
@@ -1708,7 +1922,7 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>28</v>
@@ -1743,7 +1957,7 @@
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>31</v>
@@ -1778,7 +1992,7 @@
         <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>35</v>
@@ -1813,7 +2027,7 @@
         <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>38</v>
@@ -1848,7 +2062,7 @@
         <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>41</v>
@@ -1883,7 +2097,7 @@
         <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>44</v>
@@ -1918,7 +2132,7 @@
         <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>47</v>
@@ -1953,7 +2167,7 @@
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>50</v>
@@ -1988,7 +2202,7 @@
         <v>34</v>
       </c>
       <c r="L11" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>53</v>
@@ -2026,7 +2240,7 @@
         <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>57</v>
@@ -2061,7 +2275,7 @@
         <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>61</v>
@@ -2102,7 +2316,7 @@
         <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>71</v>
@@ -2137,7 +2351,7 @@
         <v>76</v>
       </c>
       <c r="L15" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>77</v>
@@ -2175,7 +2389,7 @@
         <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>83</v>
@@ -2213,7 +2427,7 @@
         <v>87</v>
       </c>
       <c r="L17" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>88</v>
@@ -2248,7 +2462,7 @@
         <v>68</v>
       </c>
       <c r="L18" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>96</v>
@@ -2280,7 +2494,7 @@
         <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>100</v>
@@ -2312,7 +2526,7 @@
         <v>106</v>
       </c>
       <c r="L20" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>107</v>
@@ -2344,10 +2558,10 @@
         <v>106</v>
       </c>
       <c r="L21" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -2355,307 +2569,307 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
+        <v>395</v>
+      </c>
+      <c r="C22" t="s">
         <v>114</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>115</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="G22" t="s">
         <v>116</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>377</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>117</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>118</v>
       </c>
-      <c r="I22" t="s">
+      <c r="L22" t="s">
+        <v>314</v>
+      </c>
+      <c r="M22" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="L22" t="s">
-        <v>323</v>
-      </c>
-      <c r="M22" s="3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>396</v>
       </c>
       <c r="C23" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" t="s">
         <v>115</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="G23" t="s">
         <v>116</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>117</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>118</v>
       </c>
-      <c r="I23" t="s">
-        <v>119</v>
-      </c>
       <c r="L23" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>124</v>
+        <v>397</v>
       </c>
       <c r="C24" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" t="s">
         <v>115</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="G24" t="s">
         <v>116</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>375</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>117</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>118</v>
       </c>
-      <c r="I24" t="s">
-        <v>119</v>
-      </c>
       <c r="L24" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>127</v>
+        <v>398</v>
       </c>
       <c r="C25" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" t="s">
         <v>115</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="G25" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>374</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>117</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>118</v>
       </c>
-      <c r="I25" t="s">
-        <v>119</v>
-      </c>
       <c r="L25" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>130</v>
+        <v>399</v>
       </c>
       <c r="C26" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" t="s">
         <v>115</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="G26" t="s">
         <v>116</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>117</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>118</v>
       </c>
-      <c r="I26" t="s">
-        <v>119</v>
-      </c>
       <c r="L26" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B27" t="s">
-        <v>133</v>
+        <v>400</v>
       </c>
       <c r="C27" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" t="s">
         <v>115</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="G27" t="s">
         <v>116</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>372</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>117</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>118</v>
       </c>
-      <c r="I27" t="s">
-        <v>119</v>
-      </c>
       <c r="L27" t="s">
+        <v>314</v>
+      </c>
+      <c r="M27" s="3" t="s">
         <v>323</v>
-      </c>
-      <c r="M27" s="3" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>135</v>
+        <v>401</v>
       </c>
       <c r="C28" t="s">
+        <v>114</v>
+      </c>
+      <c r="E28" t="s">
         <v>115</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="G28" t="s">
         <v>116</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>117</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>118</v>
       </c>
-      <c r="I28" t="s">
-        <v>119</v>
-      </c>
       <c r="L28" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>138</v>
+        <v>402</v>
       </c>
       <c r="C29" t="s">
+        <v>114</v>
+      </c>
+      <c r="E29" t="s">
         <v>115</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="G29" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>117</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>118</v>
-      </c>
-      <c r="I29" t="s">
-        <v>119</v>
       </c>
       <c r="K29" t="s">
         <v>64</v>
       </c>
       <c r="L29" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B30" t="s">
-        <v>141</v>
+        <v>403</v>
       </c>
       <c r="C30" t="s">
+        <v>114</v>
+      </c>
+      <c r="E30" t="s">
         <v>115</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="G30" t="s">
         <v>116</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>366</v>
-      </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>117</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>118</v>
       </c>
-      <c r="I30" t="s">
-        <v>119</v>
-      </c>
       <c r="K30" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="L30" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B31" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C31" t="s">
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="E31" t="s">
         <v>19</v>
@@ -2673,18 +2887,18 @@
         <v>34</v>
       </c>
       <c r="L31" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="C32" t="s">
         <v>17</v>
@@ -2708,50 +2922,50 @@
         <v>34</v>
       </c>
       <c r="L32" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="B33" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C33" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F33" s="1">
         <v>1970</v>
       </c>
       <c r="G33" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I33" t="s">
         <v>68</v>
       </c>
       <c r="J33" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="L33" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="N33" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B34" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="C34" t="s">
         <v>64</v>
@@ -2760,7 +2974,7 @@
         <v>25063</v>
       </c>
       <c r="G34" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="H34" t="s">
         <v>21</v>
@@ -2769,30 +2983,30 @@
         <v>68</v>
       </c>
       <c r="J34" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="K34" t="s">
         <v>17</v>
       </c>
       <c r="L34" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="O34" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="P34" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="B35" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
@@ -2804,7 +3018,7 @@
         <v>25081</v>
       </c>
       <c r="G35" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="H35" t="s">
         <v>21</v>
@@ -2813,68 +3027,68 @@
         <v>68</v>
       </c>
       <c r="J35" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="K35" t="s">
         <v>64</v>
       </c>
       <c r="L35" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="O35" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="P35" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="B36" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
         <v>92</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="G36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H36" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I36" t="s">
         <v>68</v>
       </c>
       <c r="L36" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B37" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C37" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D37" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E37" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F37" s="1">
         <v>1975</v>
@@ -2883,27 +3097,27 @@
         <v>20</v>
       </c>
       <c r="H37" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I37" t="s">
         <v>106</v>
       </c>
       <c r="K37" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="L37" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B38" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
         <v>17</v>
@@ -2927,24 +3141,24 @@
         <v>34</v>
       </c>
       <c r="L38" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="B39" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="C39" t="s">
         <v>17</v>
       </c>
       <c r="D39" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="E39" t="s">
         <v>19</v>
@@ -2962,21 +3176,21 @@
         <v>34</v>
       </c>
       <c r="J39" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="L39" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="B40" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="C40" t="s">
         <v>17</v>
@@ -2997,27 +3211,27 @@
         <v>21</v>
       </c>
       <c r="I40" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="L40" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B41" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="E41" t="s">
         <v>19</v>
@@ -3035,24 +3249,24 @@
         <v>34</v>
       </c>
       <c r="L41" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B42" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="D42" t="s">
         <v>18</v>
       </c>
       <c r="E42" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="F42" s="1">
         <v>1968</v>
@@ -3061,30 +3275,30 @@
         <v>20</v>
       </c>
       <c r="H42" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I42" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="L42" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B43" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="D43" t="s">
         <v>18</v>
       </c>
       <c r="E43" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="F43" s="1">
         <v>1967</v>
@@ -3093,30 +3307,30 @@
         <v>20</v>
       </c>
       <c r="H43" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I43" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="J43" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="K43" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="L43" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B44" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C44" t="s">
         <v>17</v>
@@ -3140,18 +3354,18 @@
         <v>27</v>
       </c>
       <c r="L44" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B45" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="C45" t="s">
         <v>17</v>
@@ -3175,18 +3389,18 @@
         <v>27</v>
       </c>
       <c r="L45" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B46" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C46" t="s">
         <v>17</v>
@@ -3210,18 +3424,18 @@
         <v>27</v>
       </c>
       <c r="L46" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M46" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="B47" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C47" t="s">
         <v>17</v>
@@ -3245,18 +3459,18 @@
         <v>34</v>
       </c>
       <c r="L47" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B48" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C48" t="s">
         <v>17</v>
@@ -3280,18 +3494,18 @@
         <v>34</v>
       </c>
       <c r="L48" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M48" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="B49" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="C49" t="s">
         <v>17</v>
@@ -3315,18 +3529,18 @@
         <v>27</v>
       </c>
       <c r="L49" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B50" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C50" t="s">
         <v>17</v>
@@ -3350,18 +3564,18 @@
         <v>27</v>
       </c>
       <c r="L50" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M50" s="3" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B51" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="C51" t="s">
         <v>17</v>
@@ -3385,18 +3599,18 @@
         <v>27</v>
       </c>
       <c r="L51" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B52" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="C52" t="s">
         <v>17</v>
@@ -3420,27 +3634,27 @@
         <v>34</v>
       </c>
       <c r="L52" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="B53" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="C53" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="D53" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E53" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="F53" s="1">
         <v>1969</v>
@@ -3449,24 +3663,24 @@
         <v>20</v>
       </c>
       <c r="H53" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I53" t="s">
         <v>68</v>
       </c>
       <c r="L53" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="B54" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="C54" t="s">
         <v>92</v>
@@ -3478,68 +3692,68 @@
         <v>94</v>
       </c>
       <c r="H54" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="I54" t="s">
         <v>68</v>
       </c>
       <c r="K54" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="L54" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M54" s="3" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B55" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="C55" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="D55" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E55" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="G55" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="H55" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I55" t="s">
         <v>68</v>
       </c>
       <c r="J55" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="L55" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="N55" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B56" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="C56" t="s">
         <v>64</v>
@@ -3554,27 +3768,27 @@
         <v>1967</v>
       </c>
       <c r="G56" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="I56" t="s">
         <v>68</v>
       </c>
       <c r="L56" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M56" s="3" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="N56" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B57" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="C57" t="s">
         <v>99</v>
@@ -3592,33 +3806,33 @@
         <v>20</v>
       </c>
       <c r="H57" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I57" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="L57" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B58" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="C58" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="D58" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E58" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="F58" s="2">
         <v>28253</v>
@@ -3627,39 +3841,39 @@
         <v>75</v>
       </c>
       <c r="H58" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I58" t="s">
         <v>68</v>
       </c>
       <c r="J58" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="K58" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="L58" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M58" s="3" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="N58" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="B59" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="C59" t="s">
         <v>99</v>
       </c>
       <c r="D59" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="E59" t="s">
         <v>99</v>
@@ -3671,30 +3885,30 @@
         <v>20</v>
       </c>
       <c r="H59" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I59" t="s">
         <v>106</v>
       </c>
       <c r="L59" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="B60" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="C60" t="s">
         <v>99</v>
       </c>
       <c r="D60" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="E60" t="s">
         <v>99</v>
@@ -3706,30 +3920,30 @@
         <v>20</v>
       </c>
       <c r="H60" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I60" t="s">
         <v>106</v>
       </c>
       <c r="L60" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="B61" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="C61" t="s">
         <v>99</v>
       </c>
       <c r="D61" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="E61" t="s">
         <v>99</v>
@@ -3741,27 +3955,27 @@
         <v>20</v>
       </c>
       <c r="H61" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I61" t="s">
         <v>106</v>
       </c>
       <c r="J61" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="L61" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="B62" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="C62" t="s">
         <v>17</v>
@@ -3785,18 +3999,18 @@
         <v>27</v>
       </c>
       <c r="L62" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="B63" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="F63" s="4">
         <v>24917</v>
@@ -3805,68 +4019,68 @@
         <v>75</v>
       </c>
       <c r="H63" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="I63" t="s">
         <v>106</v>
       </c>
       <c r="K63" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="L63" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="N63" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="B64" t="s">
-        <v>349</v>
+        <v>340</v>
       </c>
       <c r="C64" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="D64" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="G64" t="s">
         <v>94</v>
       </c>
       <c r="H64" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="I64" t="s">
         <v>68</v>
       </c>
       <c r="L64" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>365</v>
+        <v>444</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="B65" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="C65" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="D65" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="F65" s="4">
         <v>26956</v>
@@ -3875,24 +4089,24 @@
         <v>94</v>
       </c>
       <c r="H65" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="I65" t="s">
         <v>68</v>
       </c>
       <c r="L65" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>364</v>
+        <v>443</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="B66" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="C66" t="s">
         <v>64</v>
@@ -3904,30 +4118,30 @@
         <v>75</v>
       </c>
       <c r="H66" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I66" t="s">
         <v>68</v>
       </c>
       <c r="L66" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="N66" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="B67" t="s">
-        <v>355</v>
+        <v>346</v>
       </c>
       <c r="C67" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="F67">
         <v>1970</v>
@@ -3936,33 +4150,33 @@
         <v>75</v>
       </c>
       <c r="H67" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I67" t="s">
         <v>68</v>
       </c>
       <c r="L67" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="N67" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="B68" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="C68" t="s">
         <v>64</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="G68" t="s">
         <v>94</v>
@@ -3974,13 +4188,749 @@
         <v>68</v>
       </c>
       <c r="L68" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>363</v>
+        <v>442</v>
       </c>
       <c r="N68" t="s">
-        <v>358</v>
+        <v>349</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>366</v>
+      </c>
+      <c r="B69" t="s">
+        <v>407</v>
+      </c>
+      <c r="C69" t="s">
+        <v>394</v>
+      </c>
+      <c r="D69" t="s">
+        <v>394</v>
+      </c>
+      <c r="F69" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="G69" t="s">
+        <v>116</v>
+      </c>
+      <c r="H69" t="s">
+        <v>112</v>
+      </c>
+      <c r="I69" t="s">
+        <v>118</v>
+      </c>
+      <c r="L69" t="s">
+        <v>314</v>
+      </c>
+      <c r="M69" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>367</v>
+      </c>
+      <c r="B70" t="s">
+        <v>406</v>
+      </c>
+      <c r="C70" t="s">
+        <v>394</v>
+      </c>
+      <c r="D70" t="s">
+        <v>394</v>
+      </c>
+      <c r="F70" s="4">
+        <v>25718</v>
+      </c>
+      <c r="G70" t="s">
+        <v>116</v>
+      </c>
+      <c r="H70" t="s">
+        <v>112</v>
+      </c>
+      <c r="I70" t="s">
+        <v>118</v>
+      </c>
+      <c r="L70" t="s">
+        <v>314</v>
+      </c>
+      <c r="M70" s="3" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>368</v>
+      </c>
+      <c r="B71" t="s">
+        <v>408</v>
+      </c>
+      <c r="C71" t="s">
+        <v>394</v>
+      </c>
+      <c r="D71" t="s">
+        <v>394</v>
+      </c>
+      <c r="F71" s="4">
+        <v>25719</v>
+      </c>
+      <c r="G71" t="s">
+        <v>116</v>
+      </c>
+      <c r="H71" t="s">
+        <v>112</v>
+      </c>
+      <c r="I71" t="s">
+        <v>118</v>
+      </c>
+      <c r="L71" t="s">
+        <v>314</v>
+      </c>
+      <c r="M71" s="3" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>369</v>
+      </c>
+      <c r="B72" t="s">
+        <v>409</v>
+      </c>
+      <c r="C72" t="s">
+        <v>394</v>
+      </c>
+      <c r="D72" t="s">
+        <v>394</v>
+      </c>
+      <c r="F72" s="4">
+        <v>25740</v>
+      </c>
+      <c r="G72" t="s">
+        <v>116</v>
+      </c>
+      <c r="H72" t="s">
+        <v>112</v>
+      </c>
+      <c r="I72" t="s">
+        <v>118</v>
+      </c>
+      <c r="L72" t="s">
+        <v>314</v>
+      </c>
+      <c r="M72" s="3" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>370</v>
+      </c>
+      <c r="B73" t="s">
+        <v>410</v>
+      </c>
+      <c r="C73" t="s">
+        <v>394</v>
+      </c>
+      <c r="D73" t="s">
+        <v>394</v>
+      </c>
+      <c r="F73" s="4">
+        <v>25765</v>
+      </c>
+      <c r="G73" t="s">
+        <v>116</v>
+      </c>
+      <c r="H73" t="s">
+        <v>112</v>
+      </c>
+      <c r="I73" t="s">
+        <v>118</v>
+      </c>
+      <c r="L73" t="s">
+        <v>314</v>
+      </c>
+      <c r="M73" s="3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>371</v>
+      </c>
+      <c r="B74" t="s">
+        <v>411</v>
+      </c>
+      <c r="C74" t="s">
+        <v>394</v>
+      </c>
+      <c r="D74" t="s">
+        <v>394</v>
+      </c>
+      <c r="F74" s="4">
+        <v>25824</v>
+      </c>
+      <c r="G74" t="s">
+        <v>116</v>
+      </c>
+      <c r="H74" t="s">
+        <v>112</v>
+      </c>
+      <c r="I74" t="s">
+        <v>118</v>
+      </c>
+      <c r="L74" t="s">
+        <v>314</v>
+      </c>
+      <c r="M74" s="3" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>372</v>
+      </c>
+      <c r="B75" t="s">
+        <v>412</v>
+      </c>
+      <c r="C75" t="s">
+        <v>394</v>
+      </c>
+      <c r="D75" t="s">
+        <v>394</v>
+      </c>
+      <c r="F75" s="4">
+        <v>25866</v>
+      </c>
+      <c r="G75" t="s">
+        <v>116</v>
+      </c>
+      <c r="H75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I75" t="s">
+        <v>118</v>
+      </c>
+      <c r="L75" t="s">
+        <v>314</v>
+      </c>
+      <c r="M75" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>373</v>
+      </c>
+      <c r="B76" t="s">
+        <v>413</v>
+      </c>
+      <c r="C76" t="s">
+        <v>394</v>
+      </c>
+      <c r="D76" t="s">
+        <v>394</v>
+      </c>
+      <c r="F76" s="4">
+        <v>25887</v>
+      </c>
+      <c r="G76" t="s">
+        <v>116</v>
+      </c>
+      <c r="H76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I76" t="s">
+        <v>118</v>
+      </c>
+      <c r="L76" t="s">
+        <v>314</v>
+      </c>
+      <c r="M76" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>374</v>
+      </c>
+      <c r="B77" t="s">
+        <v>414</v>
+      </c>
+      <c r="C77" t="s">
+        <v>394</v>
+      </c>
+      <c r="D77" t="s">
+        <v>394</v>
+      </c>
+      <c r="F77" s="4">
+        <v>25915</v>
+      </c>
+      <c r="G77" t="s">
+        <v>116</v>
+      </c>
+      <c r="H77" t="s">
+        <v>112</v>
+      </c>
+      <c r="I77" t="s">
+        <v>118</v>
+      </c>
+      <c r="L77" t="s">
+        <v>314</v>
+      </c>
+      <c r="M77" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>375</v>
+      </c>
+      <c r="B78" t="s">
+        <v>415</v>
+      </c>
+      <c r="C78" t="s">
+        <v>394</v>
+      </c>
+      <c r="D78" t="s">
+        <v>394</v>
+      </c>
+      <c r="F78" s="4">
+        <v>25950</v>
+      </c>
+      <c r="G78" t="s">
+        <v>116</v>
+      </c>
+      <c r="H78" t="s">
+        <v>112</v>
+      </c>
+      <c r="I78" t="s">
+        <v>118</v>
+      </c>
+      <c r="L78" t="s">
+        <v>314</v>
+      </c>
+      <c r="M78" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>376</v>
+      </c>
+      <c r="B79" t="s">
+        <v>416</v>
+      </c>
+      <c r="C79" t="s">
+        <v>394</v>
+      </c>
+      <c r="D79" t="s">
+        <v>394</v>
+      </c>
+      <c r="F79" s="4">
+        <v>25971</v>
+      </c>
+      <c r="G79" t="s">
+        <v>116</v>
+      </c>
+      <c r="H79" t="s">
+        <v>112</v>
+      </c>
+      <c r="I79" t="s">
+        <v>118</v>
+      </c>
+      <c r="L79" t="s">
+        <v>314</v>
+      </c>
+      <c r="M79" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>377</v>
+      </c>
+      <c r="B80" t="s">
+        <v>417</v>
+      </c>
+      <c r="C80" t="s">
+        <v>394</v>
+      </c>
+      <c r="D80" t="s">
+        <v>394</v>
+      </c>
+      <c r="F80" s="4">
+        <v>25999</v>
+      </c>
+      <c r="G80" t="s">
+        <v>116</v>
+      </c>
+      <c r="H80" t="s">
+        <v>112</v>
+      </c>
+      <c r="I80" t="s">
+        <v>118</v>
+      </c>
+      <c r="L80" t="s">
+        <v>314</v>
+      </c>
+      <c r="M80" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>378</v>
+      </c>
+      <c r="B81" t="s">
+        <v>418</v>
+      </c>
+      <c r="C81" t="s">
+        <v>394</v>
+      </c>
+      <c r="D81" t="s">
+        <v>394</v>
+      </c>
+      <c r="F81" s="4">
+        <v>26027</v>
+      </c>
+      <c r="G81" t="s">
+        <v>116</v>
+      </c>
+      <c r="H81" t="s">
+        <v>112</v>
+      </c>
+      <c r="I81" t="s">
+        <v>118</v>
+      </c>
+      <c r="L81" t="s">
+        <v>314</v>
+      </c>
+      <c r="M81" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>379</v>
+      </c>
+      <c r="B82" t="s">
+        <v>419</v>
+      </c>
+      <c r="C82" t="s">
+        <v>394</v>
+      </c>
+      <c r="D82" t="s">
+        <v>394</v>
+      </c>
+      <c r="F82" s="4">
+        <v>26054</v>
+      </c>
+      <c r="G82" t="s">
+        <v>116</v>
+      </c>
+      <c r="H82" t="s">
+        <v>112</v>
+      </c>
+      <c r="I82" t="s">
+        <v>118</v>
+      </c>
+      <c r="L82" t="s">
+        <v>314</v>
+      </c>
+      <c r="M82" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>380</v>
+      </c>
+      <c r="B83" t="s">
+        <v>420</v>
+      </c>
+      <c r="C83" t="s">
+        <v>394</v>
+      </c>
+      <c r="D83" t="s">
+        <v>394</v>
+      </c>
+      <c r="F83" s="4">
+        <v>26076</v>
+      </c>
+      <c r="G83" t="s">
+        <v>116</v>
+      </c>
+      <c r="H83" t="s">
+        <v>112</v>
+      </c>
+      <c r="I83" t="s">
+        <v>118</v>
+      </c>
+      <c r="L83" t="s">
+        <v>314</v>
+      </c>
+      <c r="M83" s="3" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>381</v>
+      </c>
+      <c r="B84" t="s">
+        <v>421</v>
+      </c>
+      <c r="C84" t="s">
+        <v>394</v>
+      </c>
+      <c r="D84" t="s">
+        <v>394</v>
+      </c>
+      <c r="F84" s="4">
+        <v>26104</v>
+      </c>
+      <c r="G84" t="s">
+        <v>116</v>
+      </c>
+      <c r="H84" t="s">
+        <v>112</v>
+      </c>
+      <c r="I84" t="s">
+        <v>118</v>
+      </c>
+      <c r="L84" t="s">
+        <v>314</v>
+      </c>
+      <c r="M84" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>382</v>
+      </c>
+      <c r="B85" t="s">
+        <v>422</v>
+      </c>
+      <c r="C85" t="s">
+        <v>394</v>
+      </c>
+      <c r="D85" t="s">
+        <v>394</v>
+      </c>
+      <c r="F85" s="4">
+        <v>26139</v>
+      </c>
+      <c r="G85" t="s">
+        <v>116</v>
+      </c>
+      <c r="H85" t="s">
+        <v>112</v>
+      </c>
+      <c r="I85" t="s">
+        <v>118</v>
+      </c>
+      <c r="L85" t="s">
+        <v>314</v>
+      </c>
+      <c r="M85" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>383</v>
+      </c>
+      <c r="B86" t="s">
+        <v>423</v>
+      </c>
+      <c r="C86" t="s">
+        <v>394</v>
+      </c>
+      <c r="D86" t="s">
+        <v>394</v>
+      </c>
+      <c r="F86" s="4">
+        <v>26265</v>
+      </c>
+      <c r="G86" t="s">
+        <v>116</v>
+      </c>
+      <c r="H86" t="s">
+        <v>112</v>
+      </c>
+      <c r="I86" t="s">
+        <v>118</v>
+      </c>
+      <c r="L86" t="s">
+        <v>314</v>
+      </c>
+      <c r="M86" s="3" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>384</v>
+      </c>
+      <c r="B87" t="s">
+        <v>389</v>
+      </c>
+      <c r="C87" t="s">
+        <v>394</v>
+      </c>
+      <c r="D87" t="s">
+        <v>394</v>
+      </c>
+      <c r="F87" s="4">
+        <v>26307</v>
+      </c>
+      <c r="G87" t="s">
+        <v>116</v>
+      </c>
+      <c r="H87" t="s">
+        <v>112</v>
+      </c>
+      <c r="I87" t="s">
+        <v>118</v>
+      </c>
+      <c r="L87" t="s">
+        <v>314</v>
+      </c>
+      <c r="M87" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>385</v>
+      </c>
+      <c r="B88" t="s">
+        <v>390</v>
+      </c>
+      <c r="C88" t="s">
+        <v>394</v>
+      </c>
+      <c r="D88" t="s">
+        <v>394</v>
+      </c>
+      <c r="F88" s="4">
+        <v>26370</v>
+      </c>
+      <c r="G88" t="s">
+        <v>116</v>
+      </c>
+      <c r="H88" t="s">
+        <v>112</v>
+      </c>
+      <c r="I88" t="s">
+        <v>118</v>
+      </c>
+      <c r="L88" t="s">
+        <v>314</v>
+      </c>
+      <c r="M88" s="3" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>386</v>
+      </c>
+      <c r="B89" t="s">
+        <v>391</v>
+      </c>
+      <c r="C89" t="s">
+        <v>394</v>
+      </c>
+      <c r="D89" t="s">
+        <v>394</v>
+      </c>
+      <c r="F89" s="4">
+        <v>26420</v>
+      </c>
+      <c r="G89" t="s">
+        <v>116</v>
+      </c>
+      <c r="H89" t="s">
+        <v>112</v>
+      </c>
+      <c r="I89" t="s">
+        <v>118</v>
+      </c>
+      <c r="L89" t="s">
+        <v>314</v>
+      </c>
+      <c r="M89" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>387</v>
+      </c>
+      <c r="B90" t="s">
+        <v>392</v>
+      </c>
+      <c r="C90" t="s">
+        <v>394</v>
+      </c>
+      <c r="D90" t="s">
+        <v>394</v>
+      </c>
+      <c r="F90" s="4">
+        <v>26608</v>
+      </c>
+      <c r="G90" t="s">
+        <v>116</v>
+      </c>
+      <c r="H90" t="s">
+        <v>112</v>
+      </c>
+      <c r="I90" t="s">
+        <v>118</v>
+      </c>
+      <c r="L90" t="s">
+        <v>314</v>
+      </c>
+      <c r="M90" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>388</v>
+      </c>
+      <c r="B91" t="s">
+        <v>393</v>
+      </c>
+      <c r="C91" t="s">
+        <v>394</v>
+      </c>
+      <c r="D91" t="s">
+        <v>394</v>
+      </c>
+      <c r="F91" s="4">
+        <v>26785</v>
+      </c>
+      <c r="G91" t="s">
+        <v>116</v>
+      </c>
+      <c r="H91" t="s">
+        <v>112</v>
+      </c>
+      <c r="I91" t="s">
+        <v>118</v>
+      </c>
+      <c r="L91" t="s">
+        <v>314</v>
+      </c>
+      <c r="M91" s="3" t="s">
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -4053,10 +5003,33 @@
     <hyperlink ref="M66" r:id="rId65" xr:uid="{8365E924-D46C-4D93-9FDD-E2A533CDCEF8}"/>
     <hyperlink ref="M67" r:id="rId66" xr:uid="{9E0E6191-2474-42FA-BA40-68DA6CAC11D8}"/>
     <hyperlink ref="M68" r:id="rId67" xr:uid="{7538D10C-1B89-41F2-8EF8-6C51156B9F3D}"/>
+    <hyperlink ref="M70" r:id="rId68" xr:uid="{992A5A10-6FA8-441D-9D96-1910EB939BD3}"/>
+    <hyperlink ref="M69" r:id="rId69" xr:uid="{006EA408-C0A6-4811-B052-83CF129EA2C0}"/>
+    <hyperlink ref="M89" r:id="rId70" xr:uid="{928D77CC-3AAA-4B77-AC03-61D687FF16B3}"/>
+    <hyperlink ref="M91" r:id="rId71" xr:uid="{45AC23F1-4EC4-4BAF-8049-0EFBB684BA5C}"/>
+    <hyperlink ref="M71" r:id="rId72" xr:uid="{C7350187-B80D-4F0F-9164-990486FA3ADE}"/>
+    <hyperlink ref="M72" r:id="rId73" xr:uid="{4AD25FBC-7B54-479D-8684-9ED95A508D3C}"/>
+    <hyperlink ref="M73" r:id="rId74" xr:uid="{6422EBC7-589E-44E2-96BD-306A215E30A6}"/>
+    <hyperlink ref="M74" r:id="rId75" xr:uid="{A3070D3B-90C9-499E-BD98-EACA481ED14E}"/>
+    <hyperlink ref="M75" r:id="rId76" xr:uid="{808FAF65-7C15-4E6A-9F54-14CA6A450A96}"/>
+    <hyperlink ref="M76" r:id="rId77" xr:uid="{1DCE5792-408E-469A-8742-17FE6E620712}"/>
+    <hyperlink ref="M77" r:id="rId78" xr:uid="{E33F0CDF-648A-446F-970E-C441D4A5FA6B}"/>
+    <hyperlink ref="M78" r:id="rId79" xr:uid="{FDF98D3A-2BDF-4222-9515-D396FE754728}"/>
+    <hyperlink ref="M79" r:id="rId80" xr:uid="{09F70555-E46E-46FA-8E11-BD505AFF380C}"/>
+    <hyperlink ref="M80" r:id="rId81" xr:uid="{B1CF9F07-1CC5-482D-9B20-938BDAE84FC4}"/>
+    <hyperlink ref="M81" r:id="rId82" xr:uid="{9B9C0FBA-9DA3-44F6-B651-2C6DEE7D8C97}"/>
+    <hyperlink ref="M82" r:id="rId83" xr:uid="{90142248-2915-4038-B9C7-282968CDDAD5}"/>
+    <hyperlink ref="M83" r:id="rId84" xr:uid="{095EBA0A-5F28-4E5A-AF60-AC6DAD8CC4E1}"/>
+    <hyperlink ref="M84" r:id="rId85" xr:uid="{91F4EEAE-C2CF-4DCA-BCB5-FF47689B42B2}"/>
+    <hyperlink ref="M85" r:id="rId86" xr:uid="{C98C421D-3FFF-4959-B494-99F2D5BF189F}"/>
+    <hyperlink ref="M86" r:id="rId87" xr:uid="{2DCC8DBF-33F4-4246-9B50-8489F6E17A99}"/>
+    <hyperlink ref="M87" r:id="rId88" xr:uid="{4D72D9B5-0915-4B7E-9F96-6275A944EE54}"/>
+    <hyperlink ref="M88" r:id="rId89" xr:uid="{8D9593CC-1AC6-4151-A7F0-9E914C39EEA1}"/>
+    <hyperlink ref="M90" r:id="rId90" xr:uid="{734F4C0D-ECE0-4D17-AED2-596C8405BA52}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId68"/>
+    <tablePart r:id="rId91"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4072,19 +5045,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B1" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="C1" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="D1" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="E1" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -4092,7 +5065,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="C2">
         <v>1893</v>
@@ -4101,15 +5074,15 @@
         <v>1976</v>
       </c>
       <c r="E2" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="C3">
         <v>1921</v>
@@ -4118,24 +5091,24 @@
         <v>1993</v>
       </c>
       <c r="E3" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C4" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="D4">
         <v>2021</v>
       </c>
       <c r="E4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -4143,7 +5116,7 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C5">
         <v>1931</v>
@@ -4154,10 +5127,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="B6" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="C6">
         <v>1960</v>
@@ -4168,26 +5141,26 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="B8" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="B9" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="C9">
         <v>1907</v>
@@ -4198,10 +5171,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="B10" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="C10">
         <v>1898</v>
@@ -4212,10 +5185,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="B11" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C11">
         <v>1898</v>
@@ -4226,10 +5199,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B12" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C12">
         <v>1904</v>
@@ -4240,10 +5213,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="B13" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C13">
         <v>1914</v>
@@ -4254,10 +5227,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="B14" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="C14">
         <v>1920</v>
@@ -4268,10 +5241,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B15" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="C15">
         <v>1920</v>
@@ -4282,10 +5255,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="B16" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="C16">
         <v>1898</v>
@@ -4313,33 +5286,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B1" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="C1" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="D1" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="E1" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B2" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="C2">
         <v>1962</v>
       </c>
       <c r="D2" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -4347,7 +5320,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="C3">
         <v>1952</v>
@@ -4358,7 +5331,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="C4">
         <v>1963</v>
@@ -4372,7 +5345,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C5">
         <v>1948</v>
@@ -4380,10 +5353,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="B6" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C6">
         <v>1958</v>
@@ -4397,7 +5370,7 @@
         <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C7">
         <v>1964</v>
@@ -4408,10 +5381,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B8" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C8">
         <v>1956</v>
@@ -4419,10 +5392,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -4430,7 +5403,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C10">
         <v>1966</v>
@@ -4444,7 +5417,7 @@
         <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C11">
         <v>1968</v>
@@ -4455,10 +5428,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="B12" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C12">
         <v>1966</v>
@@ -4469,10 +5442,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C13">
         <v>1921</v>
@@ -4483,7 +5456,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C14">
         <v>1966</v>
@@ -4492,7 +5465,7 @@
         <v>1991</v>
       </c>
       <c r="E14" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -4500,7 +5473,7 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C15">
         <v>1968</v>
@@ -4509,7 +5482,7 @@
         <v>1972</v>
       </c>
       <c r="E15" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -4517,21 +5490,21 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C16">
         <v>1921</v>
       </c>
       <c r="E16" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="B17" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C17">
         <v>1968</v>
@@ -4542,10 +5515,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B18" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C18">
         <v>1969</v>
@@ -4556,24 +5529,24 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="B19" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C19">
         <v>1968</v>
       </c>
       <c r="D19" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="B20" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C20">
         <v>1972</v>
@@ -4584,10 +5557,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="C21">
         <v>1967</v>
@@ -4598,10 +5571,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="B22" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C22">
         <v>1977</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 18/08/2026 12:29
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4409CBC-B7AB-4DB0-93DB-8F3FEC310ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B7B173-7D39-44C1-BA02-E28E555E126B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="453">
   <si>
     <t>ID</t>
   </si>
@@ -1369,6 +1369,18 @@
   </si>
   <si>
     <t>https://archive.org/details/lotta-di-classe-1972-06/mode/2up</t>
+  </si>
+  <si>
+    <t>AMI-0091</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, no. 2</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/lotta-di-classe-1970-02/mode/2up</t>
+  </si>
+  <si>
+    <t>Circoli Lenin dell'Emilia Romanga</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1440,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1437,6 +1449,7 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1456,8 +1469,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:P150" totalsRowShown="0">
-  <autoFilter ref="A1:P150" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}" name="Tabella1" displayName="Tabella1" ref="A1:P151" totalsRowShown="0">
+  <autoFilter ref="A1:P151" xr:uid="{C0C43707-2E5D-4FCB-B56E-4856FC4DF5B6}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{40EB6498-034B-4FD2-B823-BD9BDE560AB5}" name="ID"/>
     <tableColumn id="2" xr3:uid="{E00E7517-D29A-46F7-B049-8E1F1ECC043C}" name="Titolo"/>
@@ -1793,7 +1806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:P92"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="83.88671875" customWidth="1"/>
@@ -4234,7 +4247,7 @@
         <v>367</v>
       </c>
       <c r="B70" t="s">
-        <v>406</v>
+        <v>450</v>
       </c>
       <c r="C70" t="s">
         <v>394</v>
@@ -4242,8 +4255,8 @@
       <c r="D70" t="s">
         <v>394</v>
       </c>
-      <c r="F70" s="4">
-        <v>25718</v>
+      <c r="F70" s="8">
+        <v>25704</v>
       </c>
       <c r="G70" t="s">
         <v>116</v>
@@ -4258,7 +4271,7 @@
         <v>314</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>405</v>
+        <v>451</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
@@ -4266,7 +4279,7 @@
         <v>368</v>
       </c>
       <c r="B71" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C71" t="s">
         <v>394</v>
@@ -4275,7 +4288,7 @@
         <v>394</v>
       </c>
       <c r="F71" s="4">
-        <v>25719</v>
+        <v>25718</v>
       </c>
       <c r="G71" t="s">
         <v>116</v>
@@ -4290,7 +4303,7 @@
         <v>314</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>427</v>
+        <v>405</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
@@ -4298,7 +4311,7 @@
         <v>369</v>
       </c>
       <c r="B72" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C72" t="s">
         <v>394</v>
@@ -4307,7 +4320,7 @@
         <v>394</v>
       </c>
       <c r="F72" s="4">
-        <v>25740</v>
+        <v>25719</v>
       </c>
       <c r="G72" t="s">
         <v>116</v>
@@ -4322,7 +4335,7 @@
         <v>314</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
@@ -4330,7 +4343,7 @@
         <v>370</v>
       </c>
       <c r="B73" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C73" t="s">
         <v>394</v>
@@ -4339,7 +4352,7 @@
         <v>394</v>
       </c>
       <c r="F73" s="4">
-        <v>25765</v>
+        <v>25740</v>
       </c>
       <c r="G73" t="s">
         <v>116</v>
@@ -4354,7 +4367,7 @@
         <v>314</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
@@ -4362,7 +4375,7 @@
         <v>371</v>
       </c>
       <c r="B74" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C74" t="s">
         <v>394</v>
@@ -4371,7 +4384,7 @@
         <v>394</v>
       </c>
       <c r="F74" s="4">
-        <v>25824</v>
+        <v>25765</v>
       </c>
       <c r="G74" t="s">
         <v>116</v>
@@ -4386,7 +4399,7 @@
         <v>314</v>
       </c>
       <c r="M74" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
@@ -4394,7 +4407,7 @@
         <v>372</v>
       </c>
       <c r="B75" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C75" t="s">
         <v>394</v>
@@ -4403,7 +4416,7 @@
         <v>394</v>
       </c>
       <c r="F75" s="4">
-        <v>25866</v>
+        <v>25824</v>
       </c>
       <c r="G75" t="s">
         <v>116</v>
@@ -4418,7 +4431,7 @@
         <v>314</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
@@ -4426,7 +4439,7 @@
         <v>373</v>
       </c>
       <c r="B76" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C76" t="s">
         <v>394</v>
@@ -4435,7 +4448,7 @@
         <v>394</v>
       </c>
       <c r="F76" s="4">
-        <v>25887</v>
+        <v>25866</v>
       </c>
       <c r="G76" t="s">
         <v>116</v>
@@ -4450,7 +4463,7 @@
         <v>314</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
@@ -4458,7 +4471,7 @@
         <v>374</v>
       </c>
       <c r="B77" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C77" t="s">
         <v>394</v>
@@ -4467,7 +4480,7 @@
         <v>394</v>
       </c>
       <c r="F77" s="4">
-        <v>25915</v>
+        <v>25887</v>
       </c>
       <c r="G77" t="s">
         <v>116</v>
@@ -4482,7 +4495,7 @@
         <v>314</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
@@ -4490,7 +4503,7 @@
         <v>375</v>
       </c>
       <c r="B78" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C78" t="s">
         <v>394</v>
@@ -4499,7 +4512,7 @@
         <v>394</v>
       </c>
       <c r="F78" s="4">
-        <v>25950</v>
+        <v>25915</v>
       </c>
       <c r="G78" t="s">
         <v>116</v>
@@ -4514,7 +4527,7 @@
         <v>314</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
@@ -4522,7 +4535,7 @@
         <v>376</v>
       </c>
       <c r="B79" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C79" t="s">
         <v>394</v>
@@ -4531,7 +4544,7 @@
         <v>394</v>
       </c>
       <c r="F79" s="4">
-        <v>25971</v>
+        <v>25950</v>
       </c>
       <c r="G79" t="s">
         <v>116</v>
@@ -4546,7 +4559,7 @@
         <v>314</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
@@ -4554,7 +4567,7 @@
         <v>377</v>
       </c>
       <c r="B80" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C80" t="s">
         <v>394</v>
@@ -4563,7 +4576,7 @@
         <v>394</v>
       </c>
       <c r="F80" s="4">
-        <v>25999</v>
+        <v>25971</v>
       </c>
       <c r="G80" t="s">
         <v>116</v>
@@ -4578,7 +4591,7 @@
         <v>314</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
@@ -4586,7 +4599,7 @@
         <v>378</v>
       </c>
       <c r="B81" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C81" t="s">
         <v>394</v>
@@ -4595,7 +4608,7 @@
         <v>394</v>
       </c>
       <c r="F81" s="4">
-        <v>26027</v>
+        <v>25999</v>
       </c>
       <c r="G81" t="s">
         <v>116</v>
@@ -4610,7 +4623,7 @@
         <v>314</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
@@ -4618,7 +4631,7 @@
         <v>379</v>
       </c>
       <c r="B82" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C82" t="s">
         <v>394</v>
@@ -4627,7 +4640,7 @@
         <v>394</v>
       </c>
       <c r="F82" s="4">
-        <v>26054</v>
+        <v>26027</v>
       </c>
       <c r="G82" t="s">
         <v>116</v>
@@ -4642,7 +4655,7 @@
         <v>314</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
@@ -4650,7 +4663,7 @@
         <v>380</v>
       </c>
       <c r="B83" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C83" t="s">
         <v>394</v>
@@ -4659,7 +4672,7 @@
         <v>394</v>
       </c>
       <c r="F83" s="4">
-        <v>26076</v>
+        <v>26054</v>
       </c>
       <c r="G83" t="s">
         <v>116</v>
@@ -4674,7 +4687,7 @@
         <v>314</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
@@ -4682,7 +4695,7 @@
         <v>381</v>
       </c>
       <c r="B84" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C84" t="s">
         <v>394</v>
@@ -4691,7 +4704,7 @@
         <v>394</v>
       </c>
       <c r="F84" s="4">
-        <v>26104</v>
+        <v>26076</v>
       </c>
       <c r="G84" t="s">
         <v>116</v>
@@ -4706,7 +4719,7 @@
         <v>314</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
@@ -4714,7 +4727,7 @@
         <v>382</v>
       </c>
       <c r="B85" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C85" t="s">
         <v>394</v>
@@ -4723,7 +4736,7 @@
         <v>394</v>
       </c>
       <c r="F85" s="4">
-        <v>26139</v>
+        <v>26104</v>
       </c>
       <c r="G85" t="s">
         <v>116</v>
@@ -4738,7 +4751,7 @@
         <v>314</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
@@ -4746,7 +4759,7 @@
         <v>383</v>
       </c>
       <c r="B86" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C86" t="s">
         <v>394</v>
@@ -4755,7 +4768,7 @@
         <v>394</v>
       </c>
       <c r="F86" s="4">
-        <v>26265</v>
+        <v>26139</v>
       </c>
       <c r="G86" t="s">
         <v>116</v>
@@ -4770,7 +4783,7 @@
         <v>314</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
@@ -4778,7 +4791,7 @@
         <v>384</v>
       </c>
       <c r="B87" t="s">
-        <v>389</v>
+        <v>423</v>
       </c>
       <c r="C87" t="s">
         <v>394</v>
@@ -4787,7 +4800,7 @@
         <v>394</v>
       </c>
       <c r="F87" s="4">
-        <v>26307</v>
+        <v>26265</v>
       </c>
       <c r="G87" t="s">
         <v>116</v>
@@ -4802,7 +4815,7 @@
         <v>314</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
@@ -4810,7 +4823,7 @@
         <v>385</v>
       </c>
       <c r="B88" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C88" t="s">
         <v>394</v>
@@ -4819,7 +4832,7 @@
         <v>394</v>
       </c>
       <c r="F88" s="4">
-        <v>26370</v>
+        <v>26307</v>
       </c>
       <c r="G88" t="s">
         <v>116</v>
@@ -4834,7 +4847,7 @@
         <v>314</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
@@ -4842,7 +4855,7 @@
         <v>386</v>
       </c>
       <c r="B89" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C89" t="s">
         <v>394</v>
@@ -4851,7 +4864,7 @@
         <v>394</v>
       </c>
       <c r="F89" s="4">
-        <v>26420</v>
+        <v>26370</v>
       </c>
       <c r="G89" t="s">
         <v>116</v>
@@ -4866,7 +4879,7 @@
         <v>314</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>425</v>
+        <v>447</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
@@ -4874,7 +4887,7 @@
         <v>387</v>
       </c>
       <c r="B90" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C90" t="s">
         <v>394</v>
@@ -4883,7 +4896,7 @@
         <v>394</v>
       </c>
       <c r="F90" s="4">
-        <v>26608</v>
+        <v>26420</v>
       </c>
       <c r="G90" t="s">
         <v>116</v>
@@ -4898,7 +4911,7 @@
         <v>314</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>448</v>
+        <v>425</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
@@ -4906,7 +4919,7 @@
         <v>388</v>
       </c>
       <c r="B91" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C91" t="s">
         <v>394</v>
@@ -4915,7 +4928,7 @@
         <v>394</v>
       </c>
       <c r="F91" s="4">
-        <v>26785</v>
+        <v>26608</v>
       </c>
       <c r="G91" t="s">
         <v>116</v>
@@ -4930,6 +4943,38 @@
         <v>314</v>
       </c>
       <c r="M91" s="3" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>449</v>
+      </c>
+      <c r="B92" t="s">
+        <v>393</v>
+      </c>
+      <c r="C92" t="s">
+        <v>394</v>
+      </c>
+      <c r="D92" t="s">
+        <v>394</v>
+      </c>
+      <c r="F92" s="4">
+        <v>26785</v>
+      </c>
+      <c r="G92" t="s">
+        <v>116</v>
+      </c>
+      <c r="H92" t="s">
+        <v>112</v>
+      </c>
+      <c r="I92" t="s">
+        <v>118</v>
+      </c>
+      <c r="L92" t="s">
+        <v>314</v>
+      </c>
+      <c r="M92" s="3" t="s">
         <v>426</v>
       </c>
     </row>
@@ -5003,33 +5048,34 @@
     <hyperlink ref="M66" r:id="rId65" xr:uid="{8365E924-D46C-4D93-9FDD-E2A533CDCEF8}"/>
     <hyperlink ref="M67" r:id="rId66" xr:uid="{9E0E6191-2474-42FA-BA40-68DA6CAC11D8}"/>
     <hyperlink ref="M68" r:id="rId67" xr:uid="{7538D10C-1B89-41F2-8EF8-6C51156B9F3D}"/>
-    <hyperlink ref="M70" r:id="rId68" xr:uid="{992A5A10-6FA8-441D-9D96-1910EB939BD3}"/>
+    <hyperlink ref="M71" r:id="rId68" xr:uid="{992A5A10-6FA8-441D-9D96-1910EB939BD3}"/>
     <hyperlink ref="M69" r:id="rId69" xr:uid="{006EA408-C0A6-4811-B052-83CF129EA2C0}"/>
-    <hyperlink ref="M89" r:id="rId70" xr:uid="{928D77CC-3AAA-4B77-AC03-61D687FF16B3}"/>
-    <hyperlink ref="M91" r:id="rId71" xr:uid="{45AC23F1-4EC4-4BAF-8049-0EFBB684BA5C}"/>
-    <hyperlink ref="M71" r:id="rId72" xr:uid="{C7350187-B80D-4F0F-9164-990486FA3ADE}"/>
-    <hyperlink ref="M72" r:id="rId73" xr:uid="{4AD25FBC-7B54-479D-8684-9ED95A508D3C}"/>
-    <hyperlink ref="M73" r:id="rId74" xr:uid="{6422EBC7-589E-44E2-96BD-306A215E30A6}"/>
-    <hyperlink ref="M74" r:id="rId75" xr:uid="{A3070D3B-90C9-499E-BD98-EACA481ED14E}"/>
-    <hyperlink ref="M75" r:id="rId76" xr:uid="{808FAF65-7C15-4E6A-9F54-14CA6A450A96}"/>
-    <hyperlink ref="M76" r:id="rId77" xr:uid="{1DCE5792-408E-469A-8742-17FE6E620712}"/>
-    <hyperlink ref="M77" r:id="rId78" xr:uid="{E33F0CDF-648A-446F-970E-C441D4A5FA6B}"/>
-    <hyperlink ref="M78" r:id="rId79" xr:uid="{FDF98D3A-2BDF-4222-9515-D396FE754728}"/>
-    <hyperlink ref="M79" r:id="rId80" xr:uid="{09F70555-E46E-46FA-8E11-BD505AFF380C}"/>
-    <hyperlink ref="M80" r:id="rId81" xr:uid="{B1CF9F07-1CC5-482D-9B20-938BDAE84FC4}"/>
-    <hyperlink ref="M81" r:id="rId82" xr:uid="{9B9C0FBA-9DA3-44F6-B651-2C6DEE7D8C97}"/>
-    <hyperlink ref="M82" r:id="rId83" xr:uid="{90142248-2915-4038-B9C7-282968CDDAD5}"/>
-    <hyperlink ref="M83" r:id="rId84" xr:uid="{095EBA0A-5F28-4E5A-AF60-AC6DAD8CC4E1}"/>
-    <hyperlink ref="M84" r:id="rId85" xr:uid="{91F4EEAE-C2CF-4DCA-BCB5-FF47689B42B2}"/>
-    <hyperlink ref="M85" r:id="rId86" xr:uid="{C98C421D-3FFF-4959-B494-99F2D5BF189F}"/>
-    <hyperlink ref="M86" r:id="rId87" xr:uid="{2DCC8DBF-33F4-4246-9B50-8489F6E17A99}"/>
-    <hyperlink ref="M87" r:id="rId88" xr:uid="{4D72D9B5-0915-4B7E-9F96-6275A944EE54}"/>
-    <hyperlink ref="M88" r:id="rId89" xr:uid="{8D9593CC-1AC6-4151-A7F0-9E914C39EEA1}"/>
-    <hyperlink ref="M90" r:id="rId90" xr:uid="{734F4C0D-ECE0-4D17-AED2-596C8405BA52}"/>
+    <hyperlink ref="M90" r:id="rId70" xr:uid="{928D77CC-3AAA-4B77-AC03-61D687FF16B3}"/>
+    <hyperlink ref="M92" r:id="rId71" xr:uid="{45AC23F1-4EC4-4BAF-8049-0EFBB684BA5C}"/>
+    <hyperlink ref="M72" r:id="rId72" xr:uid="{C7350187-B80D-4F0F-9164-990486FA3ADE}"/>
+    <hyperlink ref="M73" r:id="rId73" xr:uid="{4AD25FBC-7B54-479D-8684-9ED95A508D3C}"/>
+    <hyperlink ref="M74" r:id="rId74" xr:uid="{6422EBC7-589E-44E2-96BD-306A215E30A6}"/>
+    <hyperlink ref="M75" r:id="rId75" xr:uid="{A3070D3B-90C9-499E-BD98-EACA481ED14E}"/>
+    <hyperlink ref="M76" r:id="rId76" xr:uid="{808FAF65-7C15-4E6A-9F54-14CA6A450A96}"/>
+    <hyperlink ref="M77" r:id="rId77" xr:uid="{1DCE5792-408E-469A-8742-17FE6E620712}"/>
+    <hyperlink ref="M78" r:id="rId78" xr:uid="{E33F0CDF-648A-446F-970E-C441D4A5FA6B}"/>
+    <hyperlink ref="M79" r:id="rId79" xr:uid="{FDF98D3A-2BDF-4222-9515-D396FE754728}"/>
+    <hyperlink ref="M80" r:id="rId80" xr:uid="{09F70555-E46E-46FA-8E11-BD505AFF380C}"/>
+    <hyperlink ref="M81" r:id="rId81" xr:uid="{B1CF9F07-1CC5-482D-9B20-938BDAE84FC4}"/>
+    <hyperlink ref="M82" r:id="rId82" xr:uid="{9B9C0FBA-9DA3-44F6-B651-2C6DEE7D8C97}"/>
+    <hyperlink ref="M83" r:id="rId83" xr:uid="{90142248-2915-4038-B9C7-282968CDDAD5}"/>
+    <hyperlink ref="M84" r:id="rId84" xr:uid="{095EBA0A-5F28-4E5A-AF60-AC6DAD8CC4E1}"/>
+    <hyperlink ref="M85" r:id="rId85" xr:uid="{91F4EEAE-C2CF-4DCA-BCB5-FF47689B42B2}"/>
+    <hyperlink ref="M86" r:id="rId86" xr:uid="{C98C421D-3FFF-4959-B494-99F2D5BF189F}"/>
+    <hyperlink ref="M87" r:id="rId87" xr:uid="{2DCC8DBF-33F4-4246-9B50-8489F6E17A99}"/>
+    <hyperlink ref="M88" r:id="rId88" xr:uid="{4D72D9B5-0915-4B7E-9F96-6275A944EE54}"/>
+    <hyperlink ref="M89" r:id="rId89" xr:uid="{8D9593CC-1AC6-4151-A7F0-9E914C39EEA1}"/>
+    <hyperlink ref="M91" r:id="rId90" xr:uid="{734F4C0D-ECE0-4D17-AED2-596C8405BA52}"/>
+    <hyperlink ref="M70" r:id="rId91" xr:uid="{410C497E-B7A6-4A52-BDB5-CD7FDB43C527}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId91"/>
+    <tablePart r:id="rId92"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5277,7 +5323,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.33203125" customWidth="1"/>
@@ -5583,6 +5629,20 @@
         <v>1984</v>
       </c>
     </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>452</v>
+      </c>
+      <c r="B23" t="s">
+        <v>295</v>
+      </c>
+      <c r="C23">
+        <v>1970</v>
+      </c>
+      <c r="D23">
+        <v>1973</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 18/08/2026 12:38
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9977EE36-C23C-44AF-A1F9-5D6B1F142855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3D3E7B-5874-435A-9405-09B5D4B391F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="452">
   <si>
     <t>ID</t>
   </si>
@@ -1378,9 +1378,6 @@
   </si>
   <si>
     <t>https://archive.org/details/lotta-di-classe-1970-02/mode/2up</t>
-  </si>
-  <si>
-    <t>Circoli Lenin dell'Emilia Romanga</t>
   </si>
 </sst>
 </file>
@@ -5632,7 +5629,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>452</v>
+        <v>394</v>
       </c>
       <c r="B23" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 23/08/2026 14:24
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3D3E7B-5874-435A-9405-09B5D4B391F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3C44EE-E131-40CD-ADF8-0B584979E005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -1203,9 +1203,6 @@
     <t>Lotta di Classe, anno III, no. 6</t>
   </si>
   <si>
-    <t>Lotta di Classe, anno IV, no. 1</t>
-  </si>
-  <si>
     <t>Circoli Lenin dell'Emilia Romagna</t>
   </si>
   <si>
@@ -1378,6 +1375,9 @@
   </si>
   <si>
     <t>https://archive.org/details/lotta-di-classe-1970-02/mode/2up</t>
+  </si>
+  <si>
+    <t>Lotta di Classe, anno IV, no. 1/2</t>
   </si>
 </sst>
 </file>
@@ -2580,7 +2580,7 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C22" t="s">
         <v>114</v>
@@ -2612,7 +2612,7 @@
         <v>120</v>
       </c>
       <c r="B23" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C23" t="s">
         <v>114</v>
@@ -2644,7 +2644,7 @@
         <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C24" t="s">
         <v>114</v>
@@ -2676,7 +2676,7 @@
         <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C25" t="s">
         <v>114</v>
@@ -2708,7 +2708,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C26" t="s">
         <v>114</v>
@@ -2740,7 +2740,7 @@
         <v>127</v>
       </c>
       <c r="B27" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C27" t="s">
         <v>114</v>
@@ -2772,7 +2772,7 @@
         <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C28" t="s">
         <v>114</v>
@@ -2804,7 +2804,7 @@
         <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C29" t="s">
         <v>114</v>
@@ -2839,7 +2839,7 @@
         <v>132</v>
       </c>
       <c r="B30" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C30" t="s">
         <v>114</v>
@@ -4077,7 +4077,7 @@
         <v>338</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
@@ -4109,7 +4109,7 @@
         <v>338</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
@@ -4202,7 +4202,7 @@
         <v>316</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="N68" t="s">
         <v>349</v>
@@ -4213,16 +4213,16 @@
         <v>366</v>
       </c>
       <c r="B69" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C69" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D69" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G69" t="s">
         <v>116</v>
@@ -4237,7 +4237,7 @@
         <v>314</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
@@ -4245,13 +4245,13 @@
         <v>367</v>
       </c>
       <c r="B70" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C70" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D70" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F70" s="8">
         <v>25704</v>
@@ -4269,7 +4269,7 @@
         <v>314</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
@@ -4277,13 +4277,13 @@
         <v>368</v>
       </c>
       <c r="B71" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C71" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D71" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F71" s="4">
         <v>25718</v>
@@ -4301,7 +4301,7 @@
         <v>314</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
@@ -4309,13 +4309,13 @@
         <v>369</v>
       </c>
       <c r="B72" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C72" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D72" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F72" s="4">
         <v>25719</v>
@@ -4333,7 +4333,7 @@
         <v>314</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
@@ -4341,13 +4341,13 @@
         <v>370</v>
       </c>
       <c r="B73" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C73" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D73" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F73" s="4">
         <v>25740</v>
@@ -4365,7 +4365,7 @@
         <v>314</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
@@ -4373,13 +4373,13 @@
         <v>371</v>
       </c>
       <c r="B74" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C74" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D74" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F74" s="4">
         <v>25765</v>
@@ -4397,7 +4397,7 @@
         <v>314</v>
       </c>
       <c r="M74" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
@@ -4405,13 +4405,13 @@
         <v>372</v>
       </c>
       <c r="B75" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C75" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D75" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F75" s="4">
         <v>25824</v>
@@ -4429,7 +4429,7 @@
         <v>314</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
@@ -4437,13 +4437,13 @@
         <v>373</v>
       </c>
       <c r="B76" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C76" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D76" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F76" s="4">
         <v>25866</v>
@@ -4461,7 +4461,7 @@
         <v>314</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
@@ -4469,13 +4469,13 @@
         <v>374</v>
       </c>
       <c r="B77" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C77" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D77" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F77" s="4">
         <v>25887</v>
@@ -4493,7 +4493,7 @@
         <v>314</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
@@ -4501,13 +4501,13 @@
         <v>375</v>
       </c>
       <c r="B78" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C78" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D78" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F78" s="4">
         <v>25915</v>
@@ -4525,7 +4525,7 @@
         <v>314</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
@@ -4533,13 +4533,13 @@
         <v>376</v>
       </c>
       <c r="B79" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C79" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D79" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F79" s="4">
         <v>25950</v>
@@ -4557,7 +4557,7 @@
         <v>314</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
@@ -4565,13 +4565,13 @@
         <v>377</v>
       </c>
       <c r="B80" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C80" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D80" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F80" s="4">
         <v>25971</v>
@@ -4589,7 +4589,7 @@
         <v>314</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
@@ -4597,13 +4597,13 @@
         <v>378</v>
       </c>
       <c r="B81" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C81" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D81" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F81" s="4">
         <v>25999</v>
@@ -4621,7 +4621,7 @@
         <v>314</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
@@ -4629,13 +4629,13 @@
         <v>379</v>
       </c>
       <c r="B82" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C82" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D82" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F82" s="4">
         <v>26027</v>
@@ -4653,7 +4653,7 @@
         <v>314</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
@@ -4661,13 +4661,13 @@
         <v>380</v>
       </c>
       <c r="B83" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C83" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D83" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F83" s="4">
         <v>26054</v>
@@ -4685,7 +4685,7 @@
         <v>314</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
@@ -4693,13 +4693,13 @@
         <v>381</v>
       </c>
       <c r="B84" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C84" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D84" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F84" s="4">
         <v>26076</v>
@@ -4717,7 +4717,7 @@
         <v>314</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
@@ -4725,13 +4725,13 @@
         <v>382</v>
       </c>
       <c r="B85" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C85" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D85" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F85" s="4">
         <v>26104</v>
@@ -4749,7 +4749,7 @@
         <v>314</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
@@ -4757,13 +4757,13 @@
         <v>383</v>
       </c>
       <c r="B86" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C86" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D86" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F86" s="4">
         <v>26139</v>
@@ -4781,7 +4781,7 @@
         <v>314</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
@@ -4789,13 +4789,13 @@
         <v>384</v>
       </c>
       <c r="B87" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C87" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D87" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F87" s="4">
         <v>26265</v>
@@ -4813,7 +4813,7 @@
         <v>314</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
@@ -4824,10 +4824,10 @@
         <v>389</v>
       </c>
       <c r="C88" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D88" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F88" s="4">
         <v>26307</v>
@@ -4845,7 +4845,7 @@
         <v>314</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
@@ -4856,10 +4856,10 @@
         <v>390</v>
       </c>
       <c r="C89" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D89" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F89" s="4">
         <v>26370</v>
@@ -4877,7 +4877,7 @@
         <v>314</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
@@ -4888,10 +4888,10 @@
         <v>391</v>
       </c>
       <c r="C90" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D90" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F90" s="4">
         <v>26420</v>
@@ -4909,7 +4909,7 @@
         <v>314</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
@@ -4920,10 +4920,10 @@
         <v>392</v>
       </c>
       <c r="C91" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D91" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F91" s="4">
         <v>26608</v>
@@ -4941,21 +4941,21 @@
         <v>314</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B92" t="s">
+        <v>451</v>
+      </c>
+      <c r="C92" t="s">
         <v>393</v>
       </c>
-      <c r="C92" t="s">
-        <v>394</v>
-      </c>
       <c r="D92" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F92" s="4">
         <v>26785</v>
@@ -4973,7 +4973,7 @@
         <v>314</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -5629,7 +5629,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B23" t="s">
         <v>295</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/09/2026 14:54
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3C44EE-E131-40CD-ADF8-0B584979E005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A35D228-921D-49C6-8E4C-C7EAA557DF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="451">
   <si>
     <t>ID</t>
   </si>
@@ -817,9 +817,6 @@
   </si>
   <si>
     <t>Pesce</t>
-  </si>
-  <si>
-    <t>193?</t>
   </si>
   <si>
     <t>pesce.webp</t>
@@ -1854,7 +1851,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M1" t="s">
         <v>11</v>
@@ -1898,7 +1895,7 @@
         <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>23</v>
@@ -1933,7 +1930,7 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>28</v>
@@ -1968,7 +1965,7 @@
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>31</v>
@@ -2003,7 +2000,7 @@
         <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>35</v>
@@ -2038,7 +2035,7 @@
         <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>38</v>
@@ -2073,7 +2070,7 @@
         <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>41</v>
@@ -2108,7 +2105,7 @@
         <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>44</v>
@@ -2143,7 +2140,7 @@
         <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>47</v>
@@ -2178,7 +2175,7 @@
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>50</v>
@@ -2213,7 +2210,7 @@
         <v>34</v>
       </c>
       <c r="L11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>53</v>
@@ -2251,7 +2248,7 @@
         <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>57</v>
@@ -2286,7 +2283,7 @@
         <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>61</v>
@@ -2327,7 +2324,7 @@
         <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>71</v>
@@ -2362,7 +2359,7 @@
         <v>76</v>
       </c>
       <c r="L15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>77</v>
@@ -2400,7 +2397,7 @@
         <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>83</v>
@@ -2438,7 +2435,7 @@
         <v>87</v>
       </c>
       <c r="L17" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>88</v>
@@ -2473,7 +2470,7 @@
         <v>68</v>
       </c>
       <c r="L18" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>96</v>
@@ -2505,7 +2502,7 @@
         <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>100</v>
@@ -2537,7 +2534,7 @@
         <v>106</v>
       </c>
       <c r="L20" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>107</v>
@@ -2569,10 +2566,10 @@
         <v>106</v>
       </c>
       <c r="L21" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -2580,7 +2577,7 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C22" t="s">
         <v>114</v>
@@ -2589,7 +2586,7 @@
         <v>115</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G22" t="s">
         <v>116</v>
@@ -2601,7 +2598,7 @@
         <v>118</v>
       </c>
       <c r="L22" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>119</v>
@@ -2612,7 +2609,7 @@
         <v>120</v>
       </c>
       <c r="B23" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C23" t="s">
         <v>114</v>
@@ -2621,7 +2618,7 @@
         <v>115</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G23" t="s">
         <v>116</v>
@@ -2633,10 +2630,10 @@
         <v>118</v>
       </c>
       <c r="L23" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -2644,7 +2641,7 @@
         <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C24" t="s">
         <v>114</v>
@@ -2653,7 +2650,7 @@
         <v>115</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G24" t="s">
         <v>116</v>
@@ -2665,7 +2662,7 @@
         <v>118</v>
       </c>
       <c r="L24" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>122</v>
@@ -2676,7 +2673,7 @@
         <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C25" t="s">
         <v>114</v>
@@ -2685,7 +2682,7 @@
         <v>115</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G25" t="s">
         <v>116</v>
@@ -2697,7 +2694,7 @@
         <v>118</v>
       </c>
       <c r="L25" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>124</v>
@@ -2708,7 +2705,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C26" t="s">
         <v>114</v>
@@ -2717,7 +2714,7 @@
         <v>115</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G26" t="s">
         <v>116</v>
@@ -2729,7 +2726,7 @@
         <v>118</v>
       </c>
       <c r="L26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>126</v>
@@ -2740,7 +2737,7 @@
         <v>127</v>
       </c>
       <c r="B27" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C27" t="s">
         <v>114</v>
@@ -2749,7 +2746,7 @@
         <v>115</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G27" t="s">
         <v>116</v>
@@ -2761,10 +2758,10 @@
         <v>118</v>
       </c>
       <c r="L27" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2772,7 +2769,7 @@
         <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C28" t="s">
         <v>114</v>
@@ -2781,7 +2778,7 @@
         <v>115</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G28" t="s">
         <v>116</v>
@@ -2793,7 +2790,7 @@
         <v>118</v>
       </c>
       <c r="L28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>129</v>
@@ -2804,7 +2801,7 @@
         <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C29" t="s">
         <v>114</v>
@@ -2813,7 +2810,7 @@
         <v>115</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G29" t="s">
         <v>116</v>
@@ -2828,7 +2825,7 @@
         <v>64</v>
       </c>
       <c r="L29" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>131</v>
@@ -2839,7 +2836,7 @@
         <v>132</v>
       </c>
       <c r="B30" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C30" t="s">
         <v>114</v>
@@ -2848,7 +2845,7 @@
         <v>115</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G30" t="s">
         <v>116</v>
@@ -2863,7 +2860,7 @@
         <v>133</v>
       </c>
       <c r="L30" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>134</v>
@@ -2898,7 +2895,7 @@
         <v>34</v>
       </c>
       <c r="L31" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>138</v>
@@ -2933,7 +2930,7 @@
         <v>34</v>
       </c>
       <c r="L32" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>141</v>
@@ -2962,7 +2959,7 @@
         <v>146</v>
       </c>
       <c r="L33" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>147</v>
@@ -3000,7 +2997,7 @@
         <v>17</v>
       </c>
       <c r="L34" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>153</v>
@@ -3044,7 +3041,7 @@
         <v>64</v>
       </c>
       <c r="L35" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>159</v>
@@ -3067,7 +3064,7 @@
         <v>92</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G36" t="s">
         <v>116</v>
@@ -3079,7 +3076,7 @@
         <v>68</v>
       </c>
       <c r="L36" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>165</v>
@@ -3117,7 +3114,7 @@
         <v>144</v>
       </c>
       <c r="L37" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>170</v>
@@ -3152,7 +3149,7 @@
         <v>34</v>
       </c>
       <c r="L38" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>173</v>
@@ -3190,7 +3187,7 @@
         <v>177</v>
       </c>
       <c r="L39" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>178</v>
@@ -3225,7 +3222,7 @@
         <v>181</v>
       </c>
       <c r="L40" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>182</v>
@@ -3260,7 +3257,7 @@
         <v>34</v>
       </c>
       <c r="L41" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>186</v>
@@ -3292,7 +3289,7 @@
         <v>190</v>
       </c>
       <c r="L42" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>191</v>
@@ -3330,7 +3327,7 @@
         <v>196</v>
       </c>
       <c r="L43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>197</v>
@@ -3365,7 +3362,7 @@
         <v>27</v>
       </c>
       <c r="L44" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>200</v>
@@ -3400,7 +3397,7 @@
         <v>27</v>
       </c>
       <c r="L45" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>203</v>
@@ -3435,7 +3432,7 @@
         <v>27</v>
       </c>
       <c r="L46" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>206</v>
@@ -3470,7 +3467,7 @@
         <v>34</v>
       </c>
       <c r="L47" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>209</v>
@@ -3505,7 +3502,7 @@
         <v>34</v>
       </c>
       <c r="L48" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>212</v>
@@ -3540,7 +3537,7 @@
         <v>27</v>
       </c>
       <c r="L49" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>215</v>
@@ -3575,7 +3572,7 @@
         <v>27</v>
       </c>
       <c r="L50" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M50" s="3" t="s">
         <v>218</v>
@@ -3610,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="L51" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M51" s="3" t="s">
         <v>221</v>
@@ -3645,7 +3642,7 @@
         <v>34</v>
       </c>
       <c r="L52" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>224</v>
@@ -3680,7 +3677,7 @@
         <v>68</v>
       </c>
       <c r="L53" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M53" s="3" t="s">
         <v>229</v>
@@ -3712,7 +3709,7 @@
         <v>233</v>
       </c>
       <c r="L54" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M54" s="3" t="s">
         <v>234</v>
@@ -3735,7 +3732,7 @@
         <v>238</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G55" t="s">
         <v>239</v>
@@ -3750,7 +3747,7 @@
         <v>240</v>
       </c>
       <c r="L55" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M55" s="3" t="s">
         <v>241</v>
@@ -3785,7 +3782,7 @@
         <v>68</v>
       </c>
       <c r="L56" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M56" s="3" t="s">
         <v>245</v>
@@ -3823,7 +3820,7 @@
         <v>190</v>
       </c>
       <c r="L57" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M57" s="3" t="s">
         <v>249</v>
@@ -3834,7 +3831,7 @@
         <v>250</v>
       </c>
       <c r="B58" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C58" t="s">
         <v>237</v>
@@ -3864,7 +3861,7 @@
         <v>251</v>
       </c>
       <c r="L58" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>252</v>
@@ -3875,16 +3872,16 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C59" t="s">
         <v>99</v>
       </c>
       <c r="D59" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E59" t="s">
         <v>99</v>
@@ -3902,24 +3899,24 @@
         <v>106</v>
       </c>
       <c r="L59" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>306</v>
+      </c>
+      <c r="B60" t="s">
         <v>307</v>
-      </c>
-      <c r="B60" t="s">
-        <v>308</v>
       </c>
       <c r="C60" t="s">
         <v>99</v>
       </c>
       <c r="D60" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E60" t="s">
         <v>99</v>
@@ -3937,24 +3934,24 @@
         <v>106</v>
       </c>
       <c r="L60" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>316</v>
+      </c>
+      <c r="B61" t="s">
         <v>317</v>
-      </c>
-      <c r="B61" t="s">
-        <v>318</v>
       </c>
       <c r="C61" t="s">
         <v>99</v>
       </c>
       <c r="D61" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E61" t="s">
         <v>99</v>
@@ -3972,21 +3969,21 @@
         <v>106</v>
       </c>
       <c r="J61" t="s">
+        <v>319</v>
+      </c>
+      <c r="L61" t="s">
+        <v>315</v>
+      </c>
+      <c r="M61" s="3" t="s">
         <v>320</v>
-      </c>
-      <c r="L61" t="s">
-        <v>316</v>
-      </c>
-      <c r="M61" s="3" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>325</v>
+      </c>
+      <c r="B62" t="s">
         <v>326</v>
-      </c>
-      <c r="B62" t="s">
-        <v>327</v>
       </c>
       <c r="C62" t="s">
         <v>17</v>
@@ -4010,18 +4007,18 @@
         <v>27</v>
       </c>
       <c r="L62" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>328</v>
+      </c>
+      <c r="B63" t="s">
         <v>329</v>
-      </c>
-      <c r="B63" t="s">
-        <v>330</v>
       </c>
       <c r="F63" s="4">
         <v>24917</v>
@@ -4030,30 +4027,30 @@
         <v>75</v>
       </c>
       <c r="H63" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I63" t="s">
         <v>106</v>
       </c>
       <c r="K63" t="s">
+        <v>331</v>
+      </c>
+      <c r="L63" t="s">
+        <v>315</v>
+      </c>
+      <c r="M63" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="L63" t="s">
-        <v>316</v>
-      </c>
-      <c r="M63" s="3" t="s">
+      <c r="N63" t="s">
         <v>333</v>
-      </c>
-      <c r="N63" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B64" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C64" t="s">
         <v>233</v>
@@ -4062,36 +4059,36 @@
         <v>233</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G64" t="s">
         <v>94</v>
       </c>
       <c r="H64" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I64" t="s">
         <v>68</v>
       </c>
       <c r="L64" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B65" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C65" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D65" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F65" s="4">
         <v>26956</v>
@@ -4100,24 +4097,24 @@
         <v>94</v>
       </c>
       <c r="H65" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I65" t="s">
         <v>68</v>
       </c>
       <c r="L65" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>341</v>
+      </c>
+      <c r="B66" t="s">
         <v>342</v>
-      </c>
-      <c r="B66" t="s">
-        <v>343</v>
       </c>
       <c r="C66" t="s">
         <v>64</v>
@@ -4135,24 +4132,24 @@
         <v>68</v>
       </c>
       <c r="L66" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="N66" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>344</v>
+      </c>
+      <c r="B67" t="s">
         <v>345</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>346</v>
-      </c>
-      <c r="C67" t="s">
-        <v>347</v>
       </c>
       <c r="F67">
         <v>1970</v>
@@ -4167,27 +4164,27 @@
         <v>68</v>
       </c>
       <c r="L67" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="N67" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>351</v>
+      </c>
+      <c r="B68" t="s">
         <v>352</v>
-      </c>
-      <c r="B68" t="s">
-        <v>353</v>
       </c>
       <c r="C68" t="s">
         <v>64</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G68" t="s">
         <v>94</v>
@@ -4199,30 +4196,30 @@
         <v>68</v>
       </c>
       <c r="L68" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="N68" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B69" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C69" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D69" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G69" t="s">
         <v>116</v>
@@ -4234,24 +4231,24 @@
         <v>118</v>
       </c>
       <c r="L69" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B70" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C70" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D70" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F70" s="8">
         <v>25704</v>
@@ -4266,24 +4263,24 @@
         <v>118</v>
       </c>
       <c r="L70" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B71" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C71" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D71" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F71" s="4">
         <v>25718</v>
@@ -4298,24 +4295,24 @@
         <v>118</v>
       </c>
       <c r="L71" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B72" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C72" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D72" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F72" s="4">
         <v>25719</v>
@@ -4330,24 +4327,24 @@
         <v>118</v>
       </c>
       <c r="L72" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B73" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C73" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D73" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F73" s="4">
         <v>25740</v>
@@ -4362,24 +4359,24 @@
         <v>118</v>
       </c>
       <c r="L73" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B74" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C74" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D74" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F74" s="4">
         <v>25765</v>
@@ -4394,24 +4391,24 @@
         <v>118</v>
       </c>
       <c r="L74" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M74" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B75" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C75" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D75" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F75" s="4">
         <v>25824</v>
@@ -4426,24 +4423,24 @@
         <v>118</v>
       </c>
       <c r="L75" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B76" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C76" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D76" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F76" s="4">
         <v>25866</v>
@@ -4458,24 +4455,24 @@
         <v>118</v>
       </c>
       <c r="L76" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B77" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C77" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D77" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F77" s="4">
         <v>25887</v>
@@ -4490,24 +4487,24 @@
         <v>118</v>
       </c>
       <c r="L77" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B78" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C78" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D78" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F78" s="4">
         <v>25915</v>
@@ -4522,24 +4519,24 @@
         <v>118</v>
       </c>
       <c r="L78" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B79" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C79" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D79" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F79" s="4">
         <v>25950</v>
@@ -4554,24 +4551,24 @@
         <v>118</v>
       </c>
       <c r="L79" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B80" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C80" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D80" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F80" s="4">
         <v>25971</v>
@@ -4586,24 +4583,24 @@
         <v>118</v>
       </c>
       <c r="L80" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B81" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C81" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D81" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F81" s="4">
         <v>25999</v>
@@ -4618,24 +4615,24 @@
         <v>118</v>
       </c>
       <c r="L81" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B82" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C82" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D82" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F82" s="4">
         <v>26027</v>
@@ -4650,24 +4647,24 @@
         <v>118</v>
       </c>
       <c r="L82" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B83" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C83" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D83" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F83" s="4">
         <v>26054</v>
@@ -4682,24 +4679,24 @@
         <v>118</v>
       </c>
       <c r="L83" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B84" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C84" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D84" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F84" s="4">
         <v>26076</v>
@@ -4714,24 +4711,24 @@
         <v>118</v>
       </c>
       <c r="L84" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B85" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C85" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D85" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F85" s="4">
         <v>26104</v>
@@ -4746,24 +4743,24 @@
         <v>118</v>
       </c>
       <c r="L85" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B86" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C86" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D86" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F86" s="4">
         <v>26139</v>
@@ -4778,24 +4775,24 @@
         <v>118</v>
       </c>
       <c r="L86" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B87" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C87" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D87" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F87" s="4">
         <v>26265</v>
@@ -4810,24 +4807,24 @@
         <v>118</v>
       </c>
       <c r="L87" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B88" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C88" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D88" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F88" s="4">
         <v>26307</v>
@@ -4842,24 +4839,24 @@
         <v>118</v>
       </c>
       <c r="L88" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B89" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C89" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D89" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F89" s="4">
         <v>26370</v>
@@ -4874,24 +4871,24 @@
         <v>118</v>
       </c>
       <c r="L89" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B90" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C90" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D90" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F90" s="4">
         <v>26420</v>
@@ -4906,24 +4903,24 @@
         <v>118</v>
       </c>
       <c r="L90" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B91" t="s">
+        <v>391</v>
+      </c>
+      <c r="C91" t="s">
         <v>392</v>
       </c>
-      <c r="C91" t="s">
-        <v>393</v>
-      </c>
       <c r="D91" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F91" s="4">
         <v>26608</v>
@@ -4938,24 +4935,24 @@
         <v>118</v>
       </c>
       <c r="L91" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B92" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C92" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D92" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F92" s="4">
         <v>26785</v>
@@ -4970,10 +4967,10 @@
         <v>118</v>
       </c>
       <c r="L92" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -5145,14 +5142,14 @@
       <c r="B4" t="s">
         <v>264</v>
       </c>
-      <c r="C4" t="s">
-        <v>265</v>
+      <c r="C4">
+        <v>1938</v>
       </c>
       <c r="D4">
         <v>2021</v>
       </c>
       <c r="E4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -5160,7 +5157,7 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C5">
         <v>1931</v>
@@ -5171,10 +5168,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>267</v>
+      </c>
+      <c r="B6" t="s">
         <v>268</v>
-      </c>
-      <c r="B6" t="s">
-        <v>269</v>
       </c>
       <c r="C6">
         <v>1960</v>
@@ -5188,23 +5185,23 @@
         <v>146</v>
       </c>
       <c r="B7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>270</v>
+      </c>
+      <c r="B8" t="s">
         <v>271</v>
-      </c>
-      <c r="B8" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B9" t="s">
         <v>273</v>
-      </c>
-      <c r="B9" t="s">
-        <v>274</v>
       </c>
       <c r="C9">
         <v>1907</v>
@@ -5215,10 +5212,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" t="s">
         <v>275</v>
-      </c>
-      <c r="B10" t="s">
-        <v>276</v>
       </c>
       <c r="C10">
         <v>1898</v>
@@ -5229,10 +5226,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B11" t="s">
         <v>277</v>
-      </c>
-      <c r="B11" t="s">
-        <v>278</v>
       </c>
       <c r="C11">
         <v>1898</v>
@@ -5243,10 +5240,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>278</v>
+      </c>
+      <c r="B12" t="s">
         <v>279</v>
-      </c>
-      <c r="B12" t="s">
-        <v>280</v>
       </c>
       <c r="C12">
         <v>1904</v>
@@ -5257,10 +5254,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>280</v>
+      </c>
+      <c r="B13" t="s">
         <v>281</v>
-      </c>
-      <c r="B13" t="s">
-        <v>282</v>
       </c>
       <c r="C13">
         <v>1914</v>
@@ -5271,10 +5268,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>282</v>
+      </c>
+      <c r="B14" t="s">
         <v>283</v>
-      </c>
-      <c r="B14" t="s">
-        <v>284</v>
       </c>
       <c r="C14">
         <v>1920</v>
@@ -5288,7 +5285,7 @@
         <v>195</v>
       </c>
       <c r="B15" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C15">
         <v>1920</v>
@@ -5299,10 +5296,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C16">
         <v>1898</v>
@@ -5333,13 +5330,13 @@
         <v>254</v>
       </c>
       <c r="B1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C1" t="s">
         <v>286</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>287</v>
-      </c>
-      <c r="D1" t="s">
-        <v>288</v>
       </c>
       <c r="E1" t="s">
         <v>258</v>
@@ -5350,13 +5347,13 @@
         <v>196</v>
       </c>
       <c r="B2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C2">
         <v>1962</v>
       </c>
       <c r="D2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -5364,7 +5361,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C3">
         <v>1952</v>
@@ -5375,7 +5372,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C4">
         <v>1963</v>
@@ -5389,7 +5386,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C5">
         <v>1948</v>
@@ -5397,10 +5394,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C6">
         <v>1958</v>
@@ -5414,7 +5411,7 @@
         <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C7">
         <v>1964</v>
@@ -5425,10 +5422,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C8">
         <v>1956</v>
@@ -5439,7 +5436,7 @@
         <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -5447,7 +5444,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C10">
         <v>1966</v>
@@ -5461,7 +5458,7 @@
         <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C11">
         <v>1968</v>
@@ -5472,10 +5469,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C12">
         <v>1966</v>
@@ -5489,7 +5486,7 @@
         <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C13">
         <v>1921</v>
@@ -5500,7 +5497,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C14">
         <v>1966</v>
@@ -5509,7 +5506,7 @@
         <v>1991</v>
       </c>
       <c r="E14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -5517,7 +5514,7 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C15">
         <v>1968</v>
@@ -5526,7 +5523,7 @@
         <v>1972</v>
       </c>
       <c r="E15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -5534,21 +5531,21 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C16">
         <v>1921</v>
       </c>
       <c r="E16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C17">
         <v>1968</v>
@@ -5562,7 +5559,7 @@
         <v>144</v>
       </c>
       <c r="B18" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C18">
         <v>1969</v>
@@ -5576,13 +5573,13 @@
         <v>227</v>
       </c>
       <c r="B19" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C19">
         <v>1968</v>
       </c>
       <c r="D19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -5590,7 +5587,7 @@
         <v>233</v>
       </c>
       <c r="B20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C20">
         <v>1972</v>
@@ -5604,7 +5601,7 @@
         <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C21">
         <v>1967</v>
@@ -5618,7 +5615,7 @@
         <v>237</v>
       </c>
       <c r="B22" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C22">
         <v>1977</v>
@@ -5629,10 +5626,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B23" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C23">
         <v>1970</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 08/09/2026 10:31
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A35D228-921D-49C6-8E4C-C7EAA557DF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD19376-AE9B-408E-9826-F4BDEE05F890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -777,9 +777,6 @@
     <t>AMI-0057</t>
   </si>
   <si>
-    <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista d'Italia (marxista-leninista) - Lotta di lunga; Partito Marxista-Leninista-Maoista Italiano</t>
-  </si>
-  <si>
     <t>https://archive.org/details/fondazione-pcudi-1977</t>
   </si>
   <si>
@@ -1375,6 +1372,9 @@
   </si>
   <si>
     <t>Lotta di Classe, anno IV, no. 1/2</t>
+  </si>
+  <si>
+    <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista (marxista-leninista) d'Italia - Lotta di lunga durata; Partito Marxista-Leninista-Maoista Italiano</t>
   </si>
 </sst>
 </file>
@@ -1851,7 +1851,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="M1" t="s">
         <v>11</v>
@@ -1895,7 +1895,7 @@
         <v>22</v>
       </c>
       <c r="L2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>23</v>
@@ -1930,7 +1930,7 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>28</v>
@@ -1965,7 +1965,7 @@
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>31</v>
@@ -2000,7 +2000,7 @@
         <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>35</v>
@@ -2035,7 +2035,7 @@
         <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>38</v>
@@ -2070,7 +2070,7 @@
         <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>41</v>
@@ -2105,7 +2105,7 @@
         <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>44</v>
@@ -2140,7 +2140,7 @@
         <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>47</v>
@@ -2175,7 +2175,7 @@
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>50</v>
@@ -2210,7 +2210,7 @@
         <v>34</v>
       </c>
       <c r="L11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>53</v>
@@ -2248,7 +2248,7 @@
         <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>57</v>
@@ -2283,7 +2283,7 @@
         <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>61</v>
@@ -2324,7 +2324,7 @@
         <v>70</v>
       </c>
       <c r="L14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>71</v>
@@ -2359,7 +2359,7 @@
         <v>76</v>
       </c>
       <c r="L15" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>77</v>
@@ -2397,7 +2397,7 @@
         <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>83</v>
@@ -2435,7 +2435,7 @@
         <v>87</v>
       </c>
       <c r="L17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>88</v>
@@ -2470,7 +2470,7 @@
         <v>68</v>
       </c>
       <c r="L18" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>96</v>
@@ -2502,7 +2502,7 @@
         <v>68</v>
       </c>
       <c r="L19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>100</v>
@@ -2534,7 +2534,7 @@
         <v>106</v>
       </c>
       <c r="L20" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>107</v>
@@ -2566,10 +2566,10 @@
         <v>106</v>
       </c>
       <c r="L21" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -2577,7 +2577,7 @@
         <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C22" t="s">
         <v>114</v>
@@ -2586,7 +2586,7 @@
         <v>115</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G22" t="s">
         <v>116</v>
@@ -2598,7 +2598,7 @@
         <v>118</v>
       </c>
       <c r="L22" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>119</v>
@@ -2609,7 +2609,7 @@
         <v>120</v>
       </c>
       <c r="B23" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C23" t="s">
         <v>114</v>
@@ -2618,7 +2618,7 @@
         <v>115</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G23" t="s">
         <v>116</v>
@@ -2630,10 +2630,10 @@
         <v>118</v>
       </c>
       <c r="L23" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -2641,7 +2641,7 @@
         <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C24" t="s">
         <v>114</v>
@@ -2650,7 +2650,7 @@
         <v>115</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G24" t="s">
         <v>116</v>
@@ -2662,7 +2662,7 @@
         <v>118</v>
       </c>
       <c r="L24" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>122</v>
@@ -2673,7 +2673,7 @@
         <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C25" t="s">
         <v>114</v>
@@ -2682,7 +2682,7 @@
         <v>115</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G25" t="s">
         <v>116</v>
@@ -2694,7 +2694,7 @@
         <v>118</v>
       </c>
       <c r="L25" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>124</v>
@@ -2705,7 +2705,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C26" t="s">
         <v>114</v>
@@ -2714,7 +2714,7 @@
         <v>115</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G26" t="s">
         <v>116</v>
@@ -2726,7 +2726,7 @@
         <v>118</v>
       </c>
       <c r="L26" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>126</v>
@@ -2737,7 +2737,7 @@
         <v>127</v>
       </c>
       <c r="B27" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C27" t="s">
         <v>114</v>
@@ -2746,7 +2746,7 @@
         <v>115</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G27" t="s">
         <v>116</v>
@@ -2758,10 +2758,10 @@
         <v>118</v>
       </c>
       <c r="L27" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2769,7 +2769,7 @@
         <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C28" t="s">
         <v>114</v>
@@ -2778,7 +2778,7 @@
         <v>115</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G28" t="s">
         <v>116</v>
@@ -2790,7 +2790,7 @@
         <v>118</v>
       </c>
       <c r="L28" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>129</v>
@@ -2801,7 +2801,7 @@
         <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C29" t="s">
         <v>114</v>
@@ -2810,7 +2810,7 @@
         <v>115</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G29" t="s">
         <v>116</v>
@@ -2825,7 +2825,7 @@
         <v>64</v>
       </c>
       <c r="L29" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>131</v>
@@ -2836,7 +2836,7 @@
         <v>132</v>
       </c>
       <c r="B30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C30" t="s">
         <v>114</v>
@@ -2845,7 +2845,7 @@
         <v>115</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G30" t="s">
         <v>116</v>
@@ -2860,7 +2860,7 @@
         <v>133</v>
       </c>
       <c r="L30" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>134</v>
@@ -2895,7 +2895,7 @@
         <v>34</v>
       </c>
       <c r="L31" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>138</v>
@@ -2930,7 +2930,7 @@
         <v>34</v>
       </c>
       <c r="L32" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>141</v>
@@ -2959,7 +2959,7 @@
         <v>146</v>
       </c>
       <c r="L33" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>147</v>
@@ -2997,7 +2997,7 @@
         <v>17</v>
       </c>
       <c r="L34" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>153</v>
@@ -3041,7 +3041,7 @@
         <v>64</v>
       </c>
       <c r="L35" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>159</v>
@@ -3064,7 +3064,7 @@
         <v>92</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G36" t="s">
         <v>116</v>
@@ -3076,7 +3076,7 @@
         <v>68</v>
       </c>
       <c r="L36" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>165</v>
@@ -3114,7 +3114,7 @@
         <v>144</v>
       </c>
       <c r="L37" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>170</v>
@@ -3149,7 +3149,7 @@
         <v>34</v>
       </c>
       <c r="L38" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>173</v>
@@ -3187,7 +3187,7 @@
         <v>177</v>
       </c>
       <c r="L39" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>178</v>
@@ -3222,7 +3222,7 @@
         <v>181</v>
       </c>
       <c r="L40" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>182</v>
@@ -3257,7 +3257,7 @@
         <v>34</v>
       </c>
       <c r="L41" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>186</v>
@@ -3289,7 +3289,7 @@
         <v>190</v>
       </c>
       <c r="L42" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>191</v>
@@ -3327,7 +3327,7 @@
         <v>196</v>
       </c>
       <c r="L43" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>197</v>
@@ -3362,7 +3362,7 @@
         <v>27</v>
       </c>
       <c r="L44" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>200</v>
@@ -3397,7 +3397,7 @@
         <v>27</v>
       </c>
       <c r="L45" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>203</v>
@@ -3432,7 +3432,7 @@
         <v>27</v>
       </c>
       <c r="L46" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>206</v>
@@ -3467,7 +3467,7 @@
         <v>34</v>
       </c>
       <c r="L47" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>209</v>
@@ -3502,7 +3502,7 @@
         <v>34</v>
       </c>
       <c r="L48" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>212</v>
@@ -3537,7 +3537,7 @@
         <v>27</v>
       </c>
       <c r="L49" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>215</v>
@@ -3572,7 +3572,7 @@
         <v>27</v>
       </c>
       <c r="L50" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M50" s="3" t="s">
         <v>218</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="L51" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M51" s="3" t="s">
         <v>221</v>
@@ -3642,7 +3642,7 @@
         <v>34</v>
       </c>
       <c r="L52" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M52" s="3" t="s">
         <v>224</v>
@@ -3677,7 +3677,7 @@
         <v>68</v>
       </c>
       <c r="L53" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M53" s="3" t="s">
         <v>229</v>
@@ -3709,7 +3709,7 @@
         <v>233</v>
       </c>
       <c r="L54" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M54" s="3" t="s">
         <v>234</v>
@@ -3732,7 +3732,7 @@
         <v>238</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G55" t="s">
         <v>239</v>
@@ -3747,7 +3747,7 @@
         <v>240</v>
       </c>
       <c r="L55" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M55" s="3" t="s">
         <v>241</v>
@@ -3782,7 +3782,7 @@
         <v>68</v>
       </c>
       <c r="L56" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M56" s="3" t="s">
         <v>245</v>
@@ -3820,7 +3820,7 @@
         <v>190</v>
       </c>
       <c r="L57" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M57" s="3" t="s">
         <v>249</v>
@@ -3831,7 +3831,7 @@
         <v>250</v>
       </c>
       <c r="B58" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C58" t="s">
         <v>237</v>
@@ -3858,30 +3858,30 @@
         <v>240</v>
       </c>
       <c r="K58" t="s">
+        <v>450</v>
+      </c>
+      <c r="L58" t="s">
+        <v>314</v>
+      </c>
+      <c r="M58" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="L58" t="s">
-        <v>315</v>
-      </c>
-      <c r="M58" s="3" t="s">
+      <c r="N58" t="s">
         <v>252</v>
-      </c>
-      <c r="N58" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B59" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C59" t="s">
         <v>99</v>
       </c>
       <c r="D59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E59" t="s">
         <v>99</v>
@@ -3899,24 +3899,24 @@
         <v>106</v>
       </c>
       <c r="L59" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>305</v>
+      </c>
+      <c r="B60" t="s">
         <v>306</v>
-      </c>
-      <c r="B60" t="s">
-        <v>307</v>
       </c>
       <c r="C60" t="s">
         <v>99</v>
       </c>
       <c r="D60" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E60" t="s">
         <v>99</v>
@@ -3934,24 +3934,24 @@
         <v>106</v>
       </c>
       <c r="L60" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>315</v>
+      </c>
+      <c r="B61" t="s">
         <v>316</v>
-      </c>
-      <c r="B61" t="s">
-        <v>317</v>
       </c>
       <c r="C61" t="s">
         <v>99</v>
       </c>
       <c r="D61" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E61" t="s">
         <v>99</v>
@@ -3969,21 +3969,21 @@
         <v>106</v>
       </c>
       <c r="J61" t="s">
+        <v>318</v>
+      </c>
+      <c r="L61" t="s">
+        <v>314</v>
+      </c>
+      <c r="M61" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="L61" t="s">
-        <v>315</v>
-      </c>
-      <c r="M61" s="3" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>324</v>
+      </c>
+      <c r="B62" t="s">
         <v>325</v>
-      </c>
-      <c r="B62" t="s">
-        <v>326</v>
       </c>
       <c r="C62" t="s">
         <v>17</v>
@@ -4007,18 +4007,18 @@
         <v>27</v>
       </c>
       <c r="L62" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>327</v>
+      </c>
+      <c r="B63" t="s">
         <v>328</v>
-      </c>
-      <c r="B63" t="s">
-        <v>329</v>
       </c>
       <c r="F63" s="4">
         <v>24917</v>
@@ -4027,30 +4027,30 @@
         <v>75</v>
       </c>
       <c r="H63" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I63" t="s">
         <v>106</v>
       </c>
       <c r="K63" t="s">
+        <v>330</v>
+      </c>
+      <c r="L63" t="s">
+        <v>314</v>
+      </c>
+      <c r="M63" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="L63" t="s">
-        <v>315</v>
-      </c>
-      <c r="M63" s="3" t="s">
+      <c r="N63" t="s">
         <v>332</v>
-      </c>
-      <c r="N63" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B64" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C64" t="s">
         <v>233</v>
@@ -4059,36 +4059,36 @@
         <v>233</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G64" t="s">
         <v>94</v>
       </c>
       <c r="H64" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I64" t="s">
         <v>68</v>
       </c>
       <c r="L64" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B65" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C65" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D65" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F65" s="4">
         <v>26956</v>
@@ -4097,24 +4097,24 @@
         <v>94</v>
       </c>
       <c r="H65" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I65" t="s">
         <v>68</v>
       </c>
       <c r="L65" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>340</v>
+      </c>
+      <c r="B66" t="s">
         <v>341</v>
-      </c>
-      <c r="B66" t="s">
-        <v>342</v>
       </c>
       <c r="C66" t="s">
         <v>64</v>
@@ -4132,24 +4132,24 @@
         <v>68</v>
       </c>
       <c r="L66" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="N66" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>343</v>
+      </c>
+      <c r="B67" t="s">
         <v>344</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>345</v>
-      </c>
-      <c r="C67" t="s">
-        <v>346</v>
       </c>
       <c r="F67">
         <v>1970</v>
@@ -4164,27 +4164,27 @@
         <v>68</v>
       </c>
       <c r="L67" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="N67" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>350</v>
+      </c>
+      <c r="B68" t="s">
         <v>351</v>
-      </c>
-      <c r="B68" t="s">
-        <v>352</v>
       </c>
       <c r="C68" t="s">
         <v>64</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G68" t="s">
         <v>94</v>
@@ -4196,30 +4196,30 @@
         <v>68</v>
       </c>
       <c r="L68" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="N68" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B69" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C69" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D69" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="G69" t="s">
         <v>116</v>
@@ -4231,24 +4231,24 @@
         <v>118</v>
       </c>
       <c r="L69" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B70" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C70" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D70" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F70" s="8">
         <v>25704</v>
@@ -4263,24 +4263,24 @@
         <v>118</v>
       </c>
       <c r="L70" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B71" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C71" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D71" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F71" s="4">
         <v>25718</v>
@@ -4295,24 +4295,24 @@
         <v>118</v>
       </c>
       <c r="L71" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B72" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C72" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D72" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F72" s="4">
         <v>25719</v>
@@ -4327,24 +4327,24 @@
         <v>118</v>
       </c>
       <c r="L72" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B73" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C73" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D73" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F73" s="4">
         <v>25740</v>
@@ -4359,24 +4359,24 @@
         <v>118</v>
       </c>
       <c r="L73" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B74" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C74" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D74" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F74" s="4">
         <v>25765</v>
@@ -4391,24 +4391,24 @@
         <v>118</v>
       </c>
       <c r="L74" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M74" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B75" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C75" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D75" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F75" s="4">
         <v>25824</v>
@@ -4423,24 +4423,24 @@
         <v>118</v>
       </c>
       <c r="L75" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B76" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C76" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D76" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F76" s="4">
         <v>25866</v>
@@ -4455,24 +4455,24 @@
         <v>118</v>
       </c>
       <c r="L76" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B77" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C77" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D77" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F77" s="4">
         <v>25887</v>
@@ -4487,24 +4487,24 @@
         <v>118</v>
       </c>
       <c r="L77" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B78" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C78" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D78" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F78" s="4">
         <v>25915</v>
@@ -4519,24 +4519,24 @@
         <v>118</v>
       </c>
       <c r="L78" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B79" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C79" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D79" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F79" s="4">
         <v>25950</v>
@@ -4551,24 +4551,24 @@
         <v>118</v>
       </c>
       <c r="L79" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B80" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C80" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D80" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F80" s="4">
         <v>25971</v>
@@ -4583,24 +4583,24 @@
         <v>118</v>
       </c>
       <c r="L80" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B81" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C81" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D81" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F81" s="4">
         <v>25999</v>
@@ -4615,24 +4615,24 @@
         <v>118</v>
       </c>
       <c r="L81" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B82" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C82" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D82" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F82" s="4">
         <v>26027</v>
@@ -4647,24 +4647,24 @@
         <v>118</v>
       </c>
       <c r="L82" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B83" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C83" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D83" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F83" s="4">
         <v>26054</v>
@@ -4679,24 +4679,24 @@
         <v>118</v>
       </c>
       <c r="L83" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B84" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C84" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D84" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F84" s="4">
         <v>26076</v>
@@ -4711,24 +4711,24 @@
         <v>118</v>
       </c>
       <c r="L84" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B85" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C85" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D85" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F85" s="4">
         <v>26104</v>
@@ -4743,24 +4743,24 @@
         <v>118</v>
       </c>
       <c r="L85" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B86" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C86" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D86" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F86" s="4">
         <v>26139</v>
@@ -4775,24 +4775,24 @@
         <v>118</v>
       </c>
       <c r="L86" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B87" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C87" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D87" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F87" s="4">
         <v>26265</v>
@@ -4807,24 +4807,24 @@
         <v>118</v>
       </c>
       <c r="L87" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B88" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C88" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D88" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F88" s="4">
         <v>26307</v>
@@ -4839,24 +4839,24 @@
         <v>118</v>
       </c>
       <c r="L88" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B89" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C89" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D89" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F89" s="4">
         <v>26370</v>
@@ -4871,24 +4871,24 @@
         <v>118</v>
       </c>
       <c r="L89" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B90" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C90" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D90" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F90" s="4">
         <v>26420</v>
@@ -4903,24 +4903,24 @@
         <v>118</v>
       </c>
       <c r="L90" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B91" t="s">
+        <v>390</v>
+      </c>
+      <c r="C91" t="s">
         <v>391</v>
       </c>
-      <c r="C91" t="s">
-        <v>392</v>
-      </c>
       <c r="D91" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F91" s="4">
         <v>26608</v>
@@ -4935,24 +4935,24 @@
         <v>118</v>
       </c>
       <c r="L91" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B92" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C92" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D92" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F92" s="4">
         <v>26785</v>
@@ -4967,10 +4967,10 @@
         <v>118</v>
       </c>
       <c r="L92" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -5086,19 +5086,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" t="s">
         <v>254</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>255</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>256</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>257</v>
-      </c>
-      <c r="E1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -5106,7 +5106,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C2">
         <v>1893</v>
@@ -5115,15 +5115,15 @@
         <v>1976</v>
       </c>
       <c r="E2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" t="s">
         <v>261</v>
-      </c>
-      <c r="B3" t="s">
-        <v>262</v>
       </c>
       <c r="C3">
         <v>1921</v>
@@ -5132,7 +5132,7 @@
         <v>1993</v>
       </c>
       <c r="E3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -5140,7 +5140,7 @@
         <v>240</v>
       </c>
       <c r="B4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C4">
         <v>1938</v>
@@ -5149,7 +5149,7 @@
         <v>2021</v>
       </c>
       <c r="E4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -5157,7 +5157,7 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C5">
         <v>1931</v>
@@ -5168,10 +5168,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B6" t="s">
         <v>267</v>
-      </c>
-      <c r="B6" t="s">
-        <v>268</v>
       </c>
       <c r="C6">
         <v>1960</v>
@@ -5185,23 +5185,23 @@
         <v>146</v>
       </c>
       <c r="B7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B8" t="s">
         <v>270</v>
-      </c>
-      <c r="B8" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B9" t="s">
         <v>272</v>
-      </c>
-      <c r="B9" t="s">
-        <v>273</v>
       </c>
       <c r="C9">
         <v>1907</v>
@@ -5212,10 +5212,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>273</v>
+      </c>
+      <c r="B10" t="s">
         <v>274</v>
-      </c>
-      <c r="B10" t="s">
-        <v>275</v>
       </c>
       <c r="C10">
         <v>1898</v>
@@ -5226,10 +5226,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>275</v>
+      </c>
+      <c r="B11" t="s">
         <v>276</v>
-      </c>
-      <c r="B11" t="s">
-        <v>277</v>
       </c>
       <c r="C11">
         <v>1898</v>
@@ -5240,10 +5240,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>277</v>
+      </c>
+      <c r="B12" t="s">
         <v>278</v>
-      </c>
-      <c r="B12" t="s">
-        <v>279</v>
       </c>
       <c r="C12">
         <v>1904</v>
@@ -5254,10 +5254,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>279</v>
+      </c>
+      <c r="B13" t="s">
         <v>280</v>
-      </c>
-      <c r="B13" t="s">
-        <v>281</v>
       </c>
       <c r="C13">
         <v>1914</v>
@@ -5268,10 +5268,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>281</v>
+      </c>
+      <c r="B14" t="s">
         <v>282</v>
-      </c>
-      <c r="B14" t="s">
-        <v>283</v>
       </c>
       <c r="C14">
         <v>1920</v>
@@ -5285,7 +5285,7 @@
         <v>195</v>
       </c>
       <c r="B15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C15">
         <v>1920</v>
@@ -5296,10 +5296,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B16" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C16">
         <v>1898</v>
@@ -5327,19 +5327,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1" t="s">
         <v>285</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>286</v>
       </c>
-      <c r="D1" t="s">
-        <v>287</v>
-      </c>
       <c r="E1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -5347,13 +5347,13 @@
         <v>196</v>
       </c>
       <c r="B2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C2">
         <v>1962</v>
       </c>
       <c r="D2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -5361,7 +5361,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C3">
         <v>1952</v>
@@ -5372,7 +5372,7 @@
         <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C4">
         <v>1963</v>
@@ -5386,7 +5386,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C5">
         <v>1948</v>
@@ -5394,10 +5394,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C6">
         <v>1958</v>
@@ -5411,7 +5411,7 @@
         <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C7">
         <v>1964</v>
@@ -5422,10 +5422,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C8">
         <v>1956</v>
@@ -5436,7 +5436,7 @@
         <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -5444,7 +5444,7 @@
         <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C10">
         <v>1966</v>
@@ -5458,7 +5458,7 @@
         <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C11">
         <v>1968</v>
@@ -5469,10 +5469,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C12">
         <v>1966</v>
@@ -5486,7 +5486,7 @@
         <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C13">
         <v>1921</v>
@@ -5497,7 +5497,7 @@
         <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C14">
         <v>1966</v>
@@ -5506,7 +5506,7 @@
         <v>1991</v>
       </c>
       <c r="E14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -5514,7 +5514,7 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C15">
         <v>1968</v>
@@ -5523,7 +5523,7 @@
         <v>1972</v>
       </c>
       <c r="E15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -5531,21 +5531,21 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C16">
         <v>1921</v>
       </c>
       <c r="E16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B17" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C17">
         <v>1968</v>
@@ -5559,7 +5559,7 @@
         <v>144</v>
       </c>
       <c r="B18" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C18">
         <v>1969</v>
@@ -5573,13 +5573,13 @@
         <v>227</v>
       </c>
       <c r="B19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C19">
         <v>1968</v>
       </c>
       <c r="D19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -5587,7 +5587,7 @@
         <v>233</v>
       </c>
       <c r="B20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C20">
         <v>1972</v>
@@ -5601,7 +5601,7 @@
         <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C21">
         <v>1967</v>
@@ -5615,7 +5615,7 @@
         <v>237</v>
       </c>
       <c r="B22" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C22">
         <v>1977</v>
@@ -5626,10 +5626,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B23" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C23">
         <v>1970</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 09/09/2026 16:08
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD19376-AE9B-408E-9826-F4BDEE05F890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3E5617-8C1A-4865-99F2-B8F56F7C1ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="455">
   <si>
     <t>ID</t>
   </si>
@@ -1375,6 +1375,18 @@
   </si>
   <si>
     <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista (marxista-leninista) d'Italia - Lotta di lunga durata; Partito Marxista-Leninista-Maoista Italiano</t>
+  </si>
+  <si>
+    <t>AMI-0092</t>
+  </si>
+  <si>
+    <t>Avanziamo lungo la via aperta dalla Rivoluzione socialista d'ottobre</t>
+  </si>
+  <si>
+    <t>Edizioni Servire il Popolo</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/avanziamo-lungo-la-via/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -1800,7 +1812,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P92"/>
+  <dimension ref="A1:P93"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -4971,6 +4983,41 @@
       </c>
       <c r="M92" s="3" t="s">
         <v>423</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>451</v>
+      </c>
+      <c r="B93" t="s">
+        <v>452</v>
+      </c>
+      <c r="C93" t="s">
+        <v>92</v>
+      </c>
+      <c r="E93" t="s">
+        <v>453</v>
+      </c>
+      <c r="F93">
+        <v>1969</v>
+      </c>
+      <c r="G93" t="s">
+        <v>20</v>
+      </c>
+      <c r="H93" t="s">
+        <v>164</v>
+      </c>
+      <c r="I93" t="s">
+        <v>34</v>
+      </c>
+      <c r="K93" t="s">
+        <v>17</v>
+      </c>
+      <c r="L93" t="s">
+        <v>314</v>
+      </c>
+      <c r="M93" s="3" t="s">
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -5067,10 +5114,11 @@
     <hyperlink ref="M89" r:id="rId89" xr:uid="{8D9593CC-1AC6-4151-A7F0-9E914C39EEA1}"/>
     <hyperlink ref="M91" r:id="rId90" xr:uid="{734F4C0D-ECE0-4D17-AED2-596C8405BA52}"/>
     <hyperlink ref="M70" r:id="rId91" xr:uid="{410C497E-B7A6-4A52-BDB5-CD7FDB43C527}"/>
+    <hyperlink ref="M93" r:id="rId92" xr:uid="{A1560D73-B423-4F16-8BB5-470F2068279E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId92"/>
+    <tablePart r:id="rId93"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>